<commit_message>
Resolve Makai radio-ID references and link resources from excerpts
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R1bb5be1cc6f842b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R60b30f5c93f84f8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R6d5046da891d43fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R77e3792d60934a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R90044babe3414fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R0afcf177922b4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R57ac693bd0ef42b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R90619854ad91468c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -215,8 +215,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S361" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:S361"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S364" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:S364"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Name in exchange"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExcludedExchanges" displayName="ExcludedExchanges" ref="A7:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:F25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ExcludedExchanges" displayName="ExcludedExchanges" ref="A7:F27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:F27"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Clip"/>
@@ -546,7 +546,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 354 selected exchanges.</x:v>
+        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 357 selected exchanges.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -652,7 +652,7 @@
         <x:v>14580155</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A10,Exchanges!$J$8:$J$361,B10)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A10,Exchanges!$J$8:$J$364,B10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -687,7 +687,7 @@
         <x:v>14590020</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A11,Exchanges!$J$8:$J$361,B11)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A11,Exchanges!$J$8:$J$364,B11)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -722,7 +722,7 @@
         <x:v>14590089</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A12,Exchanges!$J$8:$J$361,B12)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A12,Exchanges!$J$8:$J$364,B12)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -757,7 +757,7 @@
         <x:v>14590111</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A13,Exchanges!$J$8:$J$361,B13)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A13,Exchanges!$J$8:$J$364,B13)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -792,7 +792,7 @@
         <x:v>14580152</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A14,Exchanges!$J$8:$J$361,B14)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A14,Exchanges!$J$8:$J$364,B14)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -827,7 +827,7 @@
         <x:v>14590098</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A15,Exchanges!$J$8:$J$361,B15)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A15,Exchanges!$J$8:$J$364,B15)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -864,7 +864,7 @@
         <x:v>14590107</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A16,Exchanges!$J$8:$J$361,B16)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A16,Exchanges!$J$8:$J$364,B16)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -899,7 +899,7 @@
         <x:v>14590104</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A17,Exchanges!$J$8:$J$361,B17)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A17,Exchanges!$J$8:$J$364,B17)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
@@ -936,7 +936,7 @@
         <x:v>14590200</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A18,Exchanges!$J$8:$J$361,B18)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A18,Exchanges!$J$8:$J$364,B18)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
@@ -973,7 +973,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A19,Exchanges!$J$8:$J$361,B19)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A19,Exchanges!$J$8:$J$364,B19)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
@@ -1012,7 +1012,7 @@
         <x:v>14590118</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A20,Exchanges!$J$8:$J$361,B20)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A20,Exchanges!$J$8:$J$364,B20)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
@@ -1049,7 +1049,7 @@
         <x:v>14590088</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A21,Exchanges!$J$8:$J$361,B21)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A21,Exchanges!$J$8:$J$364,B21)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
@@ -1086,7 +1086,7 @@
         <x:v>14590117</x:v>
       </x:c>
       <x:c r="C22" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A22,Exchanges!$J$8:$J$361,B22)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A22,Exchanges!$J$8:$J$364,B22)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
@@ -1121,7 +1121,7 @@
         <x:v>14590320</x:v>
       </x:c>
       <x:c r="C23" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A23,Exchanges!$J$8:$J$361,B23)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A23,Exchanges!$J$8:$J$364,B23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="10" t="n">
@@ -1156,7 +1156,7 @@
         <x:v>14590084</x:v>
       </x:c>
       <x:c r="C24" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A24,Exchanges!$J$8:$J$361,B24)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A24,Exchanges!$J$8:$J$364,B24)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D24" s="10" t="n">
@@ -1175,7 +1175,9 @@
       <x:c r="I24" s="10" t="str">
         <x:v>Kelepi Makai</x:v>
       </x:c>
-      <x:c r="J24" s="10"/>
+      <x:c r="J24" s="10" t="str">
+        <x:v>Owner confirmed Makai spelling. 14590247 is also associated with Makai in named exchanges. Further confirmation is needed to attribute a particular recording.</x:v>
+      </x:c>
       <x:c r="K24" s="10" t="str">
         <x:v>2026-09-22, 2026-09-26, 2026-10-09</x:v>
       </x:c>
@@ -1191,7 +1193,7 @@
         <x:v>14590237</x:v>
       </x:c>
       <x:c r="C25" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A25,Exchanges!$J$8:$J$361,B25)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A25,Exchanges!$J$8:$J$364,B25)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
@@ -1226,7 +1228,7 @@
         <x:v>14590315</x:v>
       </x:c>
       <x:c r="C26" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A26,Exchanges!$J$8:$J$361,B26)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A26,Exchanges!$J$8:$J$364,B26)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
@@ -1261,7 +1263,7 @@
         <x:v>14590162</x:v>
       </x:c>
       <x:c r="C27" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A27,Exchanges!$J$8:$J$361,B27)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A27,Exchanges!$J$8:$J$364,B27)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
@@ -1296,7 +1298,7 @@
         <x:v>14590081</x:v>
       </x:c>
       <x:c r="C28" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A28,Exchanges!$J$8:$J$361,B28)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A28,Exchanges!$J$8:$J$364,B28)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
@@ -1331,7 +1333,7 @@
         <x:v>14590102</x:v>
       </x:c>
       <x:c r="C29" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A29,Exchanges!$J$8:$J$361,B29)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A29,Exchanges!$J$8:$J$364,B29)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
@@ -1366,7 +1368,7 @@
         <x:v>14590344</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A30,Exchanges!$J$8:$J$361,B30)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A30,Exchanges!$J$8:$J$364,B30)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
@@ -1403,7 +1405,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C31" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A31,Exchanges!$J$8:$J$361,B31)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A31,Exchanges!$J$8:$J$364,B31)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
@@ -1442,7 +1444,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C32" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A32,Exchanges!$J$8:$J$361,B32)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A32,Exchanges!$J$8:$J$364,B32)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
@@ -1479,7 +1481,7 @@
         <x:v>14590087</x:v>
       </x:c>
       <x:c r="C33" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A33,Exchanges!$J$8:$J$361,B33)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A33,Exchanges!$J$8:$J$364,B33)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
@@ -1514,7 +1516,7 @@
         <x:v>14590044</x:v>
       </x:c>
       <x:c r="C34" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A34,Exchanges!$J$8:$J$361,B34)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A34,Exchanges!$J$8:$J$364,B34)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
@@ -1549,7 +1551,7 @@
         <x:v>14590123</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A35,Exchanges!$J$8:$J$361,B35)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A35,Exchanges!$J$8:$J$364,B35)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
@@ -1584,7 +1586,7 @@
         <x:v>14590037</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A36,Exchanges!$J$8:$J$361,B36)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A36,Exchanges!$J$8:$J$364,B36)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
@@ -1621,7 +1623,7 @@
         <x:v>14590095</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A37,Exchanges!$J$8:$J$361,B37)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A37,Exchanges!$J$8:$J$364,B37)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
@@ -1658,7 +1660,7 @@
         <x:v>14590099</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A38,Exchanges!$J$8:$J$361,B38)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A38,Exchanges!$J$8:$J$364,B38)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D38" s="10" t="n">
@@ -1695,7 +1697,7 @@
         <x:v>14590207</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A39,Exchanges!$J$8:$J$361,B39)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A39,Exchanges!$J$8:$J$364,B39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
@@ -1732,7 +1734,7 @@
         <x:v>14590067</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A40,Exchanges!$J$8:$J$361,B40)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A40,Exchanges!$J$8:$J$364,B40)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
@@ -1769,7 +1771,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A41,Exchanges!$J$8:$J$361,B41)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A41,Exchanges!$J$8:$J$364,B41)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
@@ -1804,7 +1806,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A42,Exchanges!$J$8:$J$361,B42)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A42,Exchanges!$J$8:$J$364,B42)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
@@ -1839,7 +1841,7 @@
         <x:v>14590038</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A43,Exchanges!$J$8:$J$361,B43)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A43,Exchanges!$J$8:$J$364,B43)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
@@ -1874,7 +1876,7 @@
         <x:v>14590345</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A44,Exchanges!$J$8:$J$361,B44)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A44,Exchanges!$J$8:$J$364,B44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
@@ -1909,7 +1911,7 @@
         <x:v>14590079</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A45,Exchanges!$J$8:$J$361,B45)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A45,Exchanges!$J$8:$J$364,B45)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
@@ -1944,7 +1946,7 @@
         <x:v>14590026</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A46,Exchanges!$J$8:$J$361,B46)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A46,Exchanges!$J$8:$J$364,B46)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
@@ -1981,7 +1983,7 @@
         <x:v>14590031</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A47,Exchanges!$J$8:$J$361,B47)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A47,Exchanges!$J$8:$J$364,B47)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
@@ -2018,7 +2020,7 @@
         <x:v>14590101</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A48,Exchanges!$J$8:$J$361,B48)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A48,Exchanges!$J$8:$J$364,B48)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
@@ -2055,7 +2057,7 @@
         <x:v>14590103</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A49,Exchanges!$J$8:$J$361,B49)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A49,Exchanges!$J$8:$J$364,B49)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
@@ -2092,7 +2094,7 @@
         <x:v>14590043</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A50,Exchanges!$J$8:$J$361,B50)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A50,Exchanges!$J$8:$J$364,B50)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D50" s="10" t="n">
@@ -2129,7 +2131,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A51,Exchanges!$J$8:$J$361,B51)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A51,Exchanges!$J$8:$J$364,B51)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D51" s="10" t="n">
@@ -2168,7 +2170,7 @@
         <x:v>14590266</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A52,Exchanges!$J$8:$J$361,B52)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A52,Exchanges!$J$8:$J$364,B52)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D52" s="10" t="n">
@@ -2203,7 +2205,7 @@
         <x:v>14590219</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A53,Exchanges!$J$8:$J$361,B53)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A53,Exchanges!$J$8:$J$364,B53)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D53" s="10" t="n">
@@ -2238,7 +2240,7 @@
         <x:v>14590066</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A54,Exchanges!$J$8:$J$361,B54)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A54,Exchanges!$J$8:$J$364,B54)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
@@ -2275,7 +2277,7 @@
         <x:v>14590090</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A55,Exchanges!$J$8:$J$361,B55)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A55,Exchanges!$J$8:$J$364,B55)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
@@ -2312,7 +2314,7 @@
         <x:v>14590268</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A56,Exchanges!$J$8:$J$361,B56)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A56,Exchanges!$J$8:$J$364,B56)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
@@ -2349,7 +2351,7 @@
         <x:v>14590085</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A57,Exchanges!$J$8:$J$361,B57)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A57,Exchanges!$J$8:$J$364,B57)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D57" s="10" t="n">
@@ -2386,7 +2388,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A58,Exchanges!$J$8:$J$361,B58)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A58,Exchanges!$J$8:$J$364,B58)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D58" s="10" t="n">
@@ -2425,7 +2427,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A59,Exchanges!$J$8:$J$361,B59)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A59,Exchanges!$J$8:$J$364,B59)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="10" t="n">
@@ -2464,7 +2466,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A60,Exchanges!$J$8:$J$361,B60)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A60,Exchanges!$J$8:$J$364,B60)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D60" s="10" t="n">
@@ -2503,7 +2505,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A61,Exchanges!$J$8:$J$361,B61)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A61,Exchanges!$J$8:$J$364,B61)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
@@ -2542,7 +2544,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A62,Exchanges!$J$8:$J$361,B62)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A62,Exchanges!$J$8:$J$364,B62)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
@@ -2581,7 +2583,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A63,Exchanges!$J$8:$J$361,B63)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A63,Exchanges!$J$8:$J$364,B63)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
@@ -2620,7 +2622,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A64,Exchanges!$J$8:$J$361,B64)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A64,Exchanges!$J$8:$J$364,B64)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
@@ -2659,7 +2661,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A65,Exchanges!$J$8:$J$361,B65)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A65,Exchanges!$J$8:$J$364,B65)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
@@ -2698,7 +2700,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A66,Exchanges!$J$8:$J$361,B66)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A66,Exchanges!$J$8:$J$364,B66)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D66" s="10" t="n">
@@ -2737,7 +2739,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A67,Exchanges!$J$8:$J$361,B67)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A67,Exchanges!$J$8:$J$364,B67)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D67" s="10" t="n">
@@ -2774,7 +2776,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A68,Exchanges!$J$8:$J$361,B68)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A68,Exchanges!$J$8:$J$364,B68)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
@@ -2813,7 +2815,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A69,Exchanges!$J$8:$J$361,B69)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A69,Exchanges!$J$8:$J$364,B69)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D69" s="10" t="n">
@@ -2852,7 +2854,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C70" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A70,Exchanges!$J$8:$J$361,B70)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A70,Exchanges!$J$8:$J$364,B70)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D70" s="10" t="n">
@@ -2891,7 +2893,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C71" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A71,Exchanges!$J$8:$J$361,B71)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A71,Exchanges!$J$8:$J$364,B71)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D71" s="10" t="n">
@@ -2928,7 +2930,7 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="C72" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A72,Exchanges!$J$8:$J$361,B72)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A72,Exchanges!$J$8:$J$364,B72)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D72" s="10" t="n">
@@ -2959,39 +2961,39 @@
     </x:row>
     <x:row r="73" ht="60" customHeight="1">
       <x:c r="A73" s="10" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="B73" s="11" t="str">
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="C73" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A73,Exchanges!$J$8:$J$361,B73)</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A73,Exchanges!$J$8:$J$364,B73)</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D73" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E73" s="12" t="n">
-        <x:v>46282</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F73" s="12" t="n">
-        <x:v>46290</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="G73" s="10" t="str">
-        <x:v>Name spelling unresolved</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H73" s="10"/>
       <x:c r="I73" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Kelepi Makai</x:v>
       </x:c>
       <x:c r="J73" s="10" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
+        <x:v>Owner confirmed Makai spelling. Five response days; October 1 reply is unclear. These examples support an association, not permanent radio ownership.</x:v>
       </x:c>
       <x:c r="K73" s="10" t="str">
-        <x:v>2026-09-17, 2026-09-25</x:v>
+        <x:v>2026-09-12, 2026-09-17, 2026-09-25, 2026-09-26, 2026-10-01</x:v>
       </x:c>
       <x:c r="L73" s="10" t="str">
-        <x:v>E117, E177</x:v>
+        <x:v>E117, E177, E355, E356, E357</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3002,7 +3004,7 @@
         <x:v>14590112</x:v>
       </x:c>
       <x:c r="C74" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A74,Exchanges!$J$8:$J$361,B74)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A74,Exchanges!$J$8:$J$364,B74)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D74" s="10" t="n">
@@ -3039,7 +3041,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C75" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A75,Exchanges!$J$8:$J$361,B75)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A75,Exchanges!$J$8:$J$364,B75)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D75" s="10" t="n">
@@ -3078,7 +3080,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C76" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A76,Exchanges!$J$8:$J$361,B76)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A76,Exchanges!$J$8:$J$364,B76)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D76" s="10" t="n">
@@ -3117,7 +3119,7 @@
         <x:v>14590097</x:v>
       </x:c>
       <x:c r="C77" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A77,Exchanges!$J$8:$J$361,B77)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A77,Exchanges!$J$8:$J$364,B77)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D77" s="10" t="n">
@@ -3154,7 +3156,7 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C78" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A78,Exchanges!$J$8:$J$361,B78)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A78,Exchanges!$J$8:$J$364,B78)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D78" s="10" t="n">
@@ -3193,7 +3195,7 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C79" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A79,Exchanges!$J$8:$J$361,B79)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A79,Exchanges!$J$8:$J$364,B79)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="10" t="n">
@@ -3232,7 +3234,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C80" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A80,Exchanges!$J$8:$J$361,B80)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A80,Exchanges!$J$8:$J$364,B80)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D80" s="10" t="n">
@@ -3271,7 +3273,7 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C81" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A81,Exchanges!$J$8:$J$361,B81)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A81,Exchanges!$J$8:$J$364,B81)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D81" s="10" t="n">
@@ -3310,7 +3312,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C82" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$361,A82,Exchanges!$J$8:$J$361,B82)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A82,Exchanges!$J$8:$J$364,B82)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D82" s="10" t="n">
@@ -3348,7 +3350,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58eb3b08e6544be4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R628287340a7d4bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10370,7 +10372,7 @@
         <x:v>E117</x:v>
       </x:c>
       <x:c r="B124" s="13" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="C124" s="14" t="n">
         <x:v>46282</x:v>
@@ -10398,16 +10400,16 @@
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="K124" s="13" t="str">
-        <x:v>Hey, [McKay?].</x:v>
+        <x:v>Hey, Makai?</x:v>
       </x:c>
       <x:c r="L124" s="13" t="str">
-        <x:v>[What's up / that's right]?</x:v>
+        <x:v>What's up?</x:v>
       </x:c>
       <x:c r="M124" s="13" t="str">
-        <x:v>Name spelling unresolved</x:v>
+        <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N124" s="13" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
+        <x:v>Owner corrected Makai and both replies on October 23. Clip 187: I'm sorry, 10-9, my radio cut out. No independent audio review.</x:v>
       </x:c>
       <x:c r="O124" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -13892,7 +13894,7 @@
         <x:v>E177</x:v>
       </x:c>
       <x:c r="B184" s="13" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="C184" s="14" t="n">
         <x:v>46290</x:v>
@@ -13920,16 +13922,16 @@
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="K184" s="13" t="str">
-        <x:v>Hey [Makai?], you in here?</x:v>
+        <x:v>Hey Makai, you in here?</x:v>
       </x:c>
       <x:c r="L184" s="13" t="str">
         <x:v>Yeah, what's up?</x:v>
       </x:c>
       <x:c r="M184" s="13" t="str">
-        <x:v>Name spelling unresolved</x:v>
+        <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N184" s="13" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
+        <x:v>Owner confirmed Makai spelling on October 23. Reply not independently reviewed.</x:v>
       </x:c>
       <x:c r="O184" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -24345,6 +24347,186 @@
       </x:c>
       <x:c r="S361" s="13" t="n">
         <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="82" customHeight="1">
+      <x:c r="A362" s="13" t="str">
+        <x:v>E355</x:v>
+      </x:c>
+      <x:c r="B362" s="13" t="str">
+        <x:v>Makai / Kelepi</x:v>
+      </x:c>
+      <x:c r="C362" s="14" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="D362" s="13" t="n">
+        <x:v>642</x:v>
+      </x:c>
+      <x:c r="E362" s="15" t="n">
+        <x:v>0.6498032407407407</x:v>
+      </x:c>
+      <x:c r="F362" s="16" t="str">
+        <x:v>14590087</x:v>
+      </x:c>
+      <x:c r="G362" s="13" t="n">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="H362" s="15" t="n">
+        <x:v>0.6501388888888889</x:v>
+      </x:c>
+      <x:c r="I362" s="17" t="n">
+        <x:f>ROUND((H362-E362)*86400,0)</x:f>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J362" s="16" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="K362" s="13" t="str">
+        <x:v>Hey, Makai, I don't know if you saw her. There's a redhead that just walked in the Home Depot. She has, like, a gray sweater and her hair up in, like, half a ponytail.</x:v>
+      </x:c>
+      <x:c r="L362" s="13" t="str">
+        <x:v>Negative, [unclear]. I'm talking with the manager right now to see if we can get camera footage.</x:v>
+      </x:c>
+      <x:c r="M362" s="13" t="str">
+        <x:v>Transcript association</x:v>
+      </x:c>
+      <x:c r="N362" s="13" t="str">
+        <x:v>Owner confirmed addressed name as Makai on October 23. Reply follows the named hail; no independent audio review.</x:v>
+      </x:c>
+      <x:c r="O362" s="18" t="str">
+        <x:v>Not reviewed</x:v>
+      </x:c>
+      <x:c r="P362" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-12/dcfems-6001-1789248943.m4a</x:v>
+      </x:c>
+      <x:c r="Q362" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-12/dcfems-6001-1789248972.m4a</x:v>
+      </x:c>
+      <x:c r="R362" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-12</x:v>
+      </x:c>
+      <x:c r="S362" s="13" t="n">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363" ht="82" customHeight="1">
+      <x:c r="A363" s="13" t="str">
+        <x:v>E356</x:v>
+      </x:c>
+      <x:c r="B363" s="13" t="str">
+        <x:v>Makai / Kelepi</x:v>
+      </x:c>
+      <x:c r="C363" s="14" t="n">
+        <x:v>46291</x:v>
+      </x:c>
+      <x:c r="D363" s="13" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="E363" s="15" t="n">
+        <x:v>0.3010185185185185</x:v>
+      </x:c>
+      <x:c r="F363" s="16" t="str">
+        <x:v>14590087</x:v>
+      </x:c>
+      <x:c r="G363" s="13" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="H363" s="15" t="n">
+        <x:v>0.3011226851851852</x:v>
+      </x:c>
+      <x:c r="I363" s="17" t="n">
+        <x:f>ROUND((H363-E363)*86400,0)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J363" s="16" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="K363" s="13" t="str">
+        <x:v>Makai, you want some help on your call?</x:v>
+      </x:c>
+      <x:c r="L363" s="13" t="str">
+        <x:v>Okay, I just cleared the shed. I'm making contact with someone at [USBC / SBC?] right now. It looks like someone backed [the / their?] vehicle into this shed.</x:v>
+      </x:c>
+      <x:c r="M363" s="13" t="str">
+        <x:v>Transcript association</x:v>
+      </x:c>
+      <x:c r="N363" s="13" t="str">
+        <x:v>Owner confirmed addressed name as Makai on October 23. Reply follows the named hail; no independent audio review.</x:v>
+      </x:c>
+      <x:c r="O363" s="18" t="str">
+        <x:v>Not reviewed</x:v>
+      </x:c>
+      <x:c r="P363" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-26/dcfems-6001-1790428408.m4a</x:v>
+      </x:c>
+      <x:c r="Q363" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-26/dcfems-6001-1790428417.m4a</x:v>
+      </x:c>
+      <x:c r="R363" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-26</x:v>
+      </x:c>
+      <x:c r="S363" s="13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="82" customHeight="1">
+      <x:c r="A364" s="13" t="str">
+        <x:v>E357</x:v>
+      </x:c>
+      <x:c r="B364" s="13" t="str">
+        <x:v>Makai / Kelepi</x:v>
+      </x:c>
+      <x:c r="C364" s="14" t="n">
+        <x:v>46296</x:v>
+      </x:c>
+      <x:c r="D364" s="13" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="E364" s="15" t="n">
+        <x:v>0.6967129629629629</x:v>
+      </x:c>
+      <x:c r="F364" s="16" t="str">
+        <x:v>14590087</x:v>
+      </x:c>
+      <x:c r="G364" s="13" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="H364" s="15" t="n">
+        <x:v>0.6967824074074074</x:v>
+      </x:c>
+      <x:c r="I364" s="17" t="n">
+        <x:f>ROUND((H364-E364)*86400,0)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J364" s="16" t="str">
+        <x:v>14590247</x:v>
+      </x:c>
+      <x:c r="K364" s="13" t="str">
+        <x:v>Hey, Makai, are you at the trailer park?</x:v>
+      </x:c>
+      <x:c r="L364" s="13" t="str">
+        <x:v>[Okay?]</x:v>
+      </x:c>
+      <x:c r="M364" s="13" t="str">
+        <x:v>Transcript association</x:v>
+      </x:c>
+      <x:c r="N364" s="13" t="str">
+        <x:v>Owner confirmed addressed name as Makai. Reply is only [Okay?], so responder attribution remains weak. No independent audio review.</x:v>
+      </x:c>
+      <x:c r="O364" s="18" t="str">
+        <x:v>Not reviewed</x:v>
+      </x:c>
+      <x:c r="P364" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-01/dcfems-6001-1790894596.m4a</x:v>
+      </x:c>
+      <x:c r="Q364" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-01/dcfems-6001-1790894602.m4a</x:v>
+      </x:c>
+      <x:c r="R364" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-01</x:v>
+      </x:c>
+      <x:c r="S364" s="13" t="n">
+        <x:v>6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24355,7 +24537,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R124b4b45139146e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d00f139a4f246e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24804,10 +24986,50 @@
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-22/dcfems-6001-1792732459.m4a</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="100" customHeight="1">
+      <x:c r="A26" s="14" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="n">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="str">
+        <x:v>Do you want to take Makai's citizen contact, or do you want me to take it? [Unclear closing].</x:v>
+      </x:c>
+      <x:c r="D26" s="13" t="str">
+        <x:v>Clips 249–252: other radios answer. Clip 253, 14590247: Thanks, [Cox?].</x:v>
+      </x:c>
+      <x:c r="E26" s="13" t="str">
+        <x:v>Owner confirmed Makai spelling, but third-person mention and intervening responders do not establish who used the ID. Not counted as a named response day.</x:v>
+      </x:c>
+      <x:c r="F26" s="13" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-16/dcfems-6001-1789604445.m4a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="100" customHeight="1">
+      <x:c r="A27" s="14" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B27" s="13" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
+        <x:v>Makai, I believe those are Renter's cones.</x:v>
+      </x:c>
+      <x:c r="D27" s="13" t="str">
+        <x:v>Clip 80, 14590247, asks Ethan about cones; clip 82 is an unclear reply. Clip 84 uses the same ID as the named direction in clip 83.</x:v>
+      </x:c>
+      <x:c r="E27" s="13" t="str">
+        <x:v>Owner confirmed Makai and Renter wording. No following response from 14590247 to the named direction, so this is contextual evidence only and is not counted as a response day.</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-15/dcfems-6001-1792104929.m4a</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59d56c3ed05c48cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4efe34037cb418a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24882,7 +25104,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="str">
-        <x:v>Exclusions: third-person mentions, unrelated replies, missing/invalid IDs, combined-source clips, and explicit replies on another officer’s behalf. No voice recognition used.</x:v>
+        <x:v>Excluded: third-person mentions, unrelated responses, invalid IDs, combined source IDs and explicit replies on behalf of others. October 23 owner corrections resolve Makai spelling for 14590247; three reply pairs added, plus September 16 and October 15 context recorded in Exceptions.</x:v>
       </x:c>
       <x:c r="B7" s="2"/>
       <x:c r="C7" s="2"/>
@@ -25772,7 +25994,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8af3458909b429c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2560bd793f394993"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand clear recurring radio-ID associations and normalize Somerville in the reference workbook
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R90044babe3414fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R0afcf177922b4fc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R57ac693bd0ef42b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R90619854ad91468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="Rc125496310bb47a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R382100e9d162419b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R5bbd8e9812ab42e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="Ref97e9987db4469f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3350,7 +3350,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R628287340a7d4bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bb55cbe9d3d422d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3604,7 +3604,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="K8" s="13" t="str">
-        <x:v>[Somerville/Summerville?], where are you parked?</x:v>
+        <x:v>Somerville, where are you parked?</x:v>
       </x:c>
       <x:c r="L8" s="13" t="str">
         <x:v>I'm on the west side of Building C. I'm actually parked pretty close to you. I can see you now. I'm on the north side of the building right now.</x:v>
@@ -9172,7 +9172,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="K103" s="13" t="str">
-        <x:v>Hey, [Somerville?], I’m on my way down right now.</x:v>
+        <x:v>Hey, Somerville, I’m on my way down right now.</x:v>
       </x:c>
       <x:c r="L103" s="13" t="str">
         <x:v>We’ll wait for you.</x:v>
@@ -9230,7 +9230,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K104" s="13" t="str">
-        <x:v>[Summerville?], you're taking the next Spanish call.</x:v>
+        <x:v>Somerville, you're taking the next Spanish call.</x:v>
       </x:c>
       <x:c r="L104" s="13" t="str">
         <x:v>No, gracias.</x:v>
@@ -13396,7 +13396,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K175" s="13" t="str">
-        <x:v>Give me another one, [Summerville?].</x:v>
+        <x:v>Give me another one, Somerville.</x:v>
       </x:c>
       <x:c r="L175" s="13" t="str">
         <x:v>I should be all right. She's being super cooperative. Her dad's gonna come pick her up, and then I'll do the inventory. I think [you/it?] should work out with timing if everybody else [is/isn't?] busy.</x:v>
@@ -13454,7 +13454,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K176" s="13" t="str">
-        <x:v>Aren't you [at?] In-N-Out, [Summerville?]?</x:v>
+        <x:v>Aren't you [at?] In-N-Out, Somerville?</x:v>
       </x:c>
       <x:c r="L176" s="13" t="str">
         <x:v>Yeah, but I think everybody else is at the PD, so...</x:v>
@@ -13512,7 +13512,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="K177" s="13" t="str">
-        <x:v>[Somerville/Summerville?], starting to get busy down there yet?</x:v>
+        <x:v>Somerville, starting to get busy down there yet?</x:v>
       </x:c>
       <x:c r="L177" s="13" t="str">
         <x:v>Yeah, it's pretty busy, but it's not as bad as the other week when we got called down here. I think most of the [Lone Peak?] kids showed up, saw how many AF kids there were, and left.</x:v>
@@ -14216,7 +14216,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K189" s="13" t="str">
-        <x:v>Yeah, I’d say just give it like ten minutes max, [Somerville/Summerville?], and then we can [jam/check/chat?].</x:v>
+        <x:v>Yeah, I’d say just give it like ten minutes max, Somerville, and then we can [jam/check/chat?].</x:v>
       </x:c>
       <x:c r="L189" s="13" t="str">
         <x:v>Sounds good.</x:v>
@@ -16558,7 +16558,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="K229" s="13" t="str">
-        <x:v>Hey [Somerville?]</x:v>
+        <x:v>Hey Somerville</x:v>
       </x:c>
       <x:c r="L229" s="13" t="str">
         <x:v>Go ahead.</x:v>
@@ -16616,7 +16616,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K230" s="13" t="str">
-        <x:v>Well [Somerville?], since you were cheering for Lehi, you have to sit in the hall and eat your food.</x:v>
+        <x:v>Well Somerville, since you were cheering for Lehi, you have to sit in the hall and eat your food.</x:v>
       </x:c>
       <x:c r="L230" s="13" t="str">
         <x:v>Pretty sure Lehi won, so I think that means you guys have to sit in the hall.</x:v>
@@ -16850,7 +16850,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K234" s="13" t="str">
-        <x:v>Hey [Somerville?], that Jeep said it passed you out on North County.</x:v>
+        <x:v>Hey Somerville, that Jeep said it passed you out on North County.</x:v>
       </x:c>
       <x:c r="L234" s="13" t="str">
         <x:v>Sorry, I was just finishing up my traffic stop. What's going on?</x:v>
@@ -18498,7 +18498,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K262" s="13" t="str">
-        <x:v>[Summerville?], I'm going to go past the house on this street and go up to 350 South to see if I see the car in the driveway.</x:v>
+        <x:v>Somerville, I'm going to go past the house on this street and go up to 350 South to see if I see the car in the driveway.</x:v>
       </x:c>
       <x:c r="L262" s="13" t="str">
         <x:v>I'm on the phone, [unclear wording] right now.</x:v>
@@ -18556,7 +18556,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K263" s="13" t="str">
-        <x:v>[Hey / okay], [Summerville], that truck.</x:v>
+        <x:v>[Hey / okay], Somerville, that truck.</x:v>
       </x:c>
       <x:c r="L263" s="13" t="str">
         <x:v>I was too distracted by his extremely bright headlights, but it might have been.</x:v>
@@ -24142,7 +24142,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="K358" s="13" t="str">
-        <x:v>Hey, [Somerville/Summerville?], also if you can grab the second wrap, just in case.</x:v>
+        <x:v>Hey, Somerville, also if you can grab the second wrap, just in case.</x:v>
       </x:c>
       <x:c r="L358" s="13" t="str">
         <x:v>Copy.</x:v>
@@ -24537,7 +24537,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d00f139a4f246e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raec8db8254b1423c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25029,7 +25029,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4efe34037cb418a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10702eef2e594d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25994,7 +25994,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2560bd793f394993"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5ccc77407ec4e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate Tanner Ballamis radio evidence and refresh response-day workbook
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="Rc125496310bb47a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R382100e9d162419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R5bbd8e9812ab42e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="Ref97e9987db4469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="Rc6833c13207a40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Rf8a8b0e1e2e94f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="Rfcfb374cfac0470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R2f445cbd4b31404b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -194,8 +194,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RadioFindings" displayName="RadioFindings" ref="A9:L82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A9:L82"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RadioFindings" displayName="RadioFindings" ref="A9:L80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Name in exchange"/>
     <x:tableColumn id="2" name="Responding radio ID"/>
@@ -215,8 +214,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S364" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:S364"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S371" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:S371"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Name in exchange"/>
@@ -546,7 +545,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 357 selected exchanges.</x:v>
+        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 364 selected exchanges.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -578,7 +577,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="str">
-        <x:v>Roster candidates are inferences from the site roster. Keep first-name and conflicting matches unresolved until the linked audio is checked.</x:v>
+        <x:v>Roster candidates are inferences from the site roster unless owner identification is noted. Tanner Ballamis groups Tanner, T-Ball and G-Ball.</x:v>
       </x:c>
       <x:c r="B7" s="2"/>
       <x:c r="C7" s="2"/>
@@ -652,7 +651,7 @@
         <x:v>14580155</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A10,Exchanges!$J$8:$J$364,B10)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A10,Exchanges!$J$8:$J$371,B10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -687,7 +686,7 @@
         <x:v>14590020</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A11,Exchanges!$J$8:$J$364,B11)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A11,Exchanges!$J$8:$J$371,B11)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -722,7 +721,7 @@
         <x:v>14590089</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A12,Exchanges!$J$8:$J$364,B12)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A12,Exchanges!$J$8:$J$371,B12)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -757,7 +756,7 @@
         <x:v>14590111</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A13,Exchanges!$J$8:$J$364,B13)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A13,Exchanges!$J$8:$J$371,B13)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -792,7 +791,7 @@
         <x:v>14580152</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A14,Exchanges!$J$8:$J$364,B14)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A14,Exchanges!$J$8:$J$371,B14)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -827,7 +826,7 @@
         <x:v>14590098</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A15,Exchanges!$J$8:$J$364,B15)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A15,Exchanges!$J$8:$J$371,B15)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -864,7 +863,7 @@
         <x:v>14590107</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A16,Exchanges!$J$8:$J$364,B16)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A16,Exchanges!$J$8:$J$371,B16)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -899,7 +898,7 @@
         <x:v>14590104</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A17,Exchanges!$J$8:$J$364,B17)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A17,Exchanges!$J$8:$J$371,B17)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
@@ -936,7 +935,7 @@
         <x:v>14590200</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A18,Exchanges!$J$8:$J$364,B18)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A18,Exchanges!$J$8:$J$371,B18)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
@@ -973,7 +972,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A19,Exchanges!$J$8:$J$364,B19)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A19,Exchanges!$J$8:$J$371,B19)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
@@ -1012,7 +1011,7 @@
         <x:v>14590118</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A20,Exchanges!$J$8:$J$364,B20)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A20,Exchanges!$J$8:$J$371,B20)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
@@ -1049,7 +1048,7 @@
         <x:v>14590088</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A21,Exchanges!$J$8:$J$364,B21)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A21,Exchanges!$J$8:$J$371,B21)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
@@ -1086,7 +1085,7 @@
         <x:v>14590117</x:v>
       </x:c>
       <x:c r="C22" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A22,Exchanges!$J$8:$J$364,B22)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A22,Exchanges!$J$8:$J$371,B22)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
@@ -1121,7 +1120,7 @@
         <x:v>14590320</x:v>
       </x:c>
       <x:c r="C23" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A23,Exchanges!$J$8:$J$364,B23)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A23,Exchanges!$J$8:$J$371,B23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="10" t="n">
@@ -1156,7 +1155,7 @@
         <x:v>14590084</x:v>
       </x:c>
       <x:c r="C24" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A24,Exchanges!$J$8:$J$364,B24)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A24,Exchanges!$J$8:$J$371,B24)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D24" s="10" t="n">
@@ -1193,7 +1192,7 @@
         <x:v>14590237</x:v>
       </x:c>
       <x:c r="C25" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A25,Exchanges!$J$8:$J$364,B25)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A25,Exchanges!$J$8:$J$371,B25)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
@@ -1228,7 +1227,7 @@
         <x:v>14590315</x:v>
       </x:c>
       <x:c r="C26" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A26,Exchanges!$J$8:$J$364,B26)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A26,Exchanges!$J$8:$J$371,B26)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
@@ -1263,7 +1262,7 @@
         <x:v>14590162</x:v>
       </x:c>
       <x:c r="C27" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A27,Exchanges!$J$8:$J$364,B27)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A27,Exchanges!$J$8:$J$371,B27)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
@@ -1298,7 +1297,7 @@
         <x:v>14590081</x:v>
       </x:c>
       <x:c r="C28" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A28,Exchanges!$J$8:$J$364,B28)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A28,Exchanges!$J$8:$J$371,B28)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
@@ -1333,7 +1332,7 @@
         <x:v>14590102</x:v>
       </x:c>
       <x:c r="C29" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A29,Exchanges!$J$8:$J$364,B29)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A29,Exchanges!$J$8:$J$371,B29)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
@@ -1368,7 +1367,7 @@
         <x:v>14590344</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A30,Exchanges!$J$8:$J$364,B30)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A30,Exchanges!$J$8:$J$371,B30)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
@@ -1405,7 +1404,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C31" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A31,Exchanges!$J$8:$J$364,B31)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A31,Exchanges!$J$8:$J$371,B31)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
@@ -1444,7 +1443,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C32" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A32,Exchanges!$J$8:$J$364,B32)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A32,Exchanges!$J$8:$J$371,B32)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
@@ -1481,7 +1480,7 @@
         <x:v>14590087</x:v>
       </x:c>
       <x:c r="C33" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A33,Exchanges!$J$8:$J$364,B33)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A33,Exchanges!$J$8:$J$371,B33)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
@@ -1516,7 +1515,7 @@
         <x:v>14590044</x:v>
       </x:c>
       <x:c r="C34" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A34,Exchanges!$J$8:$J$364,B34)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A34,Exchanges!$J$8:$J$371,B34)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
@@ -1551,7 +1550,7 @@
         <x:v>14590123</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A35,Exchanges!$J$8:$J$364,B35)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A35,Exchanges!$J$8:$J$371,B35)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
@@ -1586,7 +1585,7 @@
         <x:v>14590037</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A36,Exchanges!$J$8:$J$364,B36)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A36,Exchanges!$J$8:$J$371,B36)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
@@ -1623,7 +1622,7 @@
         <x:v>14590095</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A37,Exchanges!$J$8:$J$364,B37)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A37,Exchanges!$J$8:$J$371,B37)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
@@ -1660,7 +1659,7 @@
         <x:v>14590099</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A38,Exchanges!$J$8:$J$364,B38)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A38,Exchanges!$J$8:$J$371,B38)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D38" s="10" t="n">
@@ -1697,7 +1696,7 @@
         <x:v>14590207</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A39,Exchanges!$J$8:$J$364,B39)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A39,Exchanges!$J$8:$J$371,B39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
@@ -1734,7 +1733,7 @@
         <x:v>14590067</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A40,Exchanges!$J$8:$J$364,B40)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A40,Exchanges!$J$8:$J$371,B40)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
@@ -1771,7 +1770,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A41,Exchanges!$J$8:$J$364,B41)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A41,Exchanges!$J$8:$J$371,B41)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
@@ -1806,7 +1805,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A42,Exchanges!$J$8:$J$364,B42)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A42,Exchanges!$J$8:$J$371,B42)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
@@ -1841,7 +1840,7 @@
         <x:v>14590038</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A43,Exchanges!$J$8:$J$364,B43)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A43,Exchanges!$J$8:$J$371,B43)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
@@ -1876,7 +1875,7 @@
         <x:v>14590345</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A44,Exchanges!$J$8:$J$364,B44)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A44,Exchanges!$J$8:$J$371,B44)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
@@ -1911,7 +1910,7 @@
         <x:v>14590079</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A45,Exchanges!$J$8:$J$364,B45)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A45,Exchanges!$J$8:$J$371,B45)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
@@ -1946,7 +1945,7 @@
         <x:v>14590026</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A46,Exchanges!$J$8:$J$364,B46)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A46,Exchanges!$J$8:$J$371,B46)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
@@ -1983,7 +1982,7 @@
         <x:v>14590031</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A47,Exchanges!$J$8:$J$364,B47)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A47,Exchanges!$J$8:$J$371,B47)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
@@ -2020,7 +2019,7 @@
         <x:v>14590101</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A48,Exchanges!$J$8:$J$364,B48)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A48,Exchanges!$J$8:$J$371,B48)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
@@ -2057,7 +2056,7 @@
         <x:v>14590103</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A49,Exchanges!$J$8:$J$364,B49)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A49,Exchanges!$J$8:$J$371,B49)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
@@ -2094,7 +2093,7 @@
         <x:v>14590043</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A50,Exchanges!$J$8:$J$364,B50)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A50,Exchanges!$J$8:$J$371,B50)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D50" s="10" t="n">
@@ -2131,7 +2130,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A51,Exchanges!$J$8:$J$364,B51)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A51,Exchanges!$J$8:$J$371,B51)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D51" s="10" t="n">
@@ -2170,7 +2169,7 @@
         <x:v>14590266</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A52,Exchanges!$J$8:$J$364,B52)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A52,Exchanges!$J$8:$J$371,B52)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D52" s="10" t="n">
@@ -2205,7 +2204,7 @@
         <x:v>14590219</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A53,Exchanges!$J$8:$J$364,B53)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A53,Exchanges!$J$8:$J$371,B53)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D53" s="10" t="n">
@@ -2240,7 +2239,7 @@
         <x:v>14590066</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A54,Exchanges!$J$8:$J$364,B54)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A54,Exchanges!$J$8:$J$371,B54)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
@@ -2277,7 +2276,7 @@
         <x:v>14590090</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A55,Exchanges!$J$8:$J$364,B55)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A55,Exchanges!$J$8:$J$371,B55)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
@@ -2314,7 +2313,7 @@
         <x:v>14590268</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A56,Exchanges!$J$8:$J$364,B56)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A56,Exchanges!$J$8:$J$371,B56)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
@@ -2351,7 +2350,7 @@
         <x:v>14590085</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A57,Exchanges!$J$8:$J$364,B57)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A57,Exchanges!$J$8:$J$371,B57)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D57" s="10" t="n">
@@ -2388,7 +2387,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A58,Exchanges!$J$8:$J$364,B58)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A58,Exchanges!$J$8:$J$371,B58)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D58" s="10" t="n">
@@ -2427,7 +2426,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A59,Exchanges!$J$8:$J$364,B59)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A59,Exchanges!$J$8:$J$371,B59)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="10" t="n">
@@ -2466,7 +2465,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A60,Exchanges!$J$8:$J$364,B60)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A60,Exchanges!$J$8:$J$371,B60)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D60" s="10" t="n">
@@ -2505,7 +2504,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A61,Exchanges!$J$8:$J$364,B61)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A61,Exchanges!$J$8:$J$371,B61)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
@@ -2544,7 +2543,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A62,Exchanges!$J$8:$J$364,B62)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A62,Exchanges!$J$8:$J$371,B62)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
@@ -2583,7 +2582,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A63,Exchanges!$J$8:$J$364,B63)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A63,Exchanges!$J$8:$J$371,B63)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
@@ -2622,7 +2621,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A64,Exchanges!$J$8:$J$364,B64)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A64,Exchanges!$J$8:$J$371,B64)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
@@ -2661,7 +2660,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A65,Exchanges!$J$8:$J$364,B65)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A65,Exchanges!$J$8:$J$371,B65)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
@@ -2700,7 +2699,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A66,Exchanges!$J$8:$J$364,B66)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A66,Exchanges!$J$8:$J$371,B66)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D66" s="10" t="n">
@@ -2739,7 +2738,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A67,Exchanges!$J$8:$J$364,B67)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A67,Exchanges!$J$8:$J$371,B67)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D67" s="10" t="n">
@@ -2776,7 +2775,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A68,Exchanges!$J$8:$J$364,B68)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A68,Exchanges!$J$8:$J$371,B68)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
@@ -2815,7 +2814,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A69,Exchanges!$J$8:$J$364,B69)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A69,Exchanges!$J$8:$J$371,B69)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D69" s="10" t="n">
@@ -2854,7 +2853,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C70" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A70,Exchanges!$J$8:$J$364,B70)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A70,Exchanges!$J$8:$J$371,B70)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D70" s="10" t="n">
@@ -2893,7 +2892,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C71" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A71,Exchanges!$J$8:$J$364,B71)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A71,Exchanges!$J$8:$J$371,B71)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D71" s="10" t="n">
@@ -2930,7 +2929,7 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="C72" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A72,Exchanges!$J$8:$J$364,B72)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A72,Exchanges!$J$8:$J$371,B72)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D72" s="10" t="n">
@@ -2967,7 +2966,7 @@
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="C73" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A73,Exchanges!$J$8:$J$364,B73)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A73,Exchanges!$J$8:$J$371,B73)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D73" s="10" t="n">
@@ -3004,7 +3003,7 @@
         <x:v>14590112</x:v>
       </x:c>
       <x:c r="C74" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A74,Exchanges!$J$8:$J$364,B74)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A74,Exchanges!$J$8:$J$371,B74)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D74" s="10" t="n">
@@ -3041,7 +3040,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C75" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A75,Exchanges!$J$8:$J$364,B75)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A75,Exchanges!$J$8:$J$371,B75)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D75" s="10" t="n">
@@ -3080,7 +3079,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C76" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A76,Exchanges!$J$8:$J$364,B76)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A76,Exchanges!$J$8:$J$371,B76)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D76" s="10" t="n">
@@ -3119,7 +3118,7 @@
         <x:v>14590097</x:v>
       </x:c>
       <x:c r="C77" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A77,Exchanges!$J$8:$J$364,B77)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A77,Exchanges!$J$8:$J$371,B77)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D77" s="10" t="n">
@@ -3148,54 +3147,52 @@
         <x:v>E345</x:v>
       </x:c>
     </x:row>
-    <x:row r="78">
+    <x:row r="78" ht="34" customHeight="1">
       <x:c r="A78" s="10" t="str">
-        <x:v>D-ball (unclear)</x:v>
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
       </x:c>
       <x:c r="B78" s="11" t="str">
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C78" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A78,Exchanges!$J$8:$J$364,B78)</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A78,Exchanges!$J$8:$J$371,B78)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D78" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E78" s="12" t="n">
-        <x:v>46317</x:v>
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="F78" s="12" t="n">
         <x:v>46317</x:v>
       </x:c>
       <x:c r="G78" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H78" s="10" t="str">
-        <x:v>G-ball (unclear), Tanner (unclear)</x:v>
-      </x:c>
+        <x:v>Repeated across days</x:v>
+      </x:c>
+      <x:c r="H78" s="10" t="str"/>
       <x:c r="I78" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Tanner M. Ballamis</x:v>
       </x:c>
       <x:c r="J78" s="10" t="str">
-        <x:v>Uncertain name or nickname. Kept separate from similar names pending audio review.</x:v>
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. ID association, not permanent ownership.</x:v>
       </x:c>
       <x:c r="K78" s="10" t="str">
-        <x:v>2026-10-22</x:v>
+        <x:v>2026-09-19, 2026-10-03, 2026-10-21, 2026-10-22</x:v>
       </x:c>
       <x:c r="L78" s="10" t="str">
-        <x:v>E349</x:v>
+        <x:v>E349, E350, E353, E358, E359, E360, E361, E362, E363, E364</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="10" t="str">
-        <x:v>Tanner (unclear)</x:v>
+        <x:v>Peter (unclear)</x:v>
       </x:c>
       <x:c r="B79" s="11" t="str">
-        <x:v>14580151</x:v>
+        <x:v>14590114</x:v>
       </x:c>
       <x:c r="C79" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A79,Exchanges!$J$8:$J$364,B79)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A79,Exchanges!$J$8:$J$371,B79)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="10" t="n">
@@ -3211,7 +3208,7 @@
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H79" s="10" t="str">
-        <x:v>D-ball (unclear), G-ball (unclear)</x:v>
+        <x:v>Pat (unclear), Pitt</x:v>
       </x:c>
       <x:c r="I79" s="10" t="str">
         <x:v>Unresolved</x:v>
@@ -3223,18 +3220,18 @@
         <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="L79" s="10" t="str">
-        <x:v>E350</x:v>
+        <x:v>E352</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="10" t="str">
-        <x:v>Peter (unclear)</x:v>
+        <x:v>Pat (unclear)</x:v>
       </x:c>
       <x:c r="B80" s="11" t="str">
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C80" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A80,Exchanges!$J$8:$J$364,B80)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A80,Exchanges!$J$8:$J$371,B80)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D80" s="10" t="n">
@@ -3250,7 +3247,7 @@
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H80" s="10" t="str">
-        <x:v>Pat (unclear), Pitt</x:v>
+        <x:v>Peter (unclear), Pitt</x:v>
       </x:c>
       <x:c r="I80" s="10" t="str">
         <x:v>Unresolved</x:v>
@@ -3262,86 +3259,36 @@
         <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="L80" s="10" t="str">
-        <x:v>E352</x:v>
+        <x:v>E354</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="10" t="str">
-        <x:v>G-ball (unclear)</x:v>
-      </x:c>
-      <x:c r="B81" s="11" t="str">
-        <x:v>14580151</x:v>
-      </x:c>
-      <x:c r="C81" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A81,Exchanges!$J$8:$J$364,B81)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D81" s="10" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E81" s="12" t="n">
-        <x:v>46317</x:v>
-      </x:c>
-      <x:c r="F81" s="12" t="n">
-        <x:v>46317</x:v>
-      </x:c>
-      <x:c r="G81" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H81" s="10" t="str">
-        <x:v>D-ball (unclear), Tanner (unclear)</x:v>
-      </x:c>
-      <x:c r="I81" s="10" t="str">
-        <x:v>Unresolved</x:v>
-      </x:c>
-      <x:c r="J81" s="10" t="str">
-        <x:v>Uncertain name or nickname. Kept separate from similar names pending audio review.</x:v>
-      </x:c>
-      <x:c r="K81" s="10" t="str">
-        <x:v>2026-10-22</x:v>
-      </x:c>
-      <x:c r="L81" s="10" t="str">
-        <x:v>E353</x:v>
-      </x:c>
+      <x:c r="A81" s="10"/>
+      <x:c r="B81" s="11"/>
+      <x:c r="C81" s="10"/>
+      <x:c r="D81" s="10"/>
+      <x:c r="E81" s="12"/>
+      <x:c r="F81" s="12"/>
+      <x:c r="G81" s="10"/>
+      <x:c r="H81" s="10"/>
+      <x:c r="I81" s="10"/>
+      <x:c r="J81" s="10"/>
+      <x:c r="K81" s="10"/>
+      <x:c r="L81" s="10"/>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="10" t="str">
-        <x:v>Pat (unclear)</x:v>
-      </x:c>
-      <x:c r="B82" s="11" t="str">
-        <x:v>14590114</x:v>
-      </x:c>
-      <x:c r="C82" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$364,A82,Exchanges!$J$8:$J$364,B82)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D82" s="10" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E82" s="12" t="n">
-        <x:v>46317</x:v>
-      </x:c>
-      <x:c r="F82" s="12" t="n">
-        <x:v>46317</x:v>
-      </x:c>
-      <x:c r="G82" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H82" s="10" t="str">
-        <x:v>Peter (unclear), Pitt</x:v>
-      </x:c>
-      <x:c r="I82" s="10" t="str">
-        <x:v>Unresolved</x:v>
-      </x:c>
-      <x:c r="J82" s="10" t="str">
-        <x:v>Uncertain name or nickname. Kept separate from similar names pending audio review.</x:v>
-      </x:c>
-      <x:c r="K82" s="10" t="str">
-        <x:v>2026-10-22</x:v>
-      </x:c>
-      <x:c r="L82" s="10" t="str">
-        <x:v>E354</x:v>
-      </x:c>
+      <x:c r="A82" s="10"/>
+      <x:c r="B82" s="11"/>
+      <x:c r="C82" s="10"/>
+      <x:c r="D82" s="10"/>
+      <x:c r="E82" s="12"/>
+      <x:c r="F82" s="12"/>
+      <x:c r="G82" s="10"/>
+      <x:c r="H82" s="10"/>
+      <x:c r="I82" s="10"/>
+      <x:c r="J82" s="10"/>
+      <x:c r="K82" s="10"/>
+      <x:c r="L82" s="10"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="G10:G73">
@@ -3350,7 +3297,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bb55cbe9d3d422d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8054ef3d10874730"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3470,7 +3417,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Quotes reproduce existing transcripts, including bracketed uncertainty. A transcript marked validated in the archive was not rechecked by listening here.</x:v>
+        <x:v>Quotes retain transcript uncertainty. October 27 owner identification groups Tanner, T-Ball and G-Ball as Tanner Ballamis; the D-Ball reading is corrected to T-Ball.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -23994,7 +23941,7 @@
         <x:v>E349</x:v>
       </x:c>
       <x:c r="B356" s="13" t="str">
-        <x:v>D-ball (unclear)</x:v>
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
       </x:c>
       <x:c r="C356" s="14" t="n">
         <x:v>46317</x:v>
@@ -24022,19 +23969,19 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="K356" s="13" t="str">
-        <x:v>[D-ball?], if you can hold the [1-4?] corner, that would be awesome.</x:v>
+        <x:v>T-Ball, if you can hold the [1-4?] corner, that would be awesome.</x:v>
       </x:c>
       <x:c r="L356" s="13" t="str">
         <x:v>Sounds good.</x:v>
       </x:c>
       <x:c r="M356" s="13" t="str">
-        <x:v>Transcript association</x:v>
+        <x:v>Owner-identified association</x:v>
       </x:c>
       <x:c r="N356" s="13" t="str">
-        <x:v>Nickname uncertain. No full-name identity assigned. Archive verification: question unverified, reply unverified. Not re-listened for this update.</x:v>
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. The former D-Ball reading is corrected to T-Ball. Other words remain unverified.</x:v>
       </x:c>
       <x:c r="O356" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner identification</x:v>
       </x:c>
       <x:c r="P356" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-22/dcfems-6001-1792711182.m4a</x:v>
@@ -24054,7 +24001,7 @@
         <x:v>E350</x:v>
       </x:c>
       <x:c r="B357" s="13" t="str">
-        <x:v>Tanner (unclear)</x:v>
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
       </x:c>
       <x:c r="C357" s="14" t="n">
         <x:v>46317</x:v>
@@ -24088,13 +24035,13 @@
         <x:v>I don't know why I'm not hearing anything. What's up?</x:v>
       </x:c>
       <x:c r="M357" s="13" t="str">
-        <x:v>Transcript association</x:v>
+        <x:v>Owner-identified association</x:v>
       </x:c>
       <x:c r="N357" s="13" t="str">
-        <x:v>Name uncertain; responder asks for repetition. No full-name identity assigned. Archive verification: question unverified, reply unverified. Not re-listened for this update.</x:v>
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. The former D-Ball reading is corrected to T-Ball. Other words remain unverified.</x:v>
       </x:c>
       <x:c r="O357" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner identification</x:v>
       </x:c>
       <x:c r="P357" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-22/dcfems-6001-1792711373.m4a</x:v>
@@ -24234,7 +24181,7 @@
         <x:v>E353</x:v>
       </x:c>
       <x:c r="B360" s="13" t="str">
-        <x:v>G-ball (unclear)</x:v>
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
       </x:c>
       <x:c r="C360" s="14" t="n">
         <x:v>46317</x:v>
@@ -24268,13 +24215,13 @@
         <x:v>700 West, [200 South?]. Getting pretty close.</x:v>
       </x:c>
       <x:c r="M360" s="13" t="str">
-        <x:v>Transcript association</x:v>
+        <x:v>Owner-identified association</x:v>
       </x:c>
       <x:c r="N360" s="13" t="str">
-        <x:v>Nickname uncertain. Kept separate from D-ball and Tanner. Archive verification: question unverified, reply unverified. Not re-listened for this update.</x:v>
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. The former D-Ball reading is corrected to T-Ball. Other words remain unverified.</x:v>
       </x:c>
       <x:c r="O360" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner identification</x:v>
       </x:c>
       <x:c r="P360" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-22/dcfems-6001-1792722875.m4a</x:v>
@@ -24527,6 +24474,426 @@
       </x:c>
       <x:c r="S364" s="13" t="n">
         <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365">
+      <x:c r="A365" s="13" t="str">
+        <x:v>E358</x:v>
+      </x:c>
+      <x:c r="B365" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C365" s="14" t="n">
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="D365" s="13" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E365" s="15" t="n">
+        <x:v>0.085625</x:v>
+      </x:c>
+      <x:c r="F365" s="16" t="str">
+        <x:v>14590073</x:v>
+      </x:c>
+      <x:c r="G365" s="13" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H365" s="15" t="n">
+        <x:v>0.08570601851851851</x:v>
+      </x:c>
+      <x:c r="I365" s="17" t="n">
+        <x:f>ROUND((H365-E365)*86400,0)</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J365" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K365" s="13" t="str">
+        <x:v>[T-ball?], if you want to stop that truck, I can take this alarm.</x:v>
+      </x:c>
+      <x:c r="L365" s="13" t="str">
+        <x:v>That would be great. Thank you.</x:v>
+      </x:c>
+      <x:c r="M365" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N365" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question unverified, reply unverified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O365" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P365" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789804998.m4a</x:v>
+      </x:c>
+      <x:c r="Q365" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789805005.m4a</x:v>
+      </x:c>
+      <x:c r="R365" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-19</x:v>
+      </x:c>
+      <x:c r="S365" s="13" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366">
+      <x:c r="A366" s="13" t="str">
+        <x:v>E359</x:v>
+      </x:c>
+      <x:c r="B366" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C366" s="14" t="n">
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="D366" s="13" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="E366" s="15" t="n">
+        <x:v>0.7708101851851852</x:v>
+      </x:c>
+      <x:c r="F366" s="16" t="str">
+        <x:v>14590073</x:v>
+      </x:c>
+      <x:c r="G366" s="13" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="H366" s="15" t="n">
+        <x:v>0.7709953703703704</x:v>
+      </x:c>
+      <x:c r="I366" s="17" t="n">
+        <x:f>ROUND((H366-E366)*86400,0)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J366" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K366" s="13" t="str">
+        <x:v>Hey, [T-ball?], so it’s not a residence, it’s a commercial office, and I just got off the phone with RP. If it’s open, he wants us to clear it.</x:v>
+      </x:c>
+      <x:c r="L366" s="13" t="str">
+        <x:v>Sounds good.</x:v>
+      </x:c>
+      <x:c r="M366" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N366" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question unverified, reply unverified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O366" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P366" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789864198.m4a</x:v>
+      </x:c>
+      <x:c r="Q366" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789864214.m4a</x:v>
+      </x:c>
+      <x:c r="R366" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-19</x:v>
+      </x:c>
+      <x:c r="S366" s="13" t="n">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367">
+      <x:c r="A367" s="13" t="str">
+        <x:v>E360</x:v>
+      </x:c>
+      <x:c r="B367" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C367" s="14" t="n">
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="D367" s="13" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="E367" s="15" t="n">
+        <x:v>0.8257291666666666</x:v>
+      </x:c>
+      <x:c r="F367" s="16" t="str">
+        <x:v>14590073</x:v>
+      </x:c>
+      <x:c r="G367" s="13" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="H367" s="15" t="n">
+        <x:v>0.8258449074074075</x:v>
+      </x:c>
+      <x:c r="I367" s="17" t="n">
+        <x:f>ROUND((H367-E367)*86400,0)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J367" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K367" s="13" t="str">
+        <x:v>[T-ball?], [what’s?] your 20?</x:v>
+      </x:c>
+      <x:c r="L367" s="13" t="str">
+        <x:v>[100 East and Main?]</x:v>
+      </x:c>
+      <x:c r="M367" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N367" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question unverified, reply unverified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O367" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P367" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789868943.m4a</x:v>
+      </x:c>
+      <x:c r="Q367" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789868953.m4a</x:v>
+      </x:c>
+      <x:c r="R367" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-19</x:v>
+      </x:c>
+      <x:c r="S367" s="13" t="n">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368">
+      <x:c r="A368" s="13" t="str">
+        <x:v>E361</x:v>
+      </x:c>
+      <x:c r="B368" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C368" s="14" t="n">
+        <x:v>46284</x:v>
+      </x:c>
+      <x:c r="D368" s="13" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="E368" s="15" t="n">
+        <x:v>0.8812152777777778</x:v>
+      </x:c>
+      <x:c r="F368" s="16" t="str">
+        <x:v>14590114</x:v>
+      </x:c>
+      <x:c r="G368" s="13" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="H368" s="15" t="n">
+        <x:v>0.8812847222222222</x:v>
+      </x:c>
+      <x:c r="I368" s="17" t="n">
+        <x:f>ROUND((H368-E368)*86400,0)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J368" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K368" s="13" t="str">
+        <x:v>Hey [T-ball?], what’s going on?</x:v>
+      </x:c>
+      <x:c r="L368" s="13" t="str">
+        <x:v>[I’m/we’re?] turning onto Center Street now.</x:v>
+      </x:c>
+      <x:c r="M368" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N368" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question unverified, reply unverified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O368" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P368" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789873737.m4a</x:v>
+      </x:c>
+      <x:c r="Q368" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-19/dcfems-6001-1789873743.m4a</x:v>
+      </x:c>
+      <x:c r="R368" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-09-19</x:v>
+      </x:c>
+      <x:c r="S368" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369">
+      <x:c r="A369" s="13" t="str">
+        <x:v>E362</x:v>
+      </x:c>
+      <x:c r="B369" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C369" s="14" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="D369" s="13" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E369" s="15" t="n">
+        <x:v>0.0425462962962963</x:v>
+      </x:c>
+      <x:c r="F369" s="16" t="str">
+        <x:v>14590114</x:v>
+      </x:c>
+      <x:c r="G369" s="13" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H369" s="15" t="n">
+        <x:v>0.042638888888888886</x:v>
+      </x:c>
+      <x:c r="I369" s="17" t="n">
+        <x:f>ROUND((H369-E369)*86400,0)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J369" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K369" s="13" t="str">
+        <x:v>Get [him / them], T-ball.</x:v>
+      </x:c>
+      <x:c r="L369" s="13" t="str">
+        <x:v>On it.</x:v>
+      </x:c>
+      <x:c r="M369" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N369" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question unverified, reply unverified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O369" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P369" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-03/dcfems-6001-1791010876.m4a</x:v>
+      </x:c>
+      <x:c r="Q369" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-03/dcfems-6001-1791010884.m4a</x:v>
+      </x:c>
+      <x:c r="R369" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-03</x:v>
+      </x:c>
+      <x:c r="S369" s="13" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370">
+      <x:c r="A370" s="13" t="str">
+        <x:v>E363</x:v>
+      </x:c>
+      <x:c r="B370" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C370" s="14" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="D370" s="13" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="E370" s="15" t="n">
+        <x:v>0.7766898148148148</x:v>
+      </x:c>
+      <x:c r="F370" s="16" t="str">
+        <x:v>14590073</x:v>
+      </x:c>
+      <x:c r="G370" s="13" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="H370" s="15" t="n">
+        <x:v>0.7770717592592593</x:v>
+      </x:c>
+      <x:c r="I370" s="17" t="n">
+        <x:f>ROUND((H370-E370)*86400,0)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J370" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K370" s="13" t="str">
+        <x:v>T-ball, will you confirm Lizzie's name, spelling, everything?</x:v>
+      </x:c>
+      <x:c r="L370" s="13" t="str">
+        <x:v>Her real name is Elizabeth.</x:v>
+      </x:c>
+      <x:c r="M370" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N370" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question verified, reply verified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O370" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P370" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-21/dcfems-6001-1792629506.m4a</x:v>
+      </x:c>
+      <x:c r="Q370" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-21/dcfems-6001-1792629539.m4a</x:v>
+      </x:c>
+      <x:c r="R370" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-21</x:v>
+      </x:c>
+      <x:c r="S370" s="13" t="n">
+        <x:v>33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371">
+      <x:c r="A371" s="13" t="str">
+        <x:v>E364</x:v>
+      </x:c>
+      <x:c r="B371" s="13" t="str">
+        <x:v>Tanner / T-Ball / G-Ball</x:v>
+      </x:c>
+      <x:c r="C371" s="14" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="D371" s="13" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="E371" s="15" t="n">
+        <x:v>0.7788541666666666</x:v>
+      </x:c>
+      <x:c r="F371" s="16" t="str">
+        <x:v>14590073</x:v>
+      </x:c>
+      <x:c r="G371" s="13" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="H371" s="15" t="n">
+        <x:v>0.7797337962962962</x:v>
+      </x:c>
+      <x:c r="I371" s="17" t="n">
+        <x:f>ROUND((H371-E371)*86400,0)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="J371" s="16" t="str">
+        <x:v>14580151</x:v>
+      </x:c>
+      <x:c r="K371" s="13" t="str">
+        <x:v>Okay Tanner, just one more. Will you confirm Britain's info?</x:v>
+      </x:c>
+      <x:c r="L371" s="13" t="str">
+        <x:v>So last name is R-E-A-D. I heard him wrong.[unclear]. That's my bad.</x:v>
+      </x:c>
+      <x:c r="M371" s="13" t="str">
+        <x:v>Named response association</x:v>
+      </x:c>
+      <x:c r="N371" s="13" t="str">
+        <x:v>Owner identifies Tanner, T-Ball and G-Ball as Tanner Ballamis. Archive verification: question verified, reply verified. No independent audio review for this workbook update.</x:v>
+      </x:c>
+      <x:c r="O371" s="18" t="str">
+        <x:v>Owner identification</x:v>
+      </x:c>
+      <x:c r="P371" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-21/dcfems-6001-1792629693.m4a</x:v>
+      </x:c>
+      <x:c r="Q371" s="19" t="str">
+        <x:v>https://media.afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-21/dcfems-6001-1792629769.m4a</x:v>
+      </x:c>
+      <x:c r="R371" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-21</x:v>
+      </x:c>
+      <x:c r="S371" s="13" t="n">
+        <x:v>76</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24537,7 +24904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raec8db8254b1423c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ebdc3f77aef4a7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25029,7 +25396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10702eef2e594d41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ffc89996584d8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25114,7 +25481,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>The selected examples are a research index, not an exhaustive list of every address/response. Radio ID 0 and -1 were treated as unavailable.</x:v>
+        <x:v>The selected examples are a research index, not an exhaustive list. October 27 owner identification groups Tanner, T-Ball and G-Ball as Tanner Ballamis. Seven earlier response pairs added; 10 pairs across four days use 14580151.</x:v>
       </x:c>
       <x:c r="B8" s="2"/>
       <x:c r="C8" s="2"/>
@@ -25994,7 +26361,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5ccc77407ec4e82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34f368bfdbdc4ec8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve Halladay and Canizalez Sam rows in radio ID workbook
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="Rc6833c13207a40dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Rf8a8b0e1e2e94f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="Rfcfb374cfac0470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R2f445cbd4b31404b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R1cf70ccea3df4089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Ra5512b5c2a4b4a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R146d1bdcc58e49ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R699e66c221434463"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1579,113 +1579,115 @@
     </x:row>
     <x:row r="36" ht="60" customHeight="1">
       <x:c r="A36" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B36" s="11" t="str">
-        <x:v>14590037</x:v>
+        <x:v>14590067</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A36,Exchanges!$J$8:$J$371,B36)</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F36" s="12" t="n">
-        <x:v>46299</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H36" s="10"/>
       <x:c r="I36" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Sammantha J. Halladay</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies the female reply in October 7 clip 55 as Halladay; October 8 uses the same ID.</x:v>
       </x:c>
       <x:c r="K36" s="10" t="str">
-        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
+        <x:v>2026-10-07, 2026-10-08</x:v>
       </x:c>
       <x:c r="L36" s="10" t="str">
-        <x:v>E095, E137, E207, E231</x:v>
+        <x:v>E248, E250</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B37" s="11" t="str">
-        <x:v>14590095</x:v>
+        <x:v>14590100</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A37,Exchanges!$J$8:$J$371,B37)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E37" s="12" t="n">
-        <x:v>46283</x:v>
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="F37" s="12" t="n">
         <x:v>46289</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
-        <x:v>Repeated across days</x:v>
-      </x:c>
-      <x:c r="H37" s="10"/>
+        <x:v>Owner identified</x:v>
+      </x:c>
+      <x:c r="H37" s="10" t="str">
+        <x:v>Heaton / Colby</x:v>
+      </x:c>
       <x:c r="I37" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Sammantha J. Halladay</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies the September 24 female replies as Halladay. September 19 and Colby references remain unverified.</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
+        <x:v>2026-09-19, 2026-09-24</x:v>
       </x:c>
       <x:c r="L37" s="10" t="str">
-        <x:v>E128, E131, E132, E167</x:v>
+        <x:v>E130, E163, E164</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="60" customHeight="1">
       <x:c r="A38" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B38" s="11" t="str">
-        <x:v>14590099</x:v>
+        <x:v>14590090</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A38,Exchanges!$J$8:$J$371,B38)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D38" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E38" s="12" t="n">
-        <x:v>46299</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="F38" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H38" s="10"/>
       <x:c r="I38" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies the September 28 Sam replies as Samuel Canizalez.</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>2026-10-04, 2026-10-15</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="L38" s="10" t="str">
-        <x:v>E232, E233, E312</x:v>
+        <x:v>E203, E204</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="60" customHeight="1">
@@ -1693,20 +1695,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B39" s="11" t="str">
-        <x:v>14590207</x:v>
+        <x:v>14590037</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A39,Exchanges!$J$8:$J$371,B39)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
-        <x:v>46291</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="F39" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1719,195 +1721,199 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>2026-09-26, 2026-10-09</x:v>
+        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
       </x:c>
       <x:c r="L39" s="10" t="str">
-        <x:v>E193, E265</x:v>
+        <x:v>E095, E137, E207, E231</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="60" customHeight="1">
       <x:c r="A40" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B40" s="11" t="str">
-        <x:v>14590067</x:v>
+        <x:v>14590095</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A40,Exchanges!$J$8:$J$371,B40)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46283</x:v>
       </x:c>
       <x:c r="F40" s="12" t="n">
-        <x:v>46303</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H40" s="10"/>
       <x:c r="I40" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>2026-10-07, 2026-10-08</x:v>
+        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
       </x:c>
       <x:c r="L40" s="10" t="str">
-        <x:v>E248, E250</x:v>
+        <x:v>E128, E131, E132, E167</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="60" customHeight="1">
       <x:c r="A41" s="10" t="str">
-        <x:v>Somerville</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B41" s="11" t="str">
-        <x:v>14590042</x:v>
+        <x:v>14590099</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A41,Exchanges!$J$8:$J$371,B41)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
-        <x:v>46274</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="F41" s="12" t="n">
-        <x:v>46297</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H41" s="10"/>
       <x:c r="I41" s="10" t="str">
-        <x:v>J. Tayler Somerville</x:v>
-      </x:c>
-      <x:c r="J41" s="10"/>
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="J41" s="10" t="str">
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+      </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
+        <x:v>2026-10-04, 2026-10-15</x:v>
       </x:c>
       <x:c r="L41" s="10" t="str">
-        <x:v>E001, E096, E170, E222</x:v>
+        <x:v>E232, E233, E312</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="60" customHeight="1">
       <x:c r="A42" s="10" t="str">
-        <x:v>Somerville</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B42" s="11" t="str">
-        <x:v>14590073</x:v>
+        <x:v>14590207</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A42,Exchanges!$J$8:$J$371,B42)</x:f>
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
-        <x:v>9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
-        <x:v>46281</x:v>
+        <x:v>46291</x:v>
       </x:c>
       <x:c r="F42" s="12" t="n">
-        <x:v>46317</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H42" s="10"/>
       <x:c r="I42" s="10" t="str">
-        <x:v>J. Tayler Somerville</x:v>
-      </x:c>
-      <x:c r="J42" s="10"/>
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="J42" s="10" t="str">
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+      </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
+        <x:v>2026-09-26, 2026-10-09</x:v>
       </x:c>
       <x:c r="L42" s="10" t="str">
-        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
+        <x:v>E193, E265</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="60" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>Tonga</x:v>
+        <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B43" s="11" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590042</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A43,Exchanges!$J$8:$J$371,B43)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E43" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="F43" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H43" s="10"/>
       <x:c r="I43" s="10" t="str">
-        <x:v>Spencer Tonga</x:v>
+        <x:v>J. Tayler Somerville</x:v>
       </x:c>
       <x:c r="J43" s="10"/>
       <x:c r="K43" s="10" t="str">
-        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
+        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
       </x:c>
       <x:c r="L43" s="10" t="str">
-        <x:v>E071, E085, E183, E278, E333</x:v>
+        <x:v>E001, E096, E170, E222</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="60" customHeight="1">
       <x:c r="A44" s="10" t="str">
-        <x:v>Tonga</x:v>
+        <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B44" s="11" t="str">
-        <x:v>14590345</x:v>
+        <x:v>14590073</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A44,Exchanges!$J$8:$J$371,B44)</x:f>
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46281</x:v>
       </x:c>
       <x:c r="F44" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46317</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H44" s="10"/>
       <x:c r="I44" s="10" t="str">
-        <x:v>Spencer Tonga</x:v>
+        <x:v>J. Tayler Somerville</x:v>
       </x:c>
       <x:c r="J44" s="10"/>
       <x:c r="K44" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
+        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
       </x:c>
       <x:c r="L44" s="10" t="str">
-        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
+        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="60" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>14590079</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A45,Exchanges!$J$8:$J$371,B45)</x:f>
@@ -1917,106 +1923,102 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
-        <x:v>46275</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F45" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H45" s="10"/>
       <x:c r="I45" s="10" t="str">
-        <x:v>Jonathan Wagley</x:v>
+        <x:v>Spencer Tonga</x:v>
       </x:c>
       <x:c r="J45" s="10"/>
       <x:c r="K45" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
+        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
       </x:c>
       <x:c r="L45" s="10" t="str">
-        <x:v>E008, E160, E201, E252, E338</x:v>
+        <x:v>E071, E085, E183, E278, E333</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="60" customHeight="1">
       <x:c r="A46" s="10" t="str">
-        <x:v>Greg</x:v>
+        <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>14590026</x:v>
+        <x:v>14590345</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A46,Exchanges!$J$8:$J$371,B46)</x:f>
-        <x:v>1</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
         <x:v>46276</x:v>
       </x:c>
       <x:c r="F46" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H46" s="10"/>
       <x:c r="I46" s="10" t="str">
-        <x:v>Greg B. Mecham</x:v>
-      </x:c>
-      <x:c r="J46" s="10" t="str">
-        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
-      </x:c>
+        <x:v>Spencer Tonga</x:v>
+      </x:c>
+      <x:c r="J46" s="10"/>
       <x:c r="K46" s="10" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
       </x:c>
       <x:c r="L46" s="10" t="str">
-        <x:v>E034</x:v>
+        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="60" customHeight="1">
       <x:c r="A47" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>14590031</x:v>
+        <x:v>14590079</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A47,Exchanges!$J$8:$J$371,B47)</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="F47" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H47" s="10"/>
       <x:c r="I47" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
-      </x:c>
-      <x:c r="J47" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
-      </x:c>
+        <x:v>Jonathan Wagley</x:v>
+      </x:c>
+      <x:c r="J47" s="10"/>
       <x:c r="K47" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
       </x:c>
       <x:c r="L47" s="10" t="str">
-        <x:v>E260</x:v>
+        <x:v>E008, E160, E201, E252, E338</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="60" customHeight="1">
       <x:c r="A48" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Greg</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
-        <x:v>14590101</x:v>
+        <x:v>14590026</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A48,Exchanges!$J$8:$J$371,B48)</x:f>
@@ -2026,34 +2028,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F48" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="G48" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H48" s="10"/>
       <x:c r="I48" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
+        <x:v>Greg B. Mecham</x:v>
       </x:c>
       <x:c r="J48" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
+        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
       </x:c>
       <x:c r="K48" s="10" t="str">
-        <x:v>2026-09-12</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L48" s="10" t="str">
-        <x:v>E046</x:v>
+        <x:v>E034</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="60" customHeight="1">
       <x:c r="A49" s="10" t="str">
-        <x:v>Jackie</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B49" s="11" t="str">
-        <x:v>14590103</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A49,Exchanges!$J$8:$J$371,B49)</x:f>
@@ -2063,34 +2065,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E49" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F49" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G49" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H49" s="10"/>
       <x:c r="I49" s="10" t="str">
-        <x:v>Jaclyn G. Strong (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J49" s="10" t="str">
-        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K49" s="10" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L49" s="10" t="str">
-        <x:v>E297</x:v>
+        <x:v>E260</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="60" customHeight="1">
       <x:c r="A50" s="10" t="str">
-        <x:v>Kitchen</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B50" s="11" t="str">
-        <x:v>14590043</x:v>
+        <x:v>14590101</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A50,Exchanges!$J$8:$J$371,B50)</x:f>
@@ -2100,34 +2102,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F50" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="G50" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H50" s="10"/>
       <x:c r="I50" s="10" t="str">
-        <x:v>Bronson T. Kitchen (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J50" s="10" t="str">
-        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K50" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-09-12</x:v>
       </x:c>
       <x:c r="L50" s="10" t="str">
-        <x:v>E259</x:v>
+        <x:v>E046</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
       <x:c r="A51" s="10" t="str">
-        <x:v>Laycock</x:v>
+        <x:v>Jackie</x:v>
       </x:c>
       <x:c r="B51" s="11" t="str">
-        <x:v>14590025</x:v>
+        <x:v>14590103</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A51,Exchanges!$J$8:$J$371,B51)</x:f>
@@ -2137,143 +2139,145 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E51" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="F51" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="G51" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H51" s="10" t="str">
-        <x:v>Jake</x:v>
-      </x:c>
+        <x:v>Single-day candidate</x:v>
+      </x:c>
+      <x:c r="H51" s="10"/>
       <x:c r="I51" s="10" t="str">
-        <x:v>Jake D. Laycock</x:v>
+        <x:v>Jaclyn G. Strong (candidate)</x:v>
       </x:c>
       <x:c r="J51" s="10" t="str">
-        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
       </x:c>
       <x:c r="K51" s="10" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="L51" s="10" t="str">
-        <x:v>E143</x:v>
+        <x:v>E297</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
       <x:c r="A52" s="10" t="str">
-        <x:v>Murray</x:v>
+        <x:v>Kitchen</x:v>
       </x:c>
       <x:c r="B52" s="11" t="str">
-        <x:v>14590266</x:v>
+        <x:v>14590043</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A52,Exchanges!$J$8:$J$371,B52)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D52" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F52" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G52" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H52" s="10"/>
       <x:c r="I52" s="10" t="str">
-        <x:v>Austin W. Murray</x:v>
-      </x:c>
-      <x:c r="J52" s="10"/>
+        <x:v>Bronson T. Kitchen (candidate)</x:v>
+      </x:c>
+      <x:c r="J52" s="10" t="str">
+        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
+      </x:c>
       <x:c r="K52" s="10" t="str">
-        <x:v>2026-10-03</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L52" s="10" t="str">
-        <x:v>E228, E229</x:v>
+        <x:v>E259</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
       <x:c r="A53" s="10" t="str">
-        <x:v>Renter</x:v>
+        <x:v>Laycock</x:v>
       </x:c>
       <x:c r="B53" s="11" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590025</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A53,Exchanges!$J$8:$J$371,B53)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D53" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E53" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="F53" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="G53" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
-      </x:c>
-      <x:c r="H53" s="10"/>
+        <x:v>Conflicting names on ID</x:v>
+      </x:c>
+      <x:c r="H53" s="10" t="str">
+        <x:v>Jake</x:v>
+      </x:c>
       <x:c r="I53" s="10" t="str">
-        <x:v>Dustin R. Renter</x:v>
-      </x:c>
-      <x:c r="J53" s="10"/>
+        <x:v>Jake D. Laycock</x:v>
+      </x:c>
+      <x:c r="J53" s="10" t="str">
+        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+      </x:c>
       <x:c r="K53" s="10" t="str">
-        <x:v>2026-10-11</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="L53" s="10" t="str">
-        <x:v>E284, E285</x:v>
+        <x:v>E143</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
       <x:c r="A54" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Murray</x:v>
       </x:c>
       <x:c r="B54" s="11" t="str">
-        <x:v>14590066</x:v>
+        <x:v>14590266</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A54,Exchanges!$J$8:$J$371,B54)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E54" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="F54" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="G54" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H54" s="10"/>
       <x:c r="I54" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
-      </x:c>
-      <x:c r="J54" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
-      </x:c>
+        <x:v>Austin W. Murray</x:v>
+      </x:c>
+      <x:c r="J54" s="10"/>
       <x:c r="K54" s="10" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="L54" s="10" t="str">
-        <x:v>E205</x:v>
+        <x:v>E228, E229</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
       <x:c r="A55" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Renter</x:v>
       </x:c>
       <x:c r="B55" s="11" t="str">
-        <x:v>14590090</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A55,Exchanges!$J$8:$J$371,B55)</x:f>
@@ -2283,26 +2287,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="F55" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G55" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H55" s="10"/>
       <x:c r="I55" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
-      </x:c>
-      <x:c r="J55" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
-      </x:c>
+        <x:v>Dustin R. Renter</x:v>
+      </x:c>
+      <x:c r="J55" s="10"/>
       <x:c r="K55" s="10" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-10-11</x:v>
       </x:c>
       <x:c r="L55" s="10" t="str">
-        <x:v>E203, E204</x:v>
+        <x:v>E284, E285</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
@@ -2310,7 +2312,7 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="B56" s="11" t="str">
-        <x:v>14590268</x:v>
+        <x:v>14590066</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A56,Exchanges!$J$8:$J$371,B56)</x:f>
@@ -2320,10 +2322,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="F56" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="G56" s="10" t="str">
         <x:v>Single-day candidate</x:v>
@@ -2336,18 +2338,18 @@
         <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
       </x:c>
       <x:c r="K56" s="10" t="str">
-        <x:v>2026-10-07</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="L56" s="10" t="str">
-        <x:v>E247</x:v>
+        <x:v>E205</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
       <x:c r="A57" s="10" t="str">
-        <x:v>Tyler</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B57" s="11" t="str">
-        <x:v>14590085</x:v>
+        <x:v>14590268</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A57,Exchanges!$J$8:$J$371,B57)</x:f>
@@ -2367,24 +2369,24 @@
       </x:c>
       <x:c r="H57" s="10"/>
       <x:c r="I57" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Multiple candidates</x:v>
       </x:c>
       <x:c r="J57" s="10" t="str">
-        <x:v>Spoken name Tyler; no full-name identity assigned. Do not equate this with Tayler Somerville.</x:v>
+        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
       </x:c>
       <x:c r="K57" s="10" t="str">
         <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="L57" s="10" t="str">
-        <x:v>E249</x:v>
+        <x:v>E247</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
       <x:c r="A58" s="10" t="str">
-        <x:v>Valadez</x:v>
+        <x:v>Tyler</x:v>
       </x:c>
       <x:c r="B58" s="11" t="str">
-        <x:v>14590126</x:v>
+        <x:v>14590085</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A58,Exchanges!$J$8:$J$371,B58)</x:f>
@@ -2394,36 +2396,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E58" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F58" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="G58" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H58" s="10" t="str">
-        <x:v>Phil</x:v>
-      </x:c>
+        <x:v>Single-day candidate</x:v>
+      </x:c>
+      <x:c r="H58" s="10"/>
       <x:c r="I58" s="10" t="str">
-        <x:v>Mckay or Philip Valadez</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="J58" s="10" t="str">
-        <x:v>Surname is uncertain in transcript. Do not use this one exchange to prove which Valadez is speaking.</x:v>
+        <x:v>Spoken name Tyler; no full-name identity assigned. Do not equate this with Tayler Somerville.</x:v>
       </x:c>
       <x:c r="K58" s="10" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="L58" s="10" t="str">
-        <x:v>E093</x:v>
+        <x:v>E249</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
       <x:c r="A59" s="10" t="str">
-        <x:v>Colton</x:v>
+        <x:v>Valadez</x:v>
       </x:c>
       <x:c r="B59" s="11" t="str">
-        <x:v>14590091</x:v>
+        <x:v>14590126</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A59,Exchanges!$J$8:$J$371,B59)</x:f>
@@ -2433,67 +2433,67 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E59" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="F59" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="G59" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H59" s="10" t="str">
-        <x:v>Ethan, Heaton / Colby</x:v>
+        <x:v>Phil</x:v>
       </x:c>
       <x:c r="I59" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Mckay or Philip Valadez</x:v>
       </x:c>
       <x:c r="J59" s="10" t="str">
-        <x:v>14590091 also answers Heaton/Colby and Ethan. Could be transcript error, shared radio, or a different responder.</x:v>
+        <x:v>Surname is uncertain in transcript. Do not use this one exchange to prove which Valadez is speaking.</x:v>
       </x:c>
       <x:c r="K59" s="10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="L59" s="10" t="str">
-        <x:v>E243</x:v>
+        <x:v>E093</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="60" customHeight="1">
       <x:c r="A60" s="10" t="str">
-        <x:v>Ethan</x:v>
+        <x:v>Colton</x:v>
       </x:c>
       <x:c r="B60" s="11" t="str">
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A60,Exchanges!$J$8:$J$371,B60)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D60" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E60" s="12" t="n">
-        <x:v>46292</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="F60" s="12" t="n">
-        <x:v>46292</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="G60" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H60" s="10" t="str">
-        <x:v>Colton, Heaton / Colby</x:v>
+        <x:v>Ethan, Heaton / Colby</x:v>
       </x:c>
       <x:c r="I60" s="10" t="str">
-        <x:v>Ethan C. Simmons</x:v>
+        <x:v>Multiple candidates</x:v>
       </x:c>
       <x:c r="J60" s="10" t="str">
-        <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
+        <x:v>14590091 also answers Heaton/Colby and Ethan. Could be transcript error, shared radio, or a different responder.</x:v>
       </x:c>
       <x:c r="K60" s="10" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
       <x:c r="L60" s="10" t="str">
-        <x:v>E197, E198</x:v>
+        <x:v>E243</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="60" customHeight="1">
@@ -2501,26 +2501,26 @@
         <x:v>Ethan</x:v>
       </x:c>
       <x:c r="B61" s="11" t="str">
-        <x:v>14590225</x:v>
+        <x:v>14590091</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A61,Exchanges!$J$8:$J$371,B61)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E61" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46292</x:v>
       </x:c>
       <x:c r="F61" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46292</x:v>
       </x:c>
       <x:c r="G61" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H61" s="10" t="str">
-        <x:v>Jensen / Josh</x:v>
+        <x:v>Colton, Heaton / Colby</x:v>
       </x:c>
       <x:c r="I61" s="10" t="str">
         <x:v>Ethan C. Simmons</x:v>
@@ -2529,28 +2529,28 @@
         <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
       </x:c>
       <x:c r="K61" s="10" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
       <x:c r="L61" s="10" t="str">
-        <x:v>E311</x:v>
+        <x:v>E197, E198</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="60" customHeight="1">
       <x:c r="A62" s="10" t="str">
-        <x:v>Hawkins</x:v>
+        <x:v>Ethan</x:v>
       </x:c>
       <x:c r="B62" s="11" t="str">
-        <x:v>14590036</x:v>
+        <x:v>14590225</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A62,Exchanges!$J$8:$J$371,B62)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="F62" s="12" t="n">
         <x:v>46310</x:v>
@@ -2559,58 +2559,58 @@
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H62" s="10" t="str">
-        <x:v>Mitch</x:v>
+        <x:v>Jensen / Josh</x:v>
       </x:c>
       <x:c r="I62" s="10" t="str">
-        <x:v>Steven G. Hawkins</x:v>
+        <x:v>Ethan C. Simmons</x:v>
       </x:c>
       <x:c r="J62" s="10" t="str">
-        <x:v>14590036 also answers hails to Mitch. Keep this as an exchange-level association.</x:v>
+        <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
       </x:c>
       <x:c r="K62" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-10-15</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="L62" s="10" t="str">
-        <x:v>E026, E068, E070, E317</x:v>
+        <x:v>E311</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="60" customHeight="1">
       <x:c r="A63" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Hawkins</x:v>
       </x:c>
       <x:c r="B63" s="11" t="str">
-        <x:v>14590091</x:v>
+        <x:v>14590036</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A63,Exchanges!$J$8:$J$371,B63)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E63" s="12" t="n">
-        <x:v>46290</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F63" s="12" t="n">
-        <x:v>46290</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G63" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H63" s="10" t="str">
-        <x:v>Colton, Ethan</x:v>
+        <x:v>Mitch</x:v>
       </x:c>
       <x:c r="I63" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
+        <x:v>Steven G. Hawkins</x:v>
       </x:c>
       <x:c r="J63" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
+        <x:v>14590036 also answers hails to Mitch. Keep this as an exchange-level association.</x:v>
       </x:c>
       <x:c r="K63" s="10" t="str">
-        <x:v>2026-09-25</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-10-15</x:v>
       </x:c>
       <x:c r="L63" s="10" t="str">
-        <x:v>E173, E175</x:v>
+        <x:v>E026, E068, E070, E317</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="60" customHeight="1">
@@ -2618,26 +2618,26 @@
         <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B64" s="11" t="str">
-        <x:v>14590100</x:v>
+        <x:v>14590091</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A64,Exchanges!$J$8:$J$371,B64)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E64" s="12" t="n">
-        <x:v>46309</x:v>
+        <x:v>46290</x:v>
       </x:c>
       <x:c r="F64" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46290</x:v>
       </x:c>
       <x:c r="G64" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H64" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Colton, Ethan</x:v>
       </x:c>
       <x:c r="I64" s="10" t="str">
         <x:v>Colby A. Heaton</x:v>
@@ -2646,57 +2646,57 @@
         <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K64" s="10" t="str">
-        <x:v>2026-10-14, 2026-10-20</x:v>
+        <x:v>2026-09-25</x:v>
       </x:c>
       <x:c r="L64" s="10" t="str">
-        <x:v>E301, E329, E331</x:v>
+        <x:v>E173, E175</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="60" customHeight="1">
       <x:c r="A65" s="10" t="str">
-        <x:v>Jensen / Josh</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B65" s="11" t="str">
-        <x:v>14590225</x:v>
+        <x:v>14590100</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A65,Exchanges!$J$8:$J$371,B65)</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E65" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="F65" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G65" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H65" s="10" t="str">
-        <x:v>Ethan</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="I65" s="10" t="str">
-        <x:v>Joshua M. Jensen (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J65" s="10" t="str">
-        <x:v>Both Jensen and Josh are represented; Joshua Jensen is a candidate. First-name replies alone do not rule out other Joshuas.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K65" s="10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-14, 2026-10-20</x:v>
       </x:c>
       <x:c r="L65" s="10" t="str">
-        <x:v>E237</x:v>
+        <x:v>E301, E329, E331</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="60" customHeight="1">
       <x:c r="A66" s="10" t="str">
-        <x:v>Luke</x:v>
+        <x:v>Jensen / Josh</x:v>
       </x:c>
       <x:c r="B66" s="11" t="str">
-        <x:v>14590221</x:v>
+        <x:v>14590225</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A66,Exchanges!$J$8:$J$371,B66)</x:f>
@@ -2706,112 +2706,112 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E66" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="F66" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="G66" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H66" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Ethan</x:v>
       </x:c>
       <x:c r="I66" s="10" t="str">
-        <x:v>Luke A. Sumbot</x:v>
+        <x:v>Joshua M. Jensen (candidate)</x:v>
       </x:c>
       <x:c r="J66" s="10" t="str">
-        <x:v>14590221 also answers hails to Sam. This short reply does not establish that the transmitter is Luke.</x:v>
+        <x:v>Both Jensen and Josh are represented; Joshua Jensen is a candidate. First-name replies alone do not rule out other Joshuas.</x:v>
       </x:c>
       <x:c r="K66" s="10" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
       <x:c r="L66" s="10" t="str">
-        <x:v>E334</x:v>
+        <x:v>E237</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="60" customHeight="1">
       <x:c r="A67" s="10" t="str">
-        <x:v>McClellan / Dennis</x:v>
+        <x:v>Luke</x:v>
       </x:c>
       <x:c r="B67" s="11" t="str">
-        <x:v>14590019</x:v>
+        <x:v>14590221</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A67,Exchanges!$J$8:$J$371,B67)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D67" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E67" s="12" t="n">
-        <x:v>46294</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="F67" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G67" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H67" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="I67" s="10" t="str">
-        <x:v>Dennis R. McClellan</x:v>
-      </x:c>
-      <x:c r="J67" s="10"/>
+        <x:v>Luke A. Sumbot</x:v>
+      </x:c>
+      <x:c r="J67" s="10" t="str">
+        <x:v>14590221 also answers hails to Sam. This short reply does not establish that the transmitter is Luke.</x:v>
+      </x:c>
       <x:c r="K67" s="10" t="str">
-        <x:v>2026-09-29, 2026-10-02, 2026-10-03</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="L67" s="10" t="str">
-        <x:v>E208, E221, E226</x:v>
+        <x:v>E334</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="60" customHeight="1">
       <x:c r="A68" s="10" t="str">
-        <x:v>Mitch</x:v>
+        <x:v>McClellan / Dennis</x:v>
       </x:c>
       <x:c r="B68" s="11" t="str">
-        <x:v>14590036</x:v>
+        <x:v>14590019</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A68,Exchanges!$J$8:$J$371,B68)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E68" s="12" t="n">
-        <x:v>46281</x:v>
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="F68" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="G68" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H68" s="10" t="str">
-        <x:v>Hawkins</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="I68" s="10" t="str">
-        <x:v>Mitchell R. Godfrey (candidate)</x:v>
-      </x:c>
-      <x:c r="J68" s="10" t="str">
-        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
-      </x:c>
+        <x:v>Dennis R. McClellan</x:v>
+      </x:c>
+      <x:c r="J68" s="10"/>
       <x:c r="K68" s="10" t="str">
-        <x:v>2026-09-16, 2026-10-15</x:v>
+        <x:v>2026-09-29, 2026-10-02, 2026-10-03</x:v>
       </x:c>
       <x:c r="L68" s="10" t="str">
-        <x:v>E110, E313, E316</x:v>
+        <x:v>E208, E221, E226</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="60" customHeight="1">
       <x:c r="A69" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Mitch</x:v>
       </x:c>
       <x:c r="B69" s="11" t="str">
-        <x:v>14590100</x:v>
+        <x:v>14590036</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A69,Exchanges!$J$8:$J$371,B69)</x:f>
@@ -2821,28 +2821,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E69" s="12" t="n">
-        <x:v>46284</x:v>
+        <x:v>46281</x:v>
       </x:c>
       <x:c r="F69" s="12" t="n">
-        <x:v>46289</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G69" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H69" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Hawkins</x:v>
       </x:c>
       <x:c r="I69" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Mitchell R. Godfrey (candidate)</x:v>
       </x:c>
       <x:c r="J69" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
       </x:c>
       <x:c r="K69" s="10" t="str">
-        <x:v>2026-09-19, 2026-09-24</x:v>
+        <x:v>2026-09-16, 2026-10-15</x:v>
       </x:c>
       <x:c r="L69" s="10" t="str">
-        <x:v>E130, E163, E164</x:v>
+        <x:v>E110, E313, E316</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="60" customHeight="1">
@@ -3170,7 +3170,7 @@
       <x:c r="G78" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
-      <x:c r="H78" s="10" t="str"/>
+      <x:c r="H78" s="10"/>
       <x:c r="I78" s="10" t="str">
         <x:v>Tanner M. Ballamis</x:v>
       </x:c>
@@ -3297,7 +3297,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8054ef3d10874730"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88f7f2b67553444b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11120,7 +11120,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N137" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>14590100 is associated with Halladay from the owner’s September 24 voice identification. This September 19 exchange remains unverified.</x:v>
       </x:c>
       <x:c r="O137" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -13056,7 +13056,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N170" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies the female reply as Sammantha J. Halladay. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O170" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -13116,7 +13116,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N171" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies the female reply as Sammantha J. Halladay. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O171" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -15398,7 +15398,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N210" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies Sam on 14590090 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O210" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -15458,7 +15458,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N211" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies Sam on 14590090 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O211" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -18040,7 +18040,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N255" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies the female reply in October 7 clip 55 as Sammantha J. Halladay. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O255" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -18160,7 +18160,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N257" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner associates 14590067 with Sammantha J. Halladay based on October 7 clip 55. This October 8 exchange uses the same ID.</x:v>
       </x:c>
       <x:c r="O257" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -24904,7 +24904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ebdc3f77aef4a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7ee122fa06740ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25396,7 +25396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ffc89996584d8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra808396c921e448e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26361,7 +26361,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34f368bfdbdc4ec8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f5af40f78df46b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Identify additional Sam radio IDs as Samuel Canizalez
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R1cf70ccea3df4089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Ra5512b5c2a4b4a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R146d1bdcc58e49ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R699e66c221434463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R217ebf8a63b24cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R8b65fba8d3cf4078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R828573d171504049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="Rfada22cec3194a3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1692,76 +1692,76 @@
     </x:row>
     <x:row r="39" ht="60" customHeight="1">
       <x:c r="A39" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B39" s="11" t="str">
-        <x:v>14590037</x:v>
+        <x:v>14590066</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A39,Exchanges!$J$8:$J$371,B39)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="F39" s="12" t="n">
-        <x:v>46299</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="G39" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H39" s="10"/>
       <x:c r="I39" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies Sam on 14590066 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
-        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="L39" s="10" t="str">
-        <x:v>E095, E137, E207, E231</x:v>
+        <x:v>E205</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="60" customHeight="1">
       <x:c r="A40" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B40" s="11" t="str">
-        <x:v>14590095</x:v>
+        <x:v>14590268</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A40,Exchanges!$J$8:$J$371,B40)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
-        <x:v>46283</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F40" s="12" t="n">
-        <x:v>46289</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H40" s="10"/>
       <x:c r="I40" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies Sam on 14590268 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
+        <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="L40" s="10" t="str">
-        <x:v>E128, E131, E132, E167</x:v>
+        <x:v>E247</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="60" customHeight="1">
@@ -1769,20 +1769,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B41" s="11" t="str">
-        <x:v>14590099</x:v>
+        <x:v>14590037</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A41,Exchanges!$J$8:$J$371,B41)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="n">
         <x:v>46299</x:v>
-      </x:c>
-      <x:c r="F41" s="12" t="n">
-        <x:v>46310</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1795,10 +1795,10 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>2026-10-04, 2026-10-15</x:v>
+        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
       </x:c>
       <x:c r="L41" s="10" t="str">
-        <x:v>E232, E233, E312</x:v>
+        <x:v>E095, E137, E207, E231</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="60" customHeight="1">
@@ -1806,20 +1806,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B42" s="11" t="str">
-        <x:v>14590207</x:v>
+        <x:v>14590095</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A42,Exchanges!$J$8:$J$371,B42)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
-        <x:v>46291</x:v>
+        <x:v>46283</x:v>
       </x:c>
       <x:c r="F42" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1832,158 +1832,162 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>2026-09-26, 2026-10-09</x:v>
+        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
       </x:c>
       <x:c r="L42" s="10" t="str">
-        <x:v>E193, E265</x:v>
+        <x:v>E128, E131, E132, E167</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="60" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>Somerville</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B43" s="11" t="str">
-        <x:v>14590042</x:v>
+        <x:v>14590099</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A43,Exchanges!$J$8:$J$371,B43)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E43" s="12" t="n">
-        <x:v>46274</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="F43" s="12" t="n">
-        <x:v>46297</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H43" s="10"/>
       <x:c r="I43" s="10" t="str">
-        <x:v>J. Tayler Somerville</x:v>
-      </x:c>
-      <x:c r="J43" s="10"/>
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="J43" s="10" t="str">
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+      </x:c>
       <x:c r="K43" s="10" t="str">
-        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
+        <x:v>2026-10-04, 2026-10-15</x:v>
       </x:c>
       <x:c r="L43" s="10" t="str">
-        <x:v>E001, E096, E170, E222</x:v>
+        <x:v>E232, E233, E312</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="60" customHeight="1">
       <x:c r="A44" s="10" t="str">
-        <x:v>Somerville</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B44" s="11" t="str">
-        <x:v>14590073</x:v>
+        <x:v>14590207</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A44,Exchanges!$J$8:$J$371,B44)</x:f>
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
-        <x:v>9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
-        <x:v>46281</x:v>
+        <x:v>46291</x:v>
       </x:c>
       <x:c r="F44" s="12" t="n">
-        <x:v>46317</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H44" s="10"/>
       <x:c r="I44" s="10" t="str">
-        <x:v>J. Tayler Somerville</x:v>
-      </x:c>
-      <x:c r="J44" s="10"/>
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="J44" s="10" t="str">
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+      </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
+        <x:v>2026-09-26, 2026-10-09</x:v>
       </x:c>
       <x:c r="L44" s="10" t="str">
-        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
+        <x:v>E193, E265</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="60" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>Tonga</x:v>
+        <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590042</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A45,Exchanges!$J$8:$J$371,B45)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="F45" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H45" s="10"/>
       <x:c r="I45" s="10" t="str">
-        <x:v>Spencer Tonga</x:v>
+        <x:v>J. Tayler Somerville</x:v>
       </x:c>
       <x:c r="J45" s="10"/>
       <x:c r="K45" s="10" t="str">
-        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
+        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
       </x:c>
       <x:c r="L45" s="10" t="str">
-        <x:v>E071, E085, E183, E278, E333</x:v>
+        <x:v>E001, E096, E170, E222</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="60" customHeight="1">
       <x:c r="A46" s="10" t="str">
-        <x:v>Tonga</x:v>
+        <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>14590345</x:v>
+        <x:v>14590073</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A46,Exchanges!$J$8:$J$371,B46)</x:f>
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46281</x:v>
       </x:c>
       <x:c r="F46" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46317</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H46" s="10"/>
       <x:c r="I46" s="10" t="str">
-        <x:v>Spencer Tonga</x:v>
+        <x:v>J. Tayler Somerville</x:v>
       </x:c>
       <x:c r="J46" s="10"/>
       <x:c r="K46" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
+        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
       </x:c>
       <x:c r="L46" s="10" t="str">
-        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
+        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="60" customHeight="1">
       <x:c r="A47" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>14590079</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A47,Exchanges!$J$8:$J$371,B47)</x:f>
@@ -1993,106 +1997,102 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
-        <x:v>46275</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F47" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H47" s="10"/>
       <x:c r="I47" s="10" t="str">
-        <x:v>Jonathan Wagley</x:v>
+        <x:v>Spencer Tonga</x:v>
       </x:c>
       <x:c r="J47" s="10"/>
       <x:c r="K47" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
+        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
       </x:c>
       <x:c r="L47" s="10" t="str">
-        <x:v>E008, E160, E201, E252, E338</x:v>
+        <x:v>E071, E085, E183, E278, E333</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="60" customHeight="1">
       <x:c r="A48" s="10" t="str">
-        <x:v>Greg</x:v>
+        <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
-        <x:v>14590026</x:v>
+        <x:v>14590345</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A48,Exchanges!$J$8:$J$371,B48)</x:f>
-        <x:v>1</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
         <x:v>46276</x:v>
       </x:c>
       <x:c r="F48" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G48" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H48" s="10"/>
       <x:c r="I48" s="10" t="str">
-        <x:v>Greg B. Mecham</x:v>
-      </x:c>
-      <x:c r="J48" s="10" t="str">
-        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
-      </x:c>
+        <x:v>Spencer Tonga</x:v>
+      </x:c>
+      <x:c r="J48" s="10"/>
       <x:c r="K48" s="10" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
       </x:c>
       <x:c r="L48" s="10" t="str">
-        <x:v>E034</x:v>
+        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="60" customHeight="1">
       <x:c r="A49" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="B49" s="11" t="str">
-        <x:v>14590031</x:v>
+        <x:v>14590079</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A49,Exchanges!$J$8:$J$371,B49)</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E49" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="F49" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G49" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H49" s="10"/>
       <x:c r="I49" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
-      </x:c>
-      <x:c r="J49" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
-      </x:c>
+        <x:v>Jonathan Wagley</x:v>
+      </x:c>
+      <x:c r="J49" s="10"/>
       <x:c r="K49" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
       </x:c>
       <x:c r="L49" s="10" t="str">
-        <x:v>E260</x:v>
+        <x:v>E008, E160, E201, E252, E338</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="60" customHeight="1">
       <x:c r="A50" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Greg</x:v>
       </x:c>
       <x:c r="B50" s="11" t="str">
-        <x:v>14590101</x:v>
+        <x:v>14590026</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A50,Exchanges!$J$8:$J$371,B50)</x:f>
@@ -2102,34 +2102,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F50" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="G50" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H50" s="10"/>
       <x:c r="I50" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
+        <x:v>Greg B. Mecham</x:v>
       </x:c>
       <x:c r="J50" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
+        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
       </x:c>
       <x:c r="K50" s="10" t="str">
-        <x:v>2026-09-12</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L50" s="10" t="str">
-        <x:v>E046</x:v>
+        <x:v>E034</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
       <x:c r="A51" s="10" t="str">
-        <x:v>Jackie</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B51" s="11" t="str">
-        <x:v>14590103</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A51,Exchanges!$J$8:$J$371,B51)</x:f>
@@ -2139,34 +2139,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E51" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F51" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G51" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H51" s="10"/>
       <x:c r="I51" s="10" t="str">
-        <x:v>Jaclyn G. Strong (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J51" s="10" t="str">
-        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K51" s="10" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L51" s="10" t="str">
-        <x:v>E297</x:v>
+        <x:v>E260</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
       <x:c r="A52" s="10" t="str">
-        <x:v>Kitchen</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B52" s="11" t="str">
-        <x:v>14590043</x:v>
+        <x:v>14590101</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A52,Exchanges!$J$8:$J$371,B52)</x:f>
@@ -2176,34 +2176,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F52" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="G52" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H52" s="10"/>
       <x:c r="I52" s="10" t="str">
-        <x:v>Bronson T. Kitchen (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J52" s="10" t="str">
-        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K52" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-09-12</x:v>
       </x:c>
       <x:c r="L52" s="10" t="str">
-        <x:v>E259</x:v>
+        <x:v>E046</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
       <x:c r="A53" s="10" t="str">
-        <x:v>Laycock</x:v>
+        <x:v>Jackie</x:v>
       </x:c>
       <x:c r="B53" s="11" t="str">
-        <x:v>14590025</x:v>
+        <x:v>14590103</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A53,Exchanges!$J$8:$J$371,B53)</x:f>
@@ -2213,172 +2213,172 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E53" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="F53" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="G53" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H53" s="10" t="str">
-        <x:v>Jake</x:v>
-      </x:c>
+        <x:v>Single-day candidate</x:v>
+      </x:c>
+      <x:c r="H53" s="10"/>
       <x:c r="I53" s="10" t="str">
-        <x:v>Jake D. Laycock</x:v>
+        <x:v>Jaclyn G. Strong (candidate)</x:v>
       </x:c>
       <x:c r="J53" s="10" t="str">
-        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
       </x:c>
       <x:c r="K53" s="10" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="L53" s="10" t="str">
-        <x:v>E143</x:v>
+        <x:v>E297</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
       <x:c r="A54" s="10" t="str">
-        <x:v>Murray</x:v>
+        <x:v>Kitchen</x:v>
       </x:c>
       <x:c r="B54" s="11" t="str">
-        <x:v>14590266</x:v>
+        <x:v>14590043</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A54,Exchanges!$J$8:$J$371,B54)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E54" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F54" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G54" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H54" s="10"/>
       <x:c r="I54" s="10" t="str">
-        <x:v>Austin W. Murray</x:v>
-      </x:c>
-      <x:c r="J54" s="10"/>
+        <x:v>Bronson T. Kitchen (candidate)</x:v>
+      </x:c>
+      <x:c r="J54" s="10" t="str">
+        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
+      </x:c>
       <x:c r="K54" s="10" t="str">
-        <x:v>2026-10-03</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L54" s="10" t="str">
-        <x:v>E228, E229</x:v>
+        <x:v>E259</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
       <x:c r="A55" s="10" t="str">
-        <x:v>Renter</x:v>
+        <x:v>Laycock</x:v>
       </x:c>
       <x:c r="B55" s="11" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590025</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A55,Exchanges!$J$8:$J$371,B55)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="F55" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="G55" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
-      </x:c>
-      <x:c r="H55" s="10"/>
+        <x:v>Conflicting names on ID</x:v>
+      </x:c>
+      <x:c r="H55" s="10" t="str">
+        <x:v>Jake</x:v>
+      </x:c>
       <x:c r="I55" s="10" t="str">
-        <x:v>Dustin R. Renter</x:v>
-      </x:c>
-      <x:c r="J55" s="10"/>
+        <x:v>Jake D. Laycock</x:v>
+      </x:c>
+      <x:c r="J55" s="10" t="str">
+        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+      </x:c>
       <x:c r="K55" s="10" t="str">
-        <x:v>2026-10-11</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="L55" s="10" t="str">
-        <x:v>E284, E285</x:v>
+        <x:v>E143</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
       <x:c r="A56" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Murray</x:v>
       </x:c>
       <x:c r="B56" s="11" t="str">
-        <x:v>14590066</x:v>
+        <x:v>14590266</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A56,Exchanges!$J$8:$J$371,B56)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="F56" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="G56" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H56" s="10"/>
       <x:c r="I56" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
-      </x:c>
-      <x:c r="J56" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
-      </x:c>
+        <x:v>Austin W. Murray</x:v>
+      </x:c>
+      <x:c r="J56" s="10"/>
       <x:c r="K56" s="10" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="L56" s="10" t="str">
-        <x:v>E205</x:v>
+        <x:v>E228, E229</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
       <x:c r="A57" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Renter</x:v>
       </x:c>
       <x:c r="B57" s="11" t="str">
-        <x:v>14590268</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A57,Exchanges!$J$8:$J$371,B57)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D57" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="F57" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G57" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H57" s="10"/>
       <x:c r="I57" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
-      </x:c>
-      <x:c r="J57" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
-      </x:c>
+        <x:v>Dustin R. Renter</x:v>
+      </x:c>
+      <x:c r="J57" s="10"/>
       <x:c r="K57" s="10" t="str">
-        <x:v>2026-10-07</x:v>
+        <x:v>2026-10-11</x:v>
       </x:c>
       <x:c r="L57" s="10" t="str">
-        <x:v>E247</x:v>
+        <x:v>E284, E285</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
@@ -3297,7 +3297,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88f7f2b67553444b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f3a02ba1fc4e56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15518,7 +15518,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N212" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies Sam on 14590066 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O212" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -17980,7 +17980,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N254" s="13" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>Owner identifies Sam on 14590268 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="O254" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -24904,7 +24904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7ee122fa06740ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b03d9616aa14153"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25396,7 +25396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra808396c921e448e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R821ecce7ecbb4586"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26361,7 +26361,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f5af40f78df46b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1143a5ea2e9f488b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify September 12 Makai clips and resolve radio ID 14590105
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R217ebf8a63b24cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R8b65fba8d3cf4078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R828573d171504049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="Rfada22cec3194a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R036cb515380e4b2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Rd57dbd6f9a6e4054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R65c3d451b0be4487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R26c757c5a2924894"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1186,37 +1186,39 @@
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="10" t="str">
-        <x:v>Mason</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>14590237</x:v>
+        <x:v>14590105</x:v>
       </x:c>
       <x:c r="C25" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A25,Exchanges!$J$8:$J$371,B25)</x:f>
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E25" s="12" t="n">
-        <x:v>46278</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F25" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H25" s="10"/>
       <x:c r="I25" s="10" t="str">
-        <x:v>Brandon K. Mason</x:v>
-      </x:c>
-      <x:c r="J25" s="10"/>
+        <x:v>Kelepi Makai</x:v>
+      </x:c>
+      <x:c r="J25" s="10" t="str">
+        <x:v>Owner verified Makai in September 12 clips 446 and 851; replies on 14590105 support a single-day association.</x:v>
+      </x:c>
       <x:c r="K25" s="10" t="str">
-        <x:v>2026-09-13, 2026-09-17, 2026-09-21, 2026-09-25, 2026-09-26, 2026-10-05, 2026-10-10, 2026-10-11</x:v>
+        <x:v>2026-09-12</x:v>
       </x:c>
       <x:c r="L25" s="10" t="str">
-        <x:v>E077, E116, E138, E172, E176, E188, E192, E241, E269, E291</x:v>
+        <x:v>E050, E062</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
@@ -1224,20 +1226,20 @@
         <x:v>Mason</x:v>
       </x:c>
       <x:c r="B26" s="11" t="str">
-        <x:v>14590315</x:v>
+        <x:v>14590237</x:v>
       </x:c>
       <x:c r="C26" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A26,Exchanges!$J$8:$J$371,B26)</x:f>
-        <x:v>22</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E26" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46278</x:v>
       </x:c>
       <x:c r="F26" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G26" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1248,80 +1250,80 @@
       </x:c>
       <x:c r="J26" s="10"/>
       <x:c r="K26" s="10" t="str">
-        <x:v>2026-09-12, 2026-09-13, 2026-09-16, 2026-09-21, 2026-09-22, 2026-09-26, 2026-10-06, 2026-10-10, 2026-10-11, 2026-10-20</x:v>
+        <x:v>2026-09-13, 2026-09-17, 2026-09-21, 2026-09-25, 2026-09-26, 2026-10-05, 2026-10-10, 2026-10-11</x:v>
       </x:c>
       <x:c r="L26" s="10" t="str">
-        <x:v>E042, E043, E049, E056, E059, E073, E076, E100, E103, E104, E105, E106, E139, E147, E150, E187, E190, E244, E270, E271, E289, E330</x:v>
+        <x:v>E077, E116, E138, E172, E176, E188, E192, E241, E269, E291</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
       <x:c r="A27" s="10" t="str">
-        <x:v>McClellan / Dennis</x:v>
+        <x:v>Mason</x:v>
       </x:c>
       <x:c r="B27" s="11" t="str">
-        <x:v>14590162</x:v>
+        <x:v>14590315</x:v>
       </x:c>
       <x:c r="C27" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A27,Exchanges!$J$8:$J$371,B27)</x:f>
-        <x:v>3</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E27" s="12" t="n">
-        <x:v>46283</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F27" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H27" s="10"/>
       <x:c r="I27" s="10" t="str">
-        <x:v>Dennis R. McClellan</x:v>
+        <x:v>Brandon K. Mason</x:v>
       </x:c>
       <x:c r="J27" s="10"/>
       <x:c r="K27" s="10" t="str">
-        <x:v>2026-09-18, 2026-09-23, 2026-09-28</x:v>
+        <x:v>2026-09-12, 2026-09-13, 2026-09-16, 2026-09-21, 2026-09-22, 2026-09-26, 2026-10-06, 2026-10-10, 2026-10-11, 2026-10-20</x:v>
       </x:c>
       <x:c r="L27" s="10" t="str">
-        <x:v>E127, E161, E202</x:v>
+        <x:v>E042, E043, E049, E056, E059, E073, E076, E100, E103, E104, E105, E106, E139, E147, E150, E187, E190, E244, E270, E271, E289, E330</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
       <x:c r="A28" s="10" t="str">
-        <x:v>McKay</x:v>
+        <x:v>McClellan / Dennis</x:v>
       </x:c>
       <x:c r="B28" s="11" t="str">
-        <x:v>14590081</x:v>
+        <x:v>14590162</x:v>
       </x:c>
       <x:c r="C28" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A28,Exchanges!$J$8:$J$371,B28)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E28" s="12" t="n">
-        <x:v>46275</x:v>
+        <x:v>46283</x:v>
       </x:c>
       <x:c r="F28" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="G28" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H28" s="10"/>
       <x:c r="I28" s="10" t="str">
-        <x:v>Mckay A. Valadez</x:v>
+        <x:v>Dennis R. McClellan</x:v>
       </x:c>
       <x:c r="J28" s="10"/>
       <x:c r="K28" s="10" t="str">
-        <x:v>2026-09-10, 2026-10-21</x:v>
+        <x:v>2026-09-18, 2026-09-23, 2026-09-28</x:v>
       </x:c>
       <x:c r="L28" s="10" t="str">
-        <x:v>E009, E336</x:v>
+        <x:v>E127, E161, E202</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -1329,14 +1331,14 @@
         <x:v>McKay</x:v>
       </x:c>
       <x:c r="B29" s="11" t="str">
-        <x:v>14590102</x:v>
+        <x:v>14590081</x:v>
       </x:c>
       <x:c r="C29" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A29,Exchanges!$J$8:$J$371,B29)</x:f>
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E29" s="12" t="n">
         <x:v>46275</x:v>
@@ -1353,193 +1355,193 @@
       </x:c>
       <x:c r="J29" s="10"/>
       <x:c r="K29" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-14, 2026-09-18, 2026-09-28, 2026-10-17, 2026-10-21</x:v>
+        <x:v>2026-09-10, 2026-10-21</x:v>
       </x:c>
       <x:c r="L29" s="10" t="str">
-        <x:v>E010, E090, E091, E126, E200, E323, E325, E335</x:v>
+        <x:v>E009, E336</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
       <x:c r="A30" s="10" t="str">
-        <x:v>Mitch</x:v>
+        <x:v>McKay</x:v>
       </x:c>
       <x:c r="B30" s="11" t="str">
-        <x:v>14590344</x:v>
+        <x:v>14590102</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A30,Exchanges!$J$8:$J$371,B30)</x:f>
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="F30" s="12" t="n">
-        <x:v>46311</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H30" s="10"/>
       <x:c r="I30" s="10" t="str">
-        <x:v>Mitchell R. Godfrey (candidate)</x:v>
-      </x:c>
-      <x:c r="J30" s="10" t="str">
-        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
-      </x:c>
+        <x:v>Mckay A. Valadez</x:v>
+      </x:c>
+      <x:c r="J30" s="10"/>
       <x:c r="K30" s="10" t="str">
-        <x:v>2026-09-12, 2026-09-17, 2026-09-23, 2026-09-25, 2026-09-27, 2026-10-01, 2026-10-15, 2026-10-16</x:v>
+        <x:v>2026-09-10, 2026-09-14, 2026-09-18, 2026-09-28, 2026-10-17, 2026-10-21</x:v>
       </x:c>
       <x:c r="L30" s="10" t="str">
-        <x:v>E039, E122, E124, E154, E178, E199, E213, E308, E318, E319</x:v>
+        <x:v>E010, E090, E091, E126, E200, E323, E325, E335</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
       <x:c r="A31" s="10" t="str">
-        <x:v>Phil</x:v>
+        <x:v>Mitch</x:v>
       </x:c>
       <x:c r="B31" s="11" t="str">
-        <x:v>14590126</x:v>
+        <x:v>14590344</x:v>
       </x:c>
       <x:c r="C31" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A31,Exchanges!$J$8:$J$371,B31)</x:f>
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E31" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F31" s="12" t="n">
-        <x:v>46308</x:v>
+        <x:v>46311</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H31" s="10" t="str">
-        <x:v>Valadez</x:v>
-      </x:c>
+        <x:v>Repeated across days</x:v>
+      </x:c>
+      <x:c r="H31" s="10"/>
       <x:c r="I31" s="10" t="str">
-        <x:v>Philip E. Valadez (candidate)</x:v>
+        <x:v>Mitchell R. Godfrey (candidate)</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>Phil is not a unique first name on the roster; Philip Valadez is a candidate because of a separate Valadez hail.</x:v>
+        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
       </x:c>
       <x:c r="K31" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-23, 2026-10-08, 2026-10-09, 2026-10-13</x:v>
+        <x:v>2026-09-12, 2026-09-17, 2026-09-23, 2026-09-25, 2026-09-27, 2026-10-01, 2026-10-15, 2026-10-16</x:v>
       </x:c>
       <x:c r="L31" s="10" t="str">
-        <x:v>E018, E023, E156, E253, E258, E262, E300</x:v>
+        <x:v>E039, E122, E124, E154, E178, E199, E213, E308, E318, E319</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
       <x:c r="A32" s="10" t="str">
-        <x:v>Pitt</x:v>
+        <x:v>Phil</x:v>
       </x:c>
       <x:c r="B32" s="11" t="str">
-        <x:v>14590114</x:v>
+        <x:v>14590126</x:v>
       </x:c>
       <x:c r="C32" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A32,Exchanges!$J$8:$J$371,B32)</x:f>
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E32" s="12" t="n">
-        <x:v>46279</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F32" s="12" t="n">
-        <x:v>46303</x:v>
+        <x:v>46308</x:v>
       </x:c>
       <x:c r="G32" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H32" s="10" t="str">
-        <x:v>Pat (unclear), Peter (unclear)</x:v>
+        <x:v>Valadez</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
-        <x:v>Kyle B. Pitt</x:v>
-      </x:c>
-      <x:c r="J32" s="10"/>
+        <x:v>Philip E. Valadez (candidate)</x:v>
+      </x:c>
+      <x:c r="J32" s="10" t="str">
+        <x:v>Phil is not a unique first name on the roster; Philip Valadez is a candidate because of a separate Valadez hail.</x:v>
+      </x:c>
       <x:c r="K32" s="10" t="str">
-        <x:v>2026-09-14, 2026-10-08</x:v>
+        <x:v>2026-09-11, 2026-09-23, 2026-10-08, 2026-10-09, 2026-10-13</x:v>
       </x:c>
       <x:c r="L32" s="10" t="str">
-        <x:v>E092, E254</x:v>
+        <x:v>E018, E023, E156, E253, E258, E262, E300</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="60" customHeight="1">
       <x:c r="A33" s="10" t="str">
-        <x:v>Renter</x:v>
+        <x:v>Pitt</x:v>
       </x:c>
       <x:c r="B33" s="11" t="str">
-        <x:v>14590087</x:v>
+        <x:v>14590114</x:v>
       </x:c>
       <x:c r="C33" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A33,Exchanges!$J$8:$J$371,B33)</x:f>
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E33" s="12" t="n">
-        <x:v>46278</x:v>
+        <x:v>46279</x:v>
       </x:c>
       <x:c r="F33" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="G33" s="10" t="str">
-        <x:v>Repeated across days</x:v>
-      </x:c>
-      <x:c r="H33" s="10"/>
+        <x:v>Conflicting names on ID</x:v>
+      </x:c>
+      <x:c r="H33" s="10" t="str">
+        <x:v>Pat (unclear), Peter (unclear)</x:v>
+      </x:c>
       <x:c r="I33" s="10" t="str">
-        <x:v>Dustin R. Renter</x:v>
+        <x:v>Kyle B. Pitt</x:v>
       </x:c>
       <x:c r="J33" s="10"/>
       <x:c r="K33" s="10" t="str">
-        <x:v>2026-09-13, 2026-09-17, 2026-09-25, 2026-09-26, 2026-09-30, 2026-10-01, 2026-10-11</x:v>
+        <x:v>2026-09-14, 2026-10-08</x:v>
       </x:c>
       <x:c r="L33" s="10" t="str">
-        <x:v>E075, E078, E120, E121, E174, E186, E191, E210, E215, E290</x:v>
+        <x:v>E092, E254</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
       <x:c r="A34" s="10" t="str">
-        <x:v>Richardson / Cole</x:v>
+        <x:v>Renter</x:v>
       </x:c>
       <x:c r="B34" s="11" t="str">
-        <x:v>14590044</x:v>
+        <x:v>14590087</x:v>
       </x:c>
       <x:c r="C34" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A34,Exchanges!$J$8:$J$371,B34)</x:f>
-        <x:v>5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E34" s="12" t="n">
-        <x:v>46286</x:v>
+        <x:v>46278</x:v>
       </x:c>
       <x:c r="F34" s="12" t="n">
-        <x:v>46311</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G34" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H34" s="10"/>
       <x:c r="I34" s="10" t="str">
-        <x:v>Cole G. Richardson</x:v>
+        <x:v>Dustin R. Renter</x:v>
       </x:c>
       <x:c r="J34" s="10"/>
       <x:c r="K34" s="10" t="str">
-        <x:v>2026-09-21, 2026-09-22, 2026-10-14, 2026-10-16</x:v>
+        <x:v>2026-09-13, 2026-09-17, 2026-09-25, 2026-09-26, 2026-09-30, 2026-10-01, 2026-10-11</x:v>
       </x:c>
       <x:c r="L34" s="10" t="str">
-        <x:v>E140, E146, E148, E304, E321</x:v>
+        <x:v>E075, E078, E120, E121, E174, E186, E191, E210, E215, E290</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="60" customHeight="1">
@@ -1547,20 +1549,20 @@
         <x:v>Richardson / Cole</x:v>
       </x:c>
       <x:c r="B35" s="11" t="str">
-        <x:v>14590123</x:v>
+        <x:v>14590044</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A35,Exchanges!$J$8:$J$371,B35)</x:f>
-        <x:v>12</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E35" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46286</x:v>
       </x:c>
       <x:c r="F35" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46311</x:v>
       </x:c>
       <x:c r="G35" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1571,47 +1573,45 @@
       </x:c>
       <x:c r="J35" s="10"/>
       <x:c r="K35" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-09-13, 2026-09-16, 2026-09-17, 2026-10-01, 2026-10-12</x:v>
+        <x:v>2026-09-21, 2026-09-22, 2026-10-14, 2026-10-16</x:v>
       </x:c>
       <x:c r="L35" s="10" t="str">
-        <x:v>E015, E047, E052, E053, E054, E055, E079, E099, E101, E114, E218, E296</x:v>
+        <x:v>E140, E146, E148, E304, E321</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="60" customHeight="1">
       <x:c r="A36" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Richardson / Cole</x:v>
       </x:c>
       <x:c r="B36" s="11" t="str">
-        <x:v>14590067</x:v>
+        <x:v>14590123</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A36,Exchanges!$J$8:$J$371,B36)</x:f>
-        <x:v>2</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F36" s="12" t="n">
-        <x:v>46303</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="G36" s="10" t="str">
-        <x:v>Owner identified</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H36" s="10"/>
       <x:c r="I36" s="10" t="str">
-        <x:v>Sammantha J. Halladay</x:v>
-      </x:c>
-      <x:c r="J36" s="10" t="str">
-        <x:v>Owner identifies the female reply in October 7 clip 55 as Halladay; October 8 uses the same ID.</x:v>
-      </x:c>
+        <x:v>Cole G. Richardson</x:v>
+      </x:c>
+      <x:c r="J36" s="10"/>
       <x:c r="K36" s="10" t="str">
-        <x:v>2026-10-07, 2026-10-08</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-09-13, 2026-09-16, 2026-09-17, 2026-10-01, 2026-10-12</x:v>
       </x:c>
       <x:c r="L36" s="10" t="str">
-        <x:v>E248, E250</x:v>
+        <x:v>E015, E047, E052, E053, E054, E055, E079, E099, E101, E114, E218, E296</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="60" customHeight="1">
@@ -1619,38 +1619,36 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="B37" s="11" t="str">
-        <x:v>14590100</x:v>
+        <x:v>14590067</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A37,Exchanges!$J$8:$J$371,B37)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E37" s="12" t="n">
-        <x:v>46284</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F37" s="12" t="n">
-        <x:v>46289</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="G37" s="10" t="str">
         <x:v>Owner identified</x:v>
       </x:c>
-      <x:c r="H37" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
-      </x:c>
+      <x:c r="H37" s="10"/>
       <x:c r="I37" s="10" t="str">
         <x:v>Sammantha J. Halladay</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>Owner identifies the September 24 female replies as Halladay. September 19 and Colby references remain unverified.</x:v>
+        <x:v>Owner identifies the female reply in October 7 clip 55 as Halladay; October 8 uses the same ID.</x:v>
       </x:c>
       <x:c r="K37" s="10" t="str">
-        <x:v>2026-09-19, 2026-09-24</x:v>
+        <x:v>2026-10-07, 2026-10-08</x:v>
       </x:c>
       <x:c r="L37" s="10" t="str">
-        <x:v>E130, E163, E164</x:v>
+        <x:v>E248, E250</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="60" customHeight="1">
@@ -1658,36 +1656,38 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="B38" s="11" t="str">
-        <x:v>14590090</x:v>
+        <x:v>14590100</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A38,Exchanges!$J$8:$J$371,B38)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D38" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D38" s="10" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="E38" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46284</x:v>
       </x:c>
       <x:c r="F38" s="12" t="n">
-        <x:v>46293</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="G38" s="10" t="str">
         <x:v>Owner identified</x:v>
       </x:c>
-      <x:c r="H38" s="10"/>
+      <x:c r="H38" s="10" t="str">
+        <x:v>Heaton / Colby</x:v>
+      </x:c>
       <x:c r="I38" s="10" t="str">
-        <x:v>Samuel Canizalez</x:v>
+        <x:v>Sammantha J. Halladay</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>Owner identifies the September 28 Sam replies as Samuel Canizalez.</x:v>
+        <x:v>Owner identifies the September 24 female replies as Halladay. September 19 and Colby references remain unverified.</x:v>
       </x:c>
       <x:c r="K38" s="10" t="str">
-        <x:v>2026-09-28</x:v>
+        <x:v>2026-09-19, 2026-09-24</x:v>
       </x:c>
       <x:c r="L38" s="10" t="str">
-        <x:v>E203, E204</x:v>
+        <x:v>E130, E163, E164</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="60" customHeight="1">
@@ -1695,11 +1695,11 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="B39" s="11" t="str">
-        <x:v>14590066</x:v>
+        <x:v>14590090</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A39,Exchanges!$J$8:$J$371,B39)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
         <x:v>1</x:v>
@@ -1718,13 +1718,13 @@
         <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>Owner identifies Sam on 14590066 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
+        <x:v>Owner identifies the September 28 Sam replies as Samuel Canizalez.</x:v>
       </x:c>
       <x:c r="K39" s="10" t="str">
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="L39" s="10" t="str">
-        <x:v>E205</x:v>
+        <x:v>E203, E204</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="60" customHeight="1">
@@ -1732,7 +1732,7 @@
         <x:v>Sam</x:v>
       </x:c>
       <x:c r="B40" s="11" t="str">
-        <x:v>14590268</x:v>
+        <x:v>14590066</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A40,Exchanges!$J$8:$J$371,B40)</x:f>
@@ -1742,10 +1742,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="F40" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="G40" s="10" t="str">
         <x:v>Owner identified</x:v>
@@ -1755,50 +1755,50 @@
         <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>Owner identifies Sam on 14590268 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
+        <x:v>Owner identifies Sam on 14590066 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="K40" s="10" t="str">
-        <x:v>2026-10-07</x:v>
+        <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="L40" s="10" t="str">
-        <x:v>E247</x:v>
+        <x:v>E205</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="60" customHeight="1">
       <x:c r="A41" s="10" t="str">
-        <x:v>Ron</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B41" s="11" t="str">
-        <x:v>14590037</x:v>
+        <x:v>14590268</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A41,Exchanges!$J$8:$J$371,B41)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F41" s="12" t="n">
-        <x:v>46299</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="G41" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner identified</x:v>
       </x:c>
       <x:c r="H41" s="10"/>
       <x:c r="I41" s="10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Samuel Canizalez</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+        <x:v>Owner identifies Sam on 14590268 as Samuel Canizalez. Full exchange wording remains unverified.</x:v>
       </x:c>
       <x:c r="K41" s="10" t="str">
-        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
+        <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="L41" s="10" t="str">
-        <x:v>E095, E137, E207, E231</x:v>
+        <x:v>E247</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="60" customHeight="1">
@@ -1806,20 +1806,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B42" s="11" t="str">
-        <x:v>14590095</x:v>
+        <x:v>14590037</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A42,Exchanges!$J$8:$J$371,B42)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
-        <x:v>46283</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="F42" s="12" t="n">
-        <x:v>46289</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="G42" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1832,10 +1832,10 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K42" s="10" t="str">
-        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
+        <x:v>2026-09-15, 2026-09-20, 2026-09-28, 2026-10-04</x:v>
       </x:c>
       <x:c r="L42" s="10" t="str">
-        <x:v>E128, E131, E132, E167</x:v>
+        <x:v>E095, E137, E207, E231</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="60" customHeight="1">
@@ -1843,20 +1843,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B43" s="11" t="str">
-        <x:v>14590099</x:v>
+        <x:v>14590095</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A43,Exchanges!$J$8:$J$371,B43)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D43" s="10" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D43" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="E43" s="12" t="n">
-        <x:v>46299</x:v>
+        <x:v>46283</x:v>
       </x:c>
       <x:c r="F43" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46289</x:v>
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1869,10 +1869,10 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K43" s="10" t="str">
-        <x:v>2026-10-04, 2026-10-15</x:v>
+        <x:v>2026-09-18, 2026-09-19, 2026-09-24</x:v>
       </x:c>
       <x:c r="L43" s="10" t="str">
-        <x:v>E232, E233, E312</x:v>
+        <x:v>E128, E131, E132, E167</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="60" customHeight="1">
@@ -1880,20 +1880,20 @@
         <x:v>Ron</x:v>
       </x:c>
       <x:c r="B44" s="11" t="str">
-        <x:v>14590207</x:v>
+        <x:v>14590099</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A44,Exchanges!$J$8:$J$371,B44)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
-        <x:v>46291</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="F44" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G44" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1906,45 +1906,47 @@
         <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
       </x:c>
       <x:c r="K44" s="10" t="str">
-        <x:v>2026-09-26, 2026-10-09</x:v>
+        <x:v>2026-10-04, 2026-10-15</x:v>
       </x:c>
       <x:c r="L44" s="10" t="str">
-        <x:v>E193, E265</x:v>
+        <x:v>E232, E233, E312</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="60" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>Somerville</x:v>
+        <x:v>Ron</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>14590042</x:v>
+        <x:v>14590207</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A45,Exchanges!$J$8:$J$371,B45)</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
-        <x:v>46274</x:v>
+        <x:v>46291</x:v>
       </x:c>
       <x:c r="F45" s="12" t="n">
-        <x:v>46297</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H45" s="10"/>
       <x:c r="I45" s="10" t="str">
-        <x:v>J. Tayler Somerville</x:v>
-      </x:c>
-      <x:c r="J45" s="10"/>
+        <x:v>Unresolved</x:v>
+      </x:c>
+      <x:c r="J45" s="10" t="str">
+        <x:v>Ron could be a name, nickname, or a transcription of Bronson. Several distinct IDs appear; no roster identity assigned.</x:v>
+      </x:c>
       <x:c r="K45" s="10" t="str">
-        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
+        <x:v>2026-09-26, 2026-10-09</x:v>
       </x:c>
       <x:c r="L45" s="10" t="str">
-        <x:v>E001, E096, E170, E222</x:v>
+        <x:v>E193, E265</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="60" customHeight="1">
@@ -1952,20 +1954,20 @@
         <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>14590073</x:v>
+        <x:v>14590042</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A46,Exchanges!$J$8:$J$371,B46)</x:f>
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
-        <x:v>46281</x:v>
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="F46" s="12" t="n">
-        <x:v>46317</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="G46" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -1976,45 +1978,45 @@
       </x:c>
       <x:c r="J46" s="10"/>
       <x:c r="K46" s="10" t="str">
-        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
+        <x:v>2026-09-09, 2026-09-15, 2026-09-24, 2026-10-02</x:v>
       </x:c>
       <x:c r="L46" s="10" t="str">
-        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
+        <x:v>E001, E096, E170, E222</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="60" customHeight="1">
       <x:c r="A47" s="10" t="str">
-        <x:v>Tonga</x:v>
+        <x:v>Somerville</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>14590038</x:v>
+        <x:v>14590073</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A47,Exchanges!$J$8:$J$371,B47)</x:f>
-        <x:v>5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46281</x:v>
       </x:c>
       <x:c r="F47" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46317</x:v>
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H47" s="10"/>
       <x:c r="I47" s="10" t="str">
-        <x:v>Spencer Tonga</x:v>
+        <x:v>J. Tayler Somerville</x:v>
       </x:c>
       <x:c r="J47" s="10"/>
       <x:c r="K47" s="10" t="str">
-        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
+        <x:v>2026-09-16, 2026-09-24, 2026-09-26, 2026-10-02, 2026-10-03, 2026-10-08, 2026-10-09, 2026-10-21, 2026-10-22</x:v>
       </x:c>
       <x:c r="L47" s="10" t="str">
-        <x:v>E071, E085, E183, E278, E333</x:v>
+        <x:v>E097, E168, E169, E182, E223, E227, E255, E256, E339, E351</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="60" customHeight="1">
@@ -2022,20 +2024,20 @@
         <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
-        <x:v>14590345</x:v>
+        <x:v>14590038</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A48,Exchanges!$J$8:$J$371,B48)</x:f>
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F48" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G48" s="10" t="str">
         <x:v>Repeated across days</x:v>
@@ -2046,90 +2048,88 @@
       </x:c>
       <x:c r="J48" s="10"/>
       <x:c r="K48" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
+        <x:v>2026-09-12, 2026-09-14, 2026-09-26, 2026-10-10, 2026-10-20</x:v>
       </x:c>
       <x:c r="L48" s="10" t="str">
-        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
+        <x:v>E071, E085, E183, E278, E333</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="60" customHeight="1">
       <x:c r="A49" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Tonga</x:v>
       </x:c>
       <x:c r="B49" s="11" t="str">
-        <x:v>14590079</x:v>
+        <x:v>14590345</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A49,Exchanges!$J$8:$J$371,B49)</x:f>
-        <x:v>5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E49" s="12" t="n">
-        <x:v>46275</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F49" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G49" s="10" t="str">
         <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H49" s="10"/>
       <x:c r="I49" s="10" t="str">
-        <x:v>Jonathan Wagley</x:v>
+        <x:v>Spencer Tonga</x:v>
       </x:c>
       <x:c r="J49" s="10"/>
       <x:c r="K49" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-09-14, 2026-09-25, 2026-09-26, 2026-10-01, 2026-10-10, 2026-10-11</x:v>
       </x:c>
       <x:c r="L49" s="10" t="str">
-        <x:v>E008, E160, E201, E252, E338</x:v>
+        <x:v>E035, E037, E061, E064, E086, E179, E180, E181, E212, E275, E276, E277, E279, E280</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="60" customHeight="1">
       <x:c r="A50" s="10" t="str">
-        <x:v>Greg</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="B50" s="11" t="str">
-        <x:v>14590026</x:v>
+        <x:v>14590079</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A50,Exchanges!$J$8:$J$371,B50)</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D50" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="F50" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G50" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
+        <x:v>Repeated across days</x:v>
       </x:c>
       <x:c r="H50" s="10"/>
       <x:c r="I50" s="10" t="str">
-        <x:v>Greg B. Mecham</x:v>
-      </x:c>
-      <x:c r="J50" s="10" t="str">
-        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
-      </x:c>
+        <x:v>Jonathan Wagley</x:v>
+      </x:c>
+      <x:c r="J50" s="10"/>
       <x:c r="K50" s="10" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-10, 2026-09-23, 2026-09-28, 2026-10-08, 2026-10-21</x:v>
       </x:c>
       <x:c r="L50" s="10" t="str">
-        <x:v>E034</x:v>
+        <x:v>E008, E160, E201, E252, E338</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
       <x:c r="A51" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Greg</x:v>
       </x:c>
       <x:c r="B51" s="11" t="str">
-        <x:v>14590031</x:v>
+        <x:v>14590026</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A51,Exchanges!$J$8:$J$371,B51)</x:f>
@@ -2139,26 +2139,26 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E51" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F51" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="G51" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H51" s="10"/>
       <x:c r="I51" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
+        <x:v>Greg B. Mecham</x:v>
       </x:c>
       <x:c r="J51" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
+        <x:v>Brief uncertain hail; most other Greg replies use 14590098. Do not assume 14590026 is Greg on other days.</x:v>
       </x:c>
       <x:c r="K51" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="L51" s="10" t="str">
-        <x:v>E260</x:v>
+        <x:v>E034</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
@@ -2166,7 +2166,7 @@
         <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B52" s="11" t="str">
-        <x:v>14590101</x:v>
+        <x:v>14590031</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A52,Exchanges!$J$8:$J$371,B52)</x:f>
@@ -2176,10 +2176,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E52" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F52" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G52" s="10" t="str">
         <x:v>Single-day candidate</x:v>
@@ -2192,18 +2192,18 @@
         <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K52" s="10" t="str">
-        <x:v>2026-09-12</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L52" s="10" t="str">
-        <x:v>E046</x:v>
+        <x:v>E260</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
       <x:c r="A53" s="10" t="str">
-        <x:v>Jackie</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B53" s="11" t="str">
-        <x:v>14590103</x:v>
+        <x:v>14590101</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A53,Exchanges!$J$8:$J$371,B53)</x:f>
@@ -2213,34 +2213,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E53" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="F53" s="12" t="n">
-        <x:v>46307</x:v>
+        <x:v>46277</x:v>
       </x:c>
       <x:c r="G53" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H53" s="10"/>
       <x:c r="I53" s="10" t="str">
-        <x:v>Jaclyn G. Strong (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J53" s="10" t="str">
-        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K53" s="10" t="str">
-        <x:v>2026-10-12</x:v>
+        <x:v>2026-09-12</x:v>
       </x:c>
       <x:c r="L53" s="10" t="str">
-        <x:v>E297</x:v>
+        <x:v>E046</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
       <x:c r="A54" s="10" t="str">
-        <x:v>Kitchen</x:v>
+        <x:v>Jackie</x:v>
       </x:c>
       <x:c r="B54" s="11" t="str">
-        <x:v>14590043</x:v>
+        <x:v>14590103</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A54,Exchanges!$J$8:$J$371,B54)</x:f>
@@ -2250,34 +2250,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E54" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="F54" s="12" t="n">
-        <x:v>46304</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="G54" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H54" s="10"/>
       <x:c r="I54" s="10" t="str">
-        <x:v>Bronson T. Kitchen (candidate)</x:v>
+        <x:v>Jaclyn G. Strong (candidate)</x:v>
       </x:c>
       <x:c r="J54" s="10" t="str">
-        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
+        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
       </x:c>
       <x:c r="K54" s="10" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="L54" s="10" t="str">
-        <x:v>E259</x:v>
+        <x:v>E297</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
       <x:c r="A55" s="10" t="str">
-        <x:v>Laycock</x:v>
+        <x:v>Kitchen</x:v>
       </x:c>
       <x:c r="B55" s="11" t="str">
-        <x:v>14590025</x:v>
+        <x:v>14590043</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A55,Exchanges!$J$8:$J$371,B55)</x:f>
@@ -2287,71 +2287,73 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E55" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="F55" s="12" t="n">
-        <x:v>46287</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="G55" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H55" s="10" t="str">
-        <x:v>Jake</x:v>
-      </x:c>
+        <x:v>Single-day candidate</x:v>
+      </x:c>
+      <x:c r="H55" s="10"/>
       <x:c r="I55" s="10" t="str">
-        <x:v>Jake D. Laycock</x:v>
+        <x:v>Bronson T. Kitchen (candidate)</x:v>
       </x:c>
       <x:c r="J55" s="10" t="str">
-        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+        <x:v>Name is transcribed as [Jason / Kitchen]; audio review needed.</x:v>
       </x:c>
       <x:c r="K55" s="10" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="L55" s="10" t="str">
-        <x:v>E143</x:v>
+        <x:v>E259</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
       <x:c r="A56" s="10" t="str">
-        <x:v>Murray</x:v>
+        <x:v>Laycock</x:v>
       </x:c>
       <x:c r="B56" s="11" t="str">
-        <x:v>14590266</x:v>
+        <x:v>14590025</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A56,Exchanges!$J$8:$J$371,B56)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="F56" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="G56" s="10" t="str">
-        <x:v>Single-day candidate</x:v>
-      </x:c>
-      <x:c r="H56" s="10"/>
+        <x:v>Conflicting names on ID</x:v>
+      </x:c>
+      <x:c r="H56" s="10" t="str">
+        <x:v>Jake</x:v>
+      </x:c>
       <x:c r="I56" s="10" t="str">
-        <x:v>Austin W. Murray</x:v>
-      </x:c>
-      <x:c r="J56" s="10"/>
+        <x:v>Jake D. Laycock</x:v>
+      </x:c>
+      <x:c r="J56" s="10" t="str">
+        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+      </x:c>
       <x:c r="K56" s="10" t="str">
-        <x:v>2026-10-03</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="L56" s="10" t="str">
-        <x:v>E228, E229</x:v>
+        <x:v>E143</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
       <x:c r="A57" s="10" t="str">
-        <x:v>Renter</x:v>
+        <x:v>Murray</x:v>
       </x:c>
       <x:c r="B57" s="11" t="str">
-        <x:v>14590219</x:v>
+        <x:v>14590266</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A57,Exchanges!$J$8:$J$371,B57)</x:f>
@@ -2361,69 +2363,67 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E57" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="F57" s="12" t="n">
-        <x:v>46306</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="G57" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H57" s="10"/>
       <x:c r="I57" s="10" t="str">
-        <x:v>Dustin R. Renter</x:v>
+        <x:v>Austin W. Murray</x:v>
       </x:c>
       <x:c r="J57" s="10"/>
       <x:c r="K57" s="10" t="str">
-        <x:v>2026-10-11</x:v>
+        <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="L57" s="10" t="str">
-        <x:v>E284, E285</x:v>
+        <x:v>E228, E229</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
       <x:c r="A58" s="10" t="str">
-        <x:v>Tyler</x:v>
+        <x:v>Renter</x:v>
       </x:c>
       <x:c r="B58" s="11" t="str">
-        <x:v>14590085</x:v>
+        <x:v>14590219</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A58,Exchanges!$J$8:$J$371,B58)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D58" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E58" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="F58" s="12" t="n">
-        <x:v>46302</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="G58" s="10" t="str">
         <x:v>Single-day candidate</x:v>
       </x:c>
       <x:c r="H58" s="10"/>
       <x:c r="I58" s="10" t="str">
-        <x:v>Unresolved</x:v>
-      </x:c>
-      <x:c r="J58" s="10" t="str">
-        <x:v>Spoken name Tyler; no full-name identity assigned. Do not equate this with Tayler Somerville.</x:v>
-      </x:c>
+        <x:v>Dustin R. Renter</x:v>
+      </x:c>
+      <x:c r="J58" s="10"/>
       <x:c r="K58" s="10" t="str">
-        <x:v>2026-10-07</x:v>
+        <x:v>2026-10-11</x:v>
       </x:c>
       <x:c r="L58" s="10" t="str">
-        <x:v>E249</x:v>
+        <x:v>E284, E285</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
       <x:c r="A59" s="10" t="str">
-        <x:v>Valadez</x:v>
+        <x:v>Tyler</x:v>
       </x:c>
       <x:c r="B59" s="11" t="str">
-        <x:v>14590126</x:v>
+        <x:v>14590085</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A59,Exchanges!$J$8:$J$371,B59)</x:f>
@@ -2433,36 +2433,34 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E59" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="F59" s="12" t="n">
-        <x:v>46280</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="G59" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H59" s="10" t="str">
-        <x:v>Phil</x:v>
-      </x:c>
+        <x:v>Single-day candidate</x:v>
+      </x:c>
+      <x:c r="H59" s="10"/>
       <x:c r="I59" s="10" t="str">
-        <x:v>Mckay or Philip Valadez</x:v>
+        <x:v>Unresolved</x:v>
       </x:c>
       <x:c r="J59" s="10" t="str">
-        <x:v>Surname is uncertain in transcript. Do not use this one exchange to prove which Valadez is speaking.</x:v>
+        <x:v>Spoken name Tyler; no full-name identity assigned. Do not equate this with Tayler Somerville.</x:v>
       </x:c>
       <x:c r="K59" s="10" t="str">
-        <x:v>2026-09-15</x:v>
+        <x:v>2026-10-07</x:v>
       </x:c>
       <x:c r="L59" s="10" t="str">
-        <x:v>E093</x:v>
+        <x:v>E249</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="60" customHeight="1">
       <x:c r="A60" s="10" t="str">
-        <x:v>Colton</x:v>
+        <x:v>Valadez</x:v>
       </x:c>
       <x:c r="B60" s="11" t="str">
-        <x:v>14590091</x:v>
+        <x:v>14590126</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A60,Exchanges!$J$8:$J$371,B60)</x:f>
@@ -2472,67 +2470,67 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E60" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="F60" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="G60" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H60" s="10" t="str">
-        <x:v>Ethan, Heaton / Colby</x:v>
+        <x:v>Phil</x:v>
       </x:c>
       <x:c r="I60" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Mckay or Philip Valadez</x:v>
       </x:c>
       <x:c r="J60" s="10" t="str">
-        <x:v>14590091 also answers Heaton/Colby and Ethan. Could be transcript error, shared radio, or a different responder.</x:v>
+        <x:v>Surname is uncertain in transcript. Do not use this one exchange to prove which Valadez is speaking.</x:v>
       </x:c>
       <x:c r="K60" s="10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-09-15</x:v>
       </x:c>
       <x:c r="L60" s="10" t="str">
-        <x:v>E243</x:v>
+        <x:v>E093</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="60" customHeight="1">
       <x:c r="A61" s="10" t="str">
-        <x:v>Ethan</x:v>
+        <x:v>Colton</x:v>
       </x:c>
       <x:c r="B61" s="11" t="str">
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A61,Exchanges!$J$8:$J$371,B61)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E61" s="12" t="n">
-        <x:v>46292</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="F61" s="12" t="n">
-        <x:v>46292</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="G61" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H61" s="10" t="str">
-        <x:v>Colton, Heaton / Colby</x:v>
+        <x:v>Ethan, Heaton / Colby</x:v>
       </x:c>
       <x:c r="I61" s="10" t="str">
-        <x:v>Ethan C. Simmons</x:v>
+        <x:v>Multiple candidates</x:v>
       </x:c>
       <x:c r="J61" s="10" t="str">
-        <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
+        <x:v>14590091 also answers Heaton/Colby and Ethan. Could be transcript error, shared radio, or a different responder.</x:v>
       </x:c>
       <x:c r="K61" s="10" t="str">
-        <x:v>2026-09-27</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
       <x:c r="L61" s="10" t="str">
-        <x:v>E197, E198</x:v>
+        <x:v>E243</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="60" customHeight="1">
@@ -2540,26 +2538,26 @@
         <x:v>Ethan</x:v>
       </x:c>
       <x:c r="B62" s="11" t="str">
-        <x:v>14590225</x:v>
+        <x:v>14590091</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A62,Exchanges!$J$8:$J$371,B62)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E62" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46292</x:v>
       </x:c>
       <x:c r="F62" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46292</x:v>
       </x:c>
       <x:c r="G62" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H62" s="10" t="str">
-        <x:v>Jensen / Josh</x:v>
+        <x:v>Colton, Heaton / Colby</x:v>
       </x:c>
       <x:c r="I62" s="10" t="str">
         <x:v>Ethan C. Simmons</x:v>
@@ -2568,28 +2566,28 @@
         <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
       </x:c>
       <x:c r="K62" s="10" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-09-27</x:v>
       </x:c>
       <x:c r="L62" s="10" t="str">
-        <x:v>E311</x:v>
+        <x:v>E197, E198</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="60" customHeight="1">
       <x:c r="A63" s="10" t="str">
-        <x:v>Hawkins</x:v>
+        <x:v>Ethan</x:v>
       </x:c>
       <x:c r="B63" s="11" t="str">
-        <x:v>14590036</x:v>
+        <x:v>14590225</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A63,Exchanges!$J$8:$J$371,B63)</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E63" s="12" t="n">
-        <x:v>46276</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="F63" s="12" t="n">
         <x:v>46310</x:v>
@@ -2598,58 +2596,58 @@
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H63" s="10" t="str">
-        <x:v>Mitch</x:v>
+        <x:v>Jensen / Josh</x:v>
       </x:c>
       <x:c r="I63" s="10" t="str">
-        <x:v>Steven G. Hawkins</x:v>
+        <x:v>Ethan C. Simmons</x:v>
       </x:c>
       <x:c r="J63" s="10" t="str">
-        <x:v>14590036 also answers hails to Mitch. Keep this as an exchange-level association.</x:v>
+        <x:v>14590091 also answers Heaton/Colby and Colton; 14590225 also answers Josh. Response adjacency may identify a crew or a different responder.</x:v>
       </x:c>
       <x:c r="K63" s="10" t="str">
-        <x:v>2026-09-11, 2026-09-12, 2026-10-15</x:v>
+        <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="L63" s="10" t="str">
-        <x:v>E026, E068, E070, E317</x:v>
+        <x:v>E311</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="60" customHeight="1">
       <x:c r="A64" s="10" t="str">
-        <x:v>Heaton / Colby</x:v>
+        <x:v>Hawkins</x:v>
       </x:c>
       <x:c r="B64" s="11" t="str">
-        <x:v>14590091</x:v>
+        <x:v>14590036</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A64,Exchanges!$J$8:$J$371,B64)</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E64" s="12" t="n">
-        <x:v>46290</x:v>
+        <x:v>46276</x:v>
       </x:c>
       <x:c r="F64" s="12" t="n">
-        <x:v>46290</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G64" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H64" s="10" t="str">
-        <x:v>Colton, Ethan</x:v>
+        <x:v>Mitch</x:v>
       </x:c>
       <x:c r="I64" s="10" t="str">
-        <x:v>Colby A. Heaton</x:v>
+        <x:v>Steven G. Hawkins</x:v>
       </x:c>
       <x:c r="J64" s="10" t="str">
-        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
+        <x:v>14590036 also answers hails to Mitch. Keep this as an exchange-level association.</x:v>
       </x:c>
       <x:c r="K64" s="10" t="str">
-        <x:v>2026-09-25</x:v>
+        <x:v>2026-09-11, 2026-09-12, 2026-10-15</x:v>
       </x:c>
       <x:c r="L64" s="10" t="str">
-        <x:v>E173, E175</x:v>
+        <x:v>E026, E068, E070, E317</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="60" customHeight="1">
@@ -2657,26 +2655,26 @@
         <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B65" s="11" t="str">
-        <x:v>14590100</x:v>
+        <x:v>14590091</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A65,Exchanges!$J$8:$J$371,B65)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E65" s="12" t="n">
-        <x:v>46309</x:v>
+        <x:v>46290</x:v>
       </x:c>
       <x:c r="F65" s="12" t="n">
-        <x:v>46315</x:v>
+        <x:v>46290</x:v>
       </x:c>
       <x:c r="G65" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H65" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Colton, Ethan</x:v>
       </x:c>
       <x:c r="I65" s="10" t="str">
         <x:v>Colby A. Heaton</x:v>
@@ -2685,57 +2683,57 @@
         <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K65" s="10" t="str">
-        <x:v>2026-10-14, 2026-10-20</x:v>
+        <x:v>2026-09-25</x:v>
       </x:c>
       <x:c r="L65" s="10" t="str">
-        <x:v>E301, E329, E331</x:v>
+        <x:v>E173, E175</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="60" customHeight="1">
       <x:c r="A66" s="10" t="str">
-        <x:v>Jensen / Josh</x:v>
+        <x:v>Heaton / Colby</x:v>
       </x:c>
       <x:c r="B66" s="11" t="str">
-        <x:v>14590225</x:v>
+        <x:v>14590100</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A66,Exchanges!$J$8:$J$371,B66)</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D66" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E66" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="F66" s="12" t="n">
-        <x:v>46300</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="G66" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H66" s="10" t="str">
-        <x:v>Ethan</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="I66" s="10" t="str">
-        <x:v>Joshua M. Jensen (candidate)</x:v>
+        <x:v>Colby A. Heaton</x:v>
       </x:c>
       <x:c r="J66" s="10" t="str">
-        <x:v>Both Jensen and Josh are represented; Joshua Jensen is a candidate. First-name replies alone do not rule out other Joshuas.</x:v>
+        <x:v>Includes both Heaton and Colby hails. 14590100 also answers Sam; 14590091 answers other names. Officer/crew assignment is unresolved.</x:v>
       </x:c>
       <x:c r="K66" s="10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-14, 2026-10-20</x:v>
       </x:c>
       <x:c r="L66" s="10" t="str">
-        <x:v>E237</x:v>
+        <x:v>E301, E329, E331</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="60" customHeight="1">
       <x:c r="A67" s="10" t="str">
-        <x:v>Luke</x:v>
+        <x:v>Jensen / Josh</x:v>
       </x:c>
       <x:c r="B67" s="11" t="str">
-        <x:v>14590221</x:v>
+        <x:v>14590225</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A67,Exchanges!$J$8:$J$371,B67)</x:f>
@@ -2745,217 +2743,219 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E67" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="F67" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="G67" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H67" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Ethan</x:v>
       </x:c>
       <x:c r="I67" s="10" t="str">
-        <x:v>Luke A. Sumbot</x:v>
+        <x:v>Joshua M. Jensen (candidate)</x:v>
       </x:c>
       <x:c r="J67" s="10" t="str">
-        <x:v>14590221 also answers hails to Sam. This short reply does not establish that the transmitter is Luke.</x:v>
+        <x:v>Both Jensen and Josh are represented; Joshua Jensen is a candidate. First-name replies alone do not rule out other Joshuas.</x:v>
       </x:c>
       <x:c r="K67" s="10" t="str">
-        <x:v>2026-10-21</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
       <x:c r="L67" s="10" t="str">
-        <x:v>E334</x:v>
+        <x:v>E237</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="60" customHeight="1">
       <x:c r="A68" s="10" t="str">
-        <x:v>McClellan / Dennis</x:v>
+        <x:v>Luke</x:v>
       </x:c>
       <x:c r="B68" s="11" t="str">
-        <x:v>14590019</x:v>
+        <x:v>14590221</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A68,Exchanges!$J$8:$J$371,B68)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E68" s="12" t="n">
-        <x:v>46294</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="F68" s="12" t="n">
-        <x:v>46298</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="G68" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H68" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="I68" s="10" t="str">
-        <x:v>Dennis R. McClellan</x:v>
-      </x:c>
-      <x:c r="J68" s="10"/>
+        <x:v>Luke A. Sumbot</x:v>
+      </x:c>
+      <x:c r="J68" s="10" t="str">
+        <x:v>14590221 also answers hails to Sam. This short reply does not establish that the transmitter is Luke.</x:v>
+      </x:c>
       <x:c r="K68" s="10" t="str">
-        <x:v>2026-09-29, 2026-10-02, 2026-10-03</x:v>
+        <x:v>2026-10-21</x:v>
       </x:c>
       <x:c r="L68" s="10" t="str">
-        <x:v>E208, E221, E226</x:v>
+        <x:v>E334</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="60" customHeight="1">
       <x:c r="A69" s="10" t="str">
-        <x:v>Mitch</x:v>
+        <x:v>McClellan / Dennis</x:v>
       </x:c>
       <x:c r="B69" s="11" t="str">
-        <x:v>14590036</x:v>
+        <x:v>14590019</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A69,Exchanges!$J$8:$J$371,B69)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D69" s="10" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E69" s="12" t="n">
-        <x:v>46281</x:v>
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="F69" s="12" t="n">
-        <x:v>46310</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="G69" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H69" s="10" t="str">
-        <x:v>Hawkins</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="I69" s="10" t="str">
-        <x:v>Mitchell R. Godfrey (candidate)</x:v>
-      </x:c>
-      <x:c r="J69" s="10" t="str">
-        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
-      </x:c>
+        <x:v>Dennis R. McClellan</x:v>
+      </x:c>
+      <x:c r="J69" s="10"/>
       <x:c r="K69" s="10" t="str">
-        <x:v>2026-09-16, 2026-10-15</x:v>
+        <x:v>2026-09-29, 2026-10-02, 2026-10-03</x:v>
       </x:c>
       <x:c r="L69" s="10" t="str">
-        <x:v>E110, E313, E316</x:v>
+        <x:v>E208, E221, E226</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="60" customHeight="1">
       <x:c r="A70" s="10" t="str">
-        <x:v>Sam</x:v>
+        <x:v>Mitch</x:v>
       </x:c>
       <x:c r="B70" s="11" t="str">
-        <x:v>14590221</x:v>
+        <x:v>14590036</x:v>
       </x:c>
       <x:c r="C70" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A70,Exchanges!$J$8:$J$371,B70)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D70" s="10" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E70" s="12" t="n">
-        <x:v>46285</x:v>
+        <x:v>46281</x:v>
       </x:c>
       <x:c r="F70" s="12" t="n">
-        <x:v>46312</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="G70" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H70" s="10" t="str">
-        <x:v>Luke</x:v>
+        <x:v>Hawkins</x:v>
       </x:c>
       <x:c r="I70" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Mitchell R. Godfrey (candidate)</x:v>
       </x:c>
       <x:c r="J70" s="10" t="str">
-        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+        <x:v>14590036 also answers Hawkins. Keep 14590344 separate from 14590036 pending audio and assignment confirmation.</x:v>
       </x:c>
       <x:c r="K70" s="10" t="str">
-        <x:v>2026-09-20, 2026-10-13, 2026-10-17</x:v>
+        <x:v>2026-09-16, 2026-10-15</x:v>
       </x:c>
       <x:c r="L70" s="10" t="str">
-        <x:v>E134, E298, E324</x:v>
+        <x:v>E110, E313, E316</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="60" customHeight="1">
       <x:c r="A71" s="10" t="str">
-        <x:v>Wagley</x:v>
+        <x:v>Sam</x:v>
       </x:c>
       <x:c r="B71" s="11" t="str">
-        <x:v>14590019</x:v>
+        <x:v>14590221</x:v>
       </x:c>
       <x:c r="C71" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A71,Exchanges!$J$8:$J$371,B71)</x:f>
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D71" s="10" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E71" s="12" t="n">
-        <x:v>46275</x:v>
+        <x:v>46285</x:v>
       </x:c>
       <x:c r="F71" s="12" t="n">
-        <x:v>46288</x:v>
+        <x:v>46312</x:v>
       </x:c>
       <x:c r="G71" s="10" t="str">
         <x:v>Conflicting names on ID</x:v>
       </x:c>
       <x:c r="H71" s="10" t="str">
-        <x:v>McClellan / Dennis</x:v>
+        <x:v>Luke</x:v>
       </x:c>
       <x:c r="I71" s="10" t="str">
-        <x:v>Jonathan Wagley</x:v>
-      </x:c>
-      <x:c r="J71" s="10"/>
+        <x:v>Multiple candidates</x:v>
+      </x:c>
+      <x:c r="J71" s="10" t="str">
+        <x:v>Several officers use Sam or Samuel. Do not combine these IDs into one officer identity.</x:v>
+      </x:c>
       <x:c r="K71" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-19, 2026-09-23</x:v>
+        <x:v>2026-09-20, 2026-10-13, 2026-10-17</x:v>
       </x:c>
       <x:c r="L71" s="10" t="str">
-        <x:v>E003, E006, E007, E129, E159</x:v>
+        <x:v>E134, E298, E324</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="60" customHeight="1">
       <x:c r="A72" s="10" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Wagley</x:v>
       </x:c>
       <x:c r="B72" s="11" t="str">
-        <x:v>14590105</x:v>
+        <x:v>14590019</x:v>
       </x:c>
       <x:c r="C72" s="10" t="n">
         <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A72,Exchanges!$J$8:$J$371,B72)</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D72" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E72" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="F72" s="12" t="n">
-        <x:v>46277</x:v>
+        <x:v>46288</x:v>
       </x:c>
       <x:c r="G72" s="10" t="str">
-        <x:v>Name spelling unresolved</x:v>
-      </x:c>
-      <x:c r="H72" s="10"/>
+        <x:v>Conflicting names on ID</x:v>
+      </x:c>
+      <x:c r="H72" s="10" t="str">
+        <x:v>McClellan / Dennis</x:v>
+      </x:c>
       <x:c r="I72" s="10" t="str">
-        <x:v>Unresolved</x:v>
-      </x:c>
-      <x:c r="J72" s="10" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
-      </x:c>
+        <x:v>Jonathan Wagley</x:v>
+      </x:c>
+      <x:c r="J72" s="10"/>
       <x:c r="K72" s="10" t="str">
-        <x:v>2026-09-12</x:v>
+        <x:v>2026-09-10, 2026-09-19, 2026-09-23</x:v>
       </x:c>
       <x:c r="L72" s="10" t="str">
-        <x:v>E050, E062</x:v>
+        <x:v>E003, E006, E007, E129, E159</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="60" customHeight="1">
@@ -3297,7 +3297,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f3a02ba1fc4e56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R119bb1e2055f4e50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6399,7 +6399,7 @@
         <x:v>E050</x:v>
       </x:c>
       <x:c r="B57" s="13" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="C57" s="14" t="n">
         <x:v>46277</x:v>
@@ -6427,19 +6427,19 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="K57" s="13" t="str">
-        <x:v>[Mackay?], you arrived? I'm parked on the northeast side of the complex.</x:v>
+        <x:v>Makai, are you arrived? I'm parked on the northeast side of the complex.</x:v>
       </x:c>
       <x:c r="L57" s="13" t="str">
         <x:v>Negative, I'm leaving the PD right now.</x:v>
       </x:c>
       <x:c r="M57" s="13" t="str">
-        <x:v>Name spelling unresolved</x:v>
+        <x:v>Named response association</x:v>
       </x:c>
       <x:c r="N57" s="13" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
+        <x:v>Owner corrected the addressed name to Makai and verified the question. The reply uses 14590105; its full wording has not been independently verified.</x:v>
       </x:c>
       <x:c r="O57" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner reviewed question</x:v>
       </x:c>
       <x:c r="P57" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-12/dcfems-6001-1789239688.m4a</x:v>
@@ -7105,7 +7105,7 @@
         <x:v>E062</x:v>
       </x:c>
       <x:c r="B69" s="13" t="str">
-        <x:v>McKay / Makai (unclear)</x:v>
+        <x:v>Makai / Kelepi</x:v>
       </x:c>
       <x:c r="C69" s="14" t="n">
         <x:v>46277</x:v>
@@ -7133,19 +7133,19 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="K69" s="13" t="str">
-        <x:v>Hey, [Mackay?], there was a phone under your car. [Is it yours?]</x:v>
+        <x:v>Hey, Makai, there was a phone under your car. Is it yours?</x:v>
       </x:c>
       <x:c r="L69" s="13" t="str">
         <x:v>A phone under my car?</x:v>
       </x:c>
       <x:c r="M69" s="13" t="str">
-        <x:v>Name spelling unresolved</x:v>
+        <x:v>Named response association</x:v>
       </x:c>
       <x:c r="N69" s="13" t="str">
-        <x:v>McKay and Makai are different roster names. Do not merge these IDs with either person without audio review.</x:v>
+        <x:v>Owner corrected the addressed name to Makai and verified the question. The reply uses 14590105; its full wording has not been independently verified.</x:v>
       </x:c>
       <x:c r="O69" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner reviewed question</x:v>
       </x:c>
       <x:c r="P69" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-09-12/dcfems-6001-1789257404.m4a</x:v>
@@ -24904,7 +24904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b03d9616aa14153"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf72f5adf98714fe9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25396,7 +25396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R821ecce7ecbb4586"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R418651804c124fb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26361,7 +26361,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1143a5ea2e9f488b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bc226f72d04874"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Confirm Jackie Strong on October 4 and add dated radio associations
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -214,8 +214,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S371" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:S371"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S372" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:S372"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Name in exchange"/>
@@ -529,7 +529,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="str">
-        <x:v>September 9–October 22, 2026. Transcript associations only; audio has not been reviewed for this collation.</x:v>
+        <x:v>September 9–October 22, 2026. Transcript associations, with October 4 Jackie identification confirmed by the owner on October 27.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -545,7 +545,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 364 selected exchanges.</x:v>
+        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 365 selected exchanges.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -651,7 +651,7 @@
         <x:v>14580155</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A10,Exchanges!$J$8:$J$371,B10)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A10,Exchanges!$J$8:$J$372,B10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -686,7 +686,7 @@
         <x:v>14590020</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A11,Exchanges!$J$8:$J$371,B11)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A11,Exchanges!$J$8:$J$372,B11)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -721,7 +721,7 @@
         <x:v>14590089</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A12,Exchanges!$J$8:$J$371,B12)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A12,Exchanges!$J$8:$J$372,B12)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -756,7 +756,7 @@
         <x:v>14590111</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A13,Exchanges!$J$8:$J$371,B13)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A13,Exchanges!$J$8:$J$372,B13)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -791,7 +791,7 @@
         <x:v>14580152</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A14,Exchanges!$J$8:$J$371,B14)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A14,Exchanges!$J$8:$J$372,B14)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -826,7 +826,7 @@
         <x:v>14590098</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A15,Exchanges!$J$8:$J$371,B15)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A15,Exchanges!$J$8:$J$372,B15)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -863,7 +863,7 @@
         <x:v>14590107</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A16,Exchanges!$J$8:$J$371,B16)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A16,Exchanges!$J$8:$J$372,B16)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -898,8 +898,8 @@
         <x:v>14590104</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A17,Exchanges!$J$8:$J$371,B17)</x:f>
-        <x:v>4</x:v>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A17,Exchanges!$J$8:$J$372,B17)</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
         <x:v>4</x:v>
@@ -915,16 +915,16 @@
       </x:c>
       <x:c r="H17" s="10"/>
       <x:c r="I17" s="10" t="str">
-        <x:v>Jaclyn G. Strong (candidate)</x:v>
+        <x:v>Jaclyn G. Strong</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
-        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
+        <x:v>Owner confirms Jaclyn G. Strong on 14590104 for October 4 only. Clip 8 corrected to Jackie? and transcript verified; other transcript verification flags are unchanged. Earlier dates remain transcript associations.</x:v>
       </x:c>
       <x:c r="K17" s="10" t="str">
         <x:v>2026-09-10, 2026-09-11, 2026-10-03, 2026-10-04</x:v>
       </x:c>
       <x:c r="L17" s="10" t="str">
-        <x:v>E012, E013, E224, E234</x:v>
+        <x:v>E012, E013, E224, E234, E365</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -935,7 +935,7 @@
         <x:v>14590200</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A18,Exchanges!$J$8:$J$371,B18)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A18,Exchanges!$J$8:$J$372,B18)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
@@ -972,7 +972,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A19,Exchanges!$J$8:$J$371,B19)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A19,Exchanges!$J$8:$J$372,B19)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
@@ -1011,7 +1011,7 @@
         <x:v>14590118</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A20,Exchanges!$J$8:$J$371,B20)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A20,Exchanges!$J$8:$J$372,B20)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
@@ -1048,7 +1048,7 @@
         <x:v>14590088</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A21,Exchanges!$J$8:$J$371,B21)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A21,Exchanges!$J$8:$J$372,B21)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
@@ -1085,7 +1085,7 @@
         <x:v>14590117</x:v>
       </x:c>
       <x:c r="C22" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A22,Exchanges!$J$8:$J$371,B22)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A22,Exchanges!$J$8:$J$372,B22)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
@@ -1120,7 +1120,7 @@
         <x:v>14590320</x:v>
       </x:c>
       <x:c r="C23" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A23,Exchanges!$J$8:$J$371,B23)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A23,Exchanges!$J$8:$J$372,B23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="10" t="n">
@@ -1155,7 +1155,7 @@
         <x:v>14590084</x:v>
       </x:c>
       <x:c r="C24" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A24,Exchanges!$J$8:$J$371,B24)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A24,Exchanges!$J$8:$J$372,B24)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D24" s="10" t="n">
@@ -1192,7 +1192,7 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="C25" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A25,Exchanges!$J$8:$J$371,B25)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A25,Exchanges!$J$8:$J$372,B25)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
@@ -1229,7 +1229,7 @@
         <x:v>14590237</x:v>
       </x:c>
       <x:c r="C26" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A26,Exchanges!$J$8:$J$371,B26)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A26,Exchanges!$J$8:$J$372,B26)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
@@ -1264,7 +1264,7 @@
         <x:v>14590315</x:v>
       </x:c>
       <x:c r="C27" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A27,Exchanges!$J$8:$J$371,B27)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A27,Exchanges!$J$8:$J$372,B27)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
@@ -1299,7 +1299,7 @@
         <x:v>14590162</x:v>
       </x:c>
       <x:c r="C28" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A28,Exchanges!$J$8:$J$371,B28)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A28,Exchanges!$J$8:$J$372,B28)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
@@ -1334,7 +1334,7 @@
         <x:v>14590081</x:v>
       </x:c>
       <x:c r="C29" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A29,Exchanges!$J$8:$J$371,B29)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A29,Exchanges!$J$8:$J$372,B29)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
@@ -1369,7 +1369,7 @@
         <x:v>14590102</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A30,Exchanges!$J$8:$J$371,B30)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A30,Exchanges!$J$8:$J$372,B30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
@@ -1404,7 +1404,7 @@
         <x:v>14590344</x:v>
       </x:c>
       <x:c r="C31" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A31,Exchanges!$J$8:$J$371,B31)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A31,Exchanges!$J$8:$J$372,B31)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
@@ -1441,7 +1441,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C32" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A32,Exchanges!$J$8:$J$371,B32)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A32,Exchanges!$J$8:$J$372,B32)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
@@ -1480,7 +1480,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C33" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A33,Exchanges!$J$8:$J$371,B33)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A33,Exchanges!$J$8:$J$372,B33)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
@@ -1517,7 +1517,7 @@
         <x:v>14590087</x:v>
       </x:c>
       <x:c r="C34" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A34,Exchanges!$J$8:$J$371,B34)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A34,Exchanges!$J$8:$J$372,B34)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
@@ -1552,7 +1552,7 @@
         <x:v>14590044</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A35,Exchanges!$J$8:$J$371,B35)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A35,Exchanges!$J$8:$J$372,B35)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
@@ -1587,7 +1587,7 @@
         <x:v>14590123</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A36,Exchanges!$J$8:$J$371,B36)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A36,Exchanges!$J$8:$J$372,B36)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
@@ -1622,7 +1622,7 @@
         <x:v>14590067</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A37,Exchanges!$J$8:$J$371,B37)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A37,Exchanges!$J$8:$J$372,B37)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
@@ -1659,7 +1659,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A38,Exchanges!$J$8:$J$371,B38)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A38,Exchanges!$J$8:$J$372,B38)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D38" s="10" t="n">
@@ -1698,7 +1698,7 @@
         <x:v>14590090</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A39,Exchanges!$J$8:$J$371,B39)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A39,Exchanges!$J$8:$J$372,B39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
@@ -1735,7 +1735,7 @@
         <x:v>14590066</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A40,Exchanges!$J$8:$J$371,B40)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A40,Exchanges!$J$8:$J$372,B40)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
@@ -1772,7 +1772,7 @@
         <x:v>14590268</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A41,Exchanges!$J$8:$J$371,B41)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A41,Exchanges!$J$8:$J$372,B41)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
@@ -1809,7 +1809,7 @@
         <x:v>14590037</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A42,Exchanges!$J$8:$J$371,B42)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A42,Exchanges!$J$8:$J$372,B42)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
@@ -1846,7 +1846,7 @@
         <x:v>14590095</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A43,Exchanges!$J$8:$J$371,B43)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A43,Exchanges!$J$8:$J$372,B43)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
@@ -1883,7 +1883,7 @@
         <x:v>14590099</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A44,Exchanges!$J$8:$J$371,B44)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A44,Exchanges!$J$8:$J$372,B44)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
@@ -1920,7 +1920,7 @@
         <x:v>14590207</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A45,Exchanges!$J$8:$J$371,B45)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A45,Exchanges!$J$8:$J$372,B45)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
@@ -1957,7 +1957,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A46,Exchanges!$J$8:$J$371,B46)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A46,Exchanges!$J$8:$J$372,B46)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
@@ -1992,7 +1992,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A47,Exchanges!$J$8:$J$371,B47)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A47,Exchanges!$J$8:$J$372,B47)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
@@ -2027,7 +2027,7 @@
         <x:v>14590038</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A48,Exchanges!$J$8:$J$371,B48)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A48,Exchanges!$J$8:$J$372,B48)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
@@ -2062,7 +2062,7 @@
         <x:v>14590345</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A49,Exchanges!$J$8:$J$371,B49)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A49,Exchanges!$J$8:$J$372,B49)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
@@ -2097,7 +2097,7 @@
         <x:v>14590079</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A50,Exchanges!$J$8:$J$371,B50)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A50,Exchanges!$J$8:$J$372,B50)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D50" s="10" t="n">
@@ -2132,7 +2132,7 @@
         <x:v>14590026</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A51,Exchanges!$J$8:$J$371,B51)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A51,Exchanges!$J$8:$J$372,B51)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D51" s="10" t="n">
@@ -2169,7 +2169,7 @@
         <x:v>14590031</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A52,Exchanges!$J$8:$J$371,B52)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A52,Exchanges!$J$8:$J$372,B52)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D52" s="10" t="n">
@@ -2206,7 +2206,7 @@
         <x:v>14590101</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A53,Exchanges!$J$8:$J$371,B53)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A53,Exchanges!$J$8:$J$372,B53)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D53" s="10" t="n">
@@ -2243,7 +2243,7 @@
         <x:v>14590103</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A54,Exchanges!$J$8:$J$371,B54)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A54,Exchanges!$J$8:$J$372,B54)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
@@ -2280,7 +2280,7 @@
         <x:v>14590043</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A55,Exchanges!$J$8:$J$371,B55)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A55,Exchanges!$J$8:$J$372,B55)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
@@ -2317,7 +2317,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A56,Exchanges!$J$8:$J$371,B56)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A56,Exchanges!$J$8:$J$372,B56)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
@@ -2356,7 +2356,7 @@
         <x:v>14590266</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A57,Exchanges!$J$8:$J$371,B57)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A57,Exchanges!$J$8:$J$372,B57)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D57" s="10" t="n">
@@ -2391,7 +2391,7 @@
         <x:v>14590219</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A58,Exchanges!$J$8:$J$371,B58)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A58,Exchanges!$J$8:$J$372,B58)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D58" s="10" t="n">
@@ -2426,7 +2426,7 @@
         <x:v>14590085</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A59,Exchanges!$J$8:$J$371,B59)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A59,Exchanges!$J$8:$J$372,B59)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="10" t="n">
@@ -2463,7 +2463,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A60,Exchanges!$J$8:$J$371,B60)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A60,Exchanges!$J$8:$J$372,B60)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D60" s="10" t="n">
@@ -2502,7 +2502,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A61,Exchanges!$J$8:$J$371,B61)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A61,Exchanges!$J$8:$J$372,B61)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
@@ -2541,7 +2541,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A62,Exchanges!$J$8:$J$371,B62)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A62,Exchanges!$J$8:$J$372,B62)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
@@ -2580,7 +2580,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A63,Exchanges!$J$8:$J$371,B63)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A63,Exchanges!$J$8:$J$372,B63)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
@@ -2619,7 +2619,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A64,Exchanges!$J$8:$J$371,B64)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A64,Exchanges!$J$8:$J$372,B64)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
@@ -2658,7 +2658,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A65,Exchanges!$J$8:$J$371,B65)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A65,Exchanges!$J$8:$J$372,B65)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
@@ -2697,7 +2697,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A66,Exchanges!$J$8:$J$371,B66)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A66,Exchanges!$J$8:$J$372,B66)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D66" s="10" t="n">
@@ -2736,7 +2736,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A67,Exchanges!$J$8:$J$371,B67)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A67,Exchanges!$J$8:$J$372,B67)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D67" s="10" t="n">
@@ -2775,7 +2775,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A68,Exchanges!$J$8:$J$371,B68)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A68,Exchanges!$J$8:$J$372,B68)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
@@ -2814,7 +2814,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A69,Exchanges!$J$8:$J$371,B69)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A69,Exchanges!$J$8:$J$372,B69)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D69" s="10" t="n">
@@ -2851,7 +2851,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C70" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A70,Exchanges!$J$8:$J$371,B70)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A70,Exchanges!$J$8:$J$372,B70)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D70" s="10" t="n">
@@ -2890,7 +2890,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C71" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A71,Exchanges!$J$8:$J$371,B71)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A71,Exchanges!$J$8:$J$372,B71)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D71" s="10" t="n">
@@ -2929,7 +2929,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C72" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A72,Exchanges!$J$8:$J$371,B72)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A72,Exchanges!$J$8:$J$372,B72)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D72" s="10" t="n">
@@ -2966,7 +2966,7 @@
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="C73" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A73,Exchanges!$J$8:$J$371,B73)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A73,Exchanges!$J$8:$J$372,B73)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D73" s="10" t="n">
@@ -3003,7 +3003,7 @@
         <x:v>14590112</x:v>
       </x:c>
       <x:c r="C74" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A74,Exchanges!$J$8:$J$371,B74)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A74,Exchanges!$J$8:$J$372,B74)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D74" s="10" t="n">
@@ -3040,7 +3040,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C75" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A75,Exchanges!$J$8:$J$371,B75)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A75,Exchanges!$J$8:$J$372,B75)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D75" s="10" t="n">
@@ -3079,7 +3079,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C76" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A76,Exchanges!$J$8:$J$371,B76)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A76,Exchanges!$J$8:$J$372,B76)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D76" s="10" t="n">
@@ -3118,7 +3118,7 @@
         <x:v>14590097</x:v>
       </x:c>
       <x:c r="C77" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A77,Exchanges!$J$8:$J$371,B77)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A77,Exchanges!$J$8:$J$372,B77)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D77" s="10" t="n">
@@ -3155,7 +3155,7 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C78" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A78,Exchanges!$J$8:$J$371,B78)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A78,Exchanges!$J$8:$J$372,B78)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D78" s="10" t="n">
@@ -3192,7 +3192,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C79" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A79,Exchanges!$J$8:$J$371,B79)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A79,Exchanges!$J$8:$J$372,B79)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="10" t="n">
@@ -3231,7 +3231,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C80" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$371,A80,Exchanges!$J$8:$J$371,B80)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A80,Exchanges!$J$8:$J$372,B80)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D80" s="10" t="n">
@@ -17218,7 +17218,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N241" s="13" t="str">
-        <x:v>Mostly 14590104 and 14590200; 14590103 has only one uncertain exchange. No roster identity assigned from the nickname alone.</x:v>
+        <x:v>Owner confirms Jaclyn G. Strong on 14590104 for October 4 only. Clip 8 corrected to Jackie? and transcript verified; other transcript verification flags are unchanged. Earlier dates remain transcript associations.</x:v>
       </x:c>
       <x:c r="O241" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -24894,6 +24894,66 @@
       </x:c>
       <x:c r="S371" s="13" t="n">
         <x:v>76</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372">
+      <x:c r="A372" s="13" t="str">
+        <x:v>E365</x:v>
+      </x:c>
+      <x:c r="B372" s="13" t="str">
+        <x:v>Jackie</x:v>
+      </x:c>
+      <x:c r="C372" s="14" t="n">
+        <x:v>46299</x:v>
+      </x:c>
+      <x:c r="D372" s="13" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E372" s="15" t="n">
+        <x:v>0.024710648148148148</x:v>
+      </x:c>
+      <x:c r="F372" s="16" t="str">
+        <x:v>14590085</x:v>
+      </x:c>
+      <x:c r="G372" s="13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H372" s="15" t="n">
+        <x:v>0.02474537037037037</x:v>
+      </x:c>
+      <x:c r="I372" s="17" t="n">
+        <x:f>ROUND((H372-E372)*86400,0)</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J372" s="16" t="str">
+        <x:v>14590104</x:v>
+      </x:c>
+      <x:c r="K372" s="13" t="str">
+        <x:v>Jackie?</x:v>
+      </x:c>
+      <x:c r="L372" s="13" t="str">
+        <x:v>Yeah.</x:v>
+      </x:c>
+      <x:c r="M372" s="13" t="str">
+        <x:v>Owner-confirmed this day</x:v>
+      </x:c>
+      <x:c r="N372" s="13" t="str">
+        <x:v>Owner confirms Jaclyn G. Strong on 14590104 for October 4 only. Clip 8 corrected to Jackie? and transcript verified; other transcript verification flags are unchanged. Earlier dates remain transcript associations.</x:v>
+      </x:c>
+      <x:c r="O372" s="18" t="str">
+        <x:v>Owner reviewed hail and confirmed day identity; reply text not separately verified</x:v>
+      </x:c>
+      <x:c r="P372" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-04/dcfems-6001-1791095735.m4a</x:v>
+      </x:c>
+      <x:c r="Q372" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-04/dcfems-6001-1791095738.m4a</x:v>
+      </x:c>
+      <x:c r="R372" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-04</x:v>
+      </x:c>
+      <x:c r="S372" s="13" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -25481,7 +25541,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>The selected examples are a research index, not an exhaustive list. October 27 owner identification groups Tanner, T-Ball and G-Ball as Tanner Ballamis. Seven earlier response pairs added; 10 pairs across four days use 14580151.</x:v>
+        <x:v>The selected examples are a research index, not an exhaustive list. October 27 owner identification groups Tanner, T-Ball and G-Ball as Tanner Ballamis. October 4 clips 8–9 added as owner-confirmed Jackie / Jaclyn Strong evidence; confirmation applies to that day only.</x:v>
       </x:c>
       <x:c r="B8" s="2"/>
       <x:c r="C8" s="2"/>

</xml_diff>

<commit_message>
Add independent Law 2 listening page and publish October 4 Manis corrections
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -194,7 +194,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RadioFindings" displayName="RadioFindings" ref="A9:L80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RadioFindings" displayName="RadioFindings" ref="A9:L81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Name in exchange"/>
     <x:tableColumn id="2" name="Responding radio ID"/>
@@ -214,8 +214,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S372" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:S372"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ResponseExchanges" displayName="ResponseExchanges" ref="A7:S373" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:S373"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="Evidence ID"/>
     <x:tableColumn id="2" name="Name in exchange"/>
@@ -545,7 +545,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 365 selected exchanges.</x:v>
+        <x:v>Response days = distinct dates with a named response example for that name and radio ID among the 366 selected exchanges.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -651,7 +651,7 @@
         <x:v>14580155</x:v>
       </x:c>
       <x:c r="C10" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A10,Exchanges!$J$8:$J$372,B10)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A10,Exchanges!$J$8:$J$373,B10)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
@@ -686,7 +686,7 @@
         <x:v>14590020</x:v>
       </x:c>
       <x:c r="C11" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A11,Exchanges!$J$8:$J$372,B11)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A11,Exchanges!$J$8:$J$373,B11)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D11" s="10" t="n">
@@ -721,7 +721,7 @@
         <x:v>14590089</x:v>
       </x:c>
       <x:c r="C12" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A12,Exchanges!$J$8:$J$372,B12)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A12,Exchanges!$J$8:$J$373,B12)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="10" t="n">
@@ -756,7 +756,7 @@
         <x:v>14590111</x:v>
       </x:c>
       <x:c r="C13" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A13,Exchanges!$J$8:$J$372,B13)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A13,Exchanges!$J$8:$J$373,B13)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D13" s="10" t="n">
@@ -791,7 +791,7 @@
         <x:v>14580152</x:v>
       </x:c>
       <x:c r="C14" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A14,Exchanges!$J$8:$J$372,B14)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A14,Exchanges!$J$8:$J$373,B14)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
@@ -826,7 +826,7 @@
         <x:v>14590098</x:v>
       </x:c>
       <x:c r="C15" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A15,Exchanges!$J$8:$J$372,B15)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A15,Exchanges!$J$8:$J$373,B15)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
@@ -863,7 +863,7 @@
         <x:v>14590107</x:v>
       </x:c>
       <x:c r="C16" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A16,Exchanges!$J$8:$J$372,B16)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A16,Exchanges!$J$8:$J$373,B16)</x:f>
         <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
@@ -898,7 +898,7 @@
         <x:v>14590104</x:v>
       </x:c>
       <x:c r="C17" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A17,Exchanges!$J$8:$J$372,B17)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A17,Exchanges!$J$8:$J$373,B17)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D17" s="10" t="n">
@@ -935,7 +935,7 @@
         <x:v>14590200</x:v>
       </x:c>
       <x:c r="C18" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A18,Exchanges!$J$8:$J$372,B18)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A18,Exchanges!$J$8:$J$373,B18)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="10" t="n">
@@ -972,7 +972,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C19" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A19,Exchanges!$J$8:$J$372,B19)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A19,Exchanges!$J$8:$J$373,B19)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
@@ -1011,7 +1011,7 @@
         <x:v>14590118</x:v>
       </x:c>
       <x:c r="C20" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A20,Exchanges!$J$8:$J$372,B20)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A20,Exchanges!$J$8:$J$373,B20)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
@@ -1048,7 +1048,7 @@
         <x:v>14590088</x:v>
       </x:c>
       <x:c r="C21" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A21,Exchanges!$J$8:$J$372,B21)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A21,Exchanges!$J$8:$J$373,B21)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
@@ -1085,7 +1085,7 @@
         <x:v>14590117</x:v>
       </x:c>
       <x:c r="C22" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A22,Exchanges!$J$8:$J$372,B22)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A22,Exchanges!$J$8:$J$373,B22)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
@@ -1120,7 +1120,7 @@
         <x:v>14590320</x:v>
       </x:c>
       <x:c r="C23" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A23,Exchanges!$J$8:$J$372,B23)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A23,Exchanges!$J$8:$J$373,B23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="10" t="n">
@@ -1155,7 +1155,7 @@
         <x:v>14590084</x:v>
       </x:c>
       <x:c r="C24" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A24,Exchanges!$J$8:$J$372,B24)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A24,Exchanges!$J$8:$J$373,B24)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D24" s="10" t="n">
@@ -1192,7 +1192,7 @@
         <x:v>14590105</x:v>
       </x:c>
       <x:c r="C25" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A25,Exchanges!$J$8:$J$372,B25)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A25,Exchanges!$J$8:$J$373,B25)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
@@ -1229,7 +1229,7 @@
         <x:v>14590237</x:v>
       </x:c>
       <x:c r="C26" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A26,Exchanges!$J$8:$J$372,B26)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A26,Exchanges!$J$8:$J$373,B26)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
@@ -1264,7 +1264,7 @@
         <x:v>14590315</x:v>
       </x:c>
       <x:c r="C27" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A27,Exchanges!$J$8:$J$372,B27)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A27,Exchanges!$J$8:$J$373,B27)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
@@ -1299,7 +1299,7 @@
         <x:v>14590162</x:v>
       </x:c>
       <x:c r="C28" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A28,Exchanges!$J$8:$J$372,B28)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A28,Exchanges!$J$8:$J$373,B28)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
@@ -1334,7 +1334,7 @@
         <x:v>14590081</x:v>
       </x:c>
       <x:c r="C29" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A29,Exchanges!$J$8:$J$372,B29)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A29,Exchanges!$J$8:$J$373,B29)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
@@ -1369,7 +1369,7 @@
         <x:v>14590102</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A30,Exchanges!$J$8:$J$372,B30)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A30,Exchanges!$J$8:$J$373,B30)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
@@ -1404,7 +1404,7 @@
         <x:v>14590344</x:v>
       </x:c>
       <x:c r="C31" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A31,Exchanges!$J$8:$J$372,B31)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A31,Exchanges!$J$8:$J$373,B31)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
@@ -1441,7 +1441,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C32" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A32,Exchanges!$J$8:$J$372,B32)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A32,Exchanges!$J$8:$J$373,B32)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
@@ -1480,7 +1480,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C33" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A33,Exchanges!$J$8:$J$372,B33)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A33,Exchanges!$J$8:$J$373,B33)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
@@ -1517,7 +1517,7 @@
         <x:v>14590087</x:v>
       </x:c>
       <x:c r="C34" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A34,Exchanges!$J$8:$J$372,B34)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A34,Exchanges!$J$8:$J$373,B34)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D34" s="10" t="n">
@@ -1552,7 +1552,7 @@
         <x:v>14590044</x:v>
       </x:c>
       <x:c r="C35" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A35,Exchanges!$J$8:$J$372,B35)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A35,Exchanges!$J$8:$J$373,B35)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D35" s="10" t="n">
@@ -1587,7 +1587,7 @@
         <x:v>14590123</x:v>
       </x:c>
       <x:c r="C36" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A36,Exchanges!$J$8:$J$372,B36)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A36,Exchanges!$J$8:$J$373,B36)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D36" s="10" t="n">
@@ -1622,7 +1622,7 @@
         <x:v>14590067</x:v>
       </x:c>
       <x:c r="C37" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A37,Exchanges!$J$8:$J$372,B37)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A37,Exchanges!$J$8:$J$373,B37)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D37" s="10" t="n">
@@ -1659,7 +1659,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C38" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A38,Exchanges!$J$8:$J$372,B38)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A38,Exchanges!$J$8:$J$373,B38)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D38" s="10" t="n">
@@ -1698,7 +1698,7 @@
         <x:v>14590090</x:v>
       </x:c>
       <x:c r="C39" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A39,Exchanges!$J$8:$J$372,B39)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A39,Exchanges!$J$8:$J$373,B39)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D39" s="10" t="n">
@@ -1735,7 +1735,7 @@
         <x:v>14590066</x:v>
       </x:c>
       <x:c r="C40" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A40,Exchanges!$J$8:$J$372,B40)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A40,Exchanges!$J$8:$J$373,B40)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D40" s="10" t="n">
@@ -1772,7 +1772,7 @@
         <x:v>14590268</x:v>
       </x:c>
       <x:c r="C41" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A41,Exchanges!$J$8:$J$372,B41)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A41,Exchanges!$J$8:$J$373,B41)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="10" t="n">
@@ -1809,7 +1809,7 @@
         <x:v>14590037</x:v>
       </x:c>
       <x:c r="C42" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A42,Exchanges!$J$8:$J$372,B42)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A42,Exchanges!$J$8:$J$373,B42)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D42" s="10" t="n">
@@ -1846,7 +1846,7 @@
         <x:v>14590095</x:v>
       </x:c>
       <x:c r="C43" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A43,Exchanges!$J$8:$J$372,B43)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A43,Exchanges!$J$8:$J$373,B43)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D43" s="10" t="n">
@@ -1883,7 +1883,7 @@
         <x:v>14590099</x:v>
       </x:c>
       <x:c r="C44" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A44,Exchanges!$J$8:$J$372,B44)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A44,Exchanges!$J$8:$J$373,B44)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D44" s="10" t="n">
@@ -1920,7 +1920,7 @@
         <x:v>14590207</x:v>
       </x:c>
       <x:c r="C45" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A45,Exchanges!$J$8:$J$372,B45)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A45,Exchanges!$J$8:$J$373,B45)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D45" s="10" t="n">
@@ -1957,7 +1957,7 @@
         <x:v>14590042</x:v>
       </x:c>
       <x:c r="C46" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A46,Exchanges!$J$8:$J$372,B46)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A46,Exchanges!$J$8:$J$373,B46)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D46" s="10" t="n">
@@ -1992,7 +1992,7 @@
         <x:v>14590073</x:v>
       </x:c>
       <x:c r="C47" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A47,Exchanges!$J$8:$J$372,B47)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A47,Exchanges!$J$8:$J$373,B47)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D47" s="10" t="n">
@@ -2027,7 +2027,7 @@
         <x:v>14590038</x:v>
       </x:c>
       <x:c r="C48" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A48,Exchanges!$J$8:$J$372,B48)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A48,Exchanges!$J$8:$J$373,B48)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D48" s="10" t="n">
@@ -2062,7 +2062,7 @@
         <x:v>14590345</x:v>
       </x:c>
       <x:c r="C49" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A49,Exchanges!$J$8:$J$372,B49)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A49,Exchanges!$J$8:$J$373,B49)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D49" s="10" t="n">
@@ -2097,7 +2097,7 @@
         <x:v>14590079</x:v>
       </x:c>
       <x:c r="C50" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A50,Exchanges!$J$8:$J$372,B50)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A50,Exchanges!$J$8:$J$373,B50)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D50" s="10" t="n">
@@ -2132,7 +2132,7 @@
         <x:v>14590026</x:v>
       </x:c>
       <x:c r="C51" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A51,Exchanges!$J$8:$J$372,B51)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A51,Exchanges!$J$8:$J$373,B51)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D51" s="10" t="n">
@@ -2169,7 +2169,7 @@
         <x:v>14590031</x:v>
       </x:c>
       <x:c r="C52" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A52,Exchanges!$J$8:$J$372,B52)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A52,Exchanges!$J$8:$J$373,B52)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D52" s="10" t="n">
@@ -2206,7 +2206,7 @@
         <x:v>14590101</x:v>
       </x:c>
       <x:c r="C53" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A53,Exchanges!$J$8:$J$372,B53)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A53,Exchanges!$J$8:$J$373,B53)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D53" s="10" t="n">
@@ -2243,7 +2243,7 @@
         <x:v>14590103</x:v>
       </x:c>
       <x:c r="C54" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A54,Exchanges!$J$8:$J$372,B54)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A54,Exchanges!$J$8:$J$373,B54)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
@@ -2280,7 +2280,7 @@
         <x:v>14590043</x:v>
       </x:c>
       <x:c r="C55" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A55,Exchanges!$J$8:$J$372,B55)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A55,Exchanges!$J$8:$J$373,B55)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
@@ -2317,7 +2317,7 @@
         <x:v>14590025</x:v>
       </x:c>
       <x:c r="C56" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A56,Exchanges!$J$8:$J$372,B56)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A56,Exchanges!$J$8:$J$373,B56)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
@@ -2356,7 +2356,7 @@
         <x:v>14590266</x:v>
       </x:c>
       <x:c r="C57" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A57,Exchanges!$J$8:$J$372,B57)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A57,Exchanges!$J$8:$J$373,B57)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D57" s="10" t="n">
@@ -2391,7 +2391,7 @@
         <x:v>14590219</x:v>
       </x:c>
       <x:c r="C58" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A58,Exchanges!$J$8:$J$372,B58)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A58,Exchanges!$J$8:$J$373,B58)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D58" s="10" t="n">
@@ -2426,7 +2426,7 @@
         <x:v>14590085</x:v>
       </x:c>
       <x:c r="C59" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A59,Exchanges!$J$8:$J$372,B59)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A59,Exchanges!$J$8:$J$373,B59)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D59" s="10" t="n">
@@ -2463,7 +2463,7 @@
         <x:v>14590126</x:v>
       </x:c>
       <x:c r="C60" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A60,Exchanges!$J$8:$J$372,B60)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A60,Exchanges!$J$8:$J$373,B60)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D60" s="10" t="n">
@@ -2502,7 +2502,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C61" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A61,Exchanges!$J$8:$J$372,B61)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A61,Exchanges!$J$8:$J$373,B61)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="10" t="n">
@@ -2541,7 +2541,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C62" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A62,Exchanges!$J$8:$J$372,B62)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A62,Exchanges!$J$8:$J$373,B62)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D62" s="10" t="n">
@@ -2580,7 +2580,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C63" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A63,Exchanges!$J$8:$J$372,B63)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A63,Exchanges!$J$8:$J$373,B63)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D63" s="10" t="n">
@@ -2619,7 +2619,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C64" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A64,Exchanges!$J$8:$J$372,B64)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A64,Exchanges!$J$8:$J$373,B64)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D64" s="10" t="n">
@@ -2658,7 +2658,7 @@
         <x:v>14590091</x:v>
       </x:c>
       <x:c r="C65" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A65,Exchanges!$J$8:$J$372,B65)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A65,Exchanges!$J$8:$J$373,B65)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D65" s="10" t="n">
@@ -2697,7 +2697,7 @@
         <x:v>14590100</x:v>
       </x:c>
       <x:c r="C66" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A66,Exchanges!$J$8:$J$372,B66)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A66,Exchanges!$J$8:$J$373,B66)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D66" s="10" t="n">
@@ -2736,7 +2736,7 @@
         <x:v>14590225</x:v>
       </x:c>
       <x:c r="C67" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A67,Exchanges!$J$8:$J$372,B67)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A67,Exchanges!$J$8:$J$373,B67)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D67" s="10" t="n">
@@ -2775,7 +2775,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C68" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A68,Exchanges!$J$8:$J$372,B68)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A68,Exchanges!$J$8:$J$373,B68)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D68" s="10" t="n">
@@ -2814,7 +2814,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C69" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A69,Exchanges!$J$8:$J$372,B69)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A69,Exchanges!$J$8:$J$373,B69)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D69" s="10" t="n">
@@ -2851,7 +2851,7 @@
         <x:v>14590036</x:v>
       </x:c>
       <x:c r="C70" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A70,Exchanges!$J$8:$J$372,B70)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A70,Exchanges!$J$8:$J$373,B70)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D70" s="10" t="n">
@@ -2890,7 +2890,7 @@
         <x:v>14590221</x:v>
       </x:c>
       <x:c r="C71" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A71,Exchanges!$J$8:$J$372,B71)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A71,Exchanges!$J$8:$J$373,B71)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D71" s="10" t="n">
@@ -2929,7 +2929,7 @@
         <x:v>14590019</x:v>
       </x:c>
       <x:c r="C72" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A72,Exchanges!$J$8:$J$372,B72)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A72,Exchanges!$J$8:$J$373,B72)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D72" s="10" t="n">
@@ -2966,7 +2966,7 @@
         <x:v>14590247</x:v>
       </x:c>
       <x:c r="C73" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A73,Exchanges!$J$8:$J$372,B73)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A73,Exchanges!$J$8:$J$373,B73)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D73" s="10" t="n">
@@ -3003,7 +3003,7 @@
         <x:v>14590112</x:v>
       </x:c>
       <x:c r="C74" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A74,Exchanges!$J$8:$J$372,B74)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A74,Exchanges!$J$8:$J$373,B74)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D74" s="10" t="n">
@@ -3040,7 +3040,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C75" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A75,Exchanges!$J$8:$J$372,B75)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A75,Exchanges!$J$8:$J$373,B75)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D75" s="10" t="n">
@@ -3079,7 +3079,7 @@
         <x:v>14590027</x:v>
       </x:c>
       <x:c r="C76" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A76,Exchanges!$J$8:$J$372,B76)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A76,Exchanges!$J$8:$J$373,B76)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D76" s="10" t="n">
@@ -3118,7 +3118,7 @@
         <x:v>14590097</x:v>
       </x:c>
       <x:c r="C77" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A77,Exchanges!$J$8:$J$372,B77)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A77,Exchanges!$J$8:$J$373,B77)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D77" s="10" t="n">
@@ -3155,7 +3155,7 @@
         <x:v>14580151</x:v>
       </x:c>
       <x:c r="C78" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A78,Exchanges!$J$8:$J$372,B78)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A78,Exchanges!$J$8:$J$373,B78)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D78" s="10" t="n">
@@ -3192,7 +3192,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C79" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A79,Exchanges!$J$8:$J$372,B79)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A79,Exchanges!$J$8:$J$373,B79)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="10" t="n">
@@ -3231,7 +3231,7 @@
         <x:v>14590114</x:v>
       </x:c>
       <x:c r="C80" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$372,A80,Exchanges!$J$8:$J$372,B80)</x:f>
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A80,Exchanges!$J$8:$J$373,B80)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D80" s="10" t="n">
@@ -3263,18 +3263,41 @@
       </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="10"/>
-      <x:c r="B81" s="11"/>
-      <x:c r="C81" s="10"/>
-      <x:c r="D81" s="10"/>
-      <x:c r="E81" s="12"/>
-      <x:c r="F81" s="12"/>
-      <x:c r="G81" s="10"/>
+      <x:c r="A81" s="10" t="str">
+        <x:v>Manis</x:v>
+      </x:c>
+      <x:c r="B81" s="11" t="str">
+        <x:v>14590314</x:v>
+      </x:c>
+      <x:c r="C81" s="10" t="n">
+        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A81,Exchanges!$J$8:$J$373,B81)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D81" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E81" s="12" t="n">
+        <x:v>46299</x:v>
+      </x:c>
+      <x:c r="F81" s="12" t="n">
+        <x:v>46299</x:v>
+      </x:c>
+      <x:c r="G81" s="10" t="str">
+        <x:v>Owner-confirmed this day</x:v>
+      </x:c>
       <x:c r="H81" s="10"/>
-      <x:c r="I81" s="10"/>
-      <x:c r="J81" s="10"/>
-      <x:c r="K81" s="10"/>
-      <x:c r="L81" s="10"/>
+      <x:c r="I81" s="10" t="str">
+        <x:v>Dustin K. Manis</x:v>
+      </x:c>
+      <x:c r="J81" s="10" t="str">
+        <x:v>Owner confirms Dustin K. Manis on 14590314 for October 4 only. Clips 15 and 16 transcript-verified; the reply text is not separately verified. September 11 and October 3 similar-sounding hails remain tentative.</x:v>
+      </x:c>
+      <x:c r="K81" s="10" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="L81" s="10" t="str">
+        <x:v>E366</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="10"/>
@@ -24956,6 +24979,66 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="373">
+      <x:c r="A373" s="13" t="str">
+        <x:v>E366</x:v>
+      </x:c>
+      <x:c r="B373" s="13" t="str">
+        <x:v>Manis</x:v>
+      </x:c>
+      <x:c r="C373" s="14" t="n">
+        <x:v>46299</x:v>
+      </x:c>
+      <x:c r="D373" s="13" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E373" s="15" t="n">
+        <x:v>0.04393518518518519</x:v>
+      </x:c>
+      <x:c r="F373" s="16" t="str">
+        <x:v>14590104</x:v>
+      </x:c>
+      <x:c r="G373" s="13" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H373" s="15" t="n">
+        <x:v>0.04400462962962963</x:v>
+      </x:c>
+      <x:c r="I373" s="17" t="n">
+        <x:f>ROUND((H373-E373)*86400,0)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J373" s="16" t="str">
+        <x:v>14590314</x:v>
+      </x:c>
+      <x:c r="K373" s="13" t="str">
+        <x:v>Manis?</x:v>
+      </x:c>
+      <x:c r="L373" s="13" t="str">
+        <x:v>Yeah.</x:v>
+      </x:c>
+      <x:c r="M373" s="13" t="str">
+        <x:v>Owner-confirmed this day</x:v>
+      </x:c>
+      <x:c r="N373" s="13" t="str">
+        <x:v>Owner confirms Dustin K. Manis on 14590314 for October 4 only. Clips 15 and 16 transcript-verified; the reply text is not separately verified. September 11 and October 3 similar-sounding hails remain tentative.</x:v>
+      </x:c>
+      <x:c r="O373" s="18" t="str">
+        <x:v>Owner reviewed hail and confirmed day identity; reply text not separately verified</x:v>
+      </x:c>
+      <x:c r="P373" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-04/dcfems-6001-1791097396.m4a</x:v>
+      </x:c>
+      <x:c r="Q373" s="19" t="str">
+        <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-04/dcfems-6001-1791097402.m4a</x:v>
+      </x:c>
+      <x:c r="R373" s="19" t="str">
+        <x:v>https://afpd-accountability.com/police-radio/?date=2026-10-04</x:v>
+      </x:c>
+      <x:c r="S373" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="O8:O346">

</xml_diff>

<commit_message>
Distinguish confirmed October 21 McKay ID from strong association
</commit_message>
<xml_diff>
--- a/public/records/openmhz/afpd-radio-id-response-days.xlsx
+++ b/public/records/openmhz/afpd-radio-id-response-days.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R036cb515380e4b2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="Rd57dbd6f9a6e4054"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R65c3d451b0be4487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="R26c757c5a2924894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R76490b10e0954b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchanges" sheetId="2" r:id="R3326e0b204d44882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" r:id="R172420d008f44377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="4" r:id="Rcc94bd3712d74a1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -964,7 +964,7 @@
         <x:v>E002, E014</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="60" customHeight="1">
+    <x:row r="19" ht="150" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>Jake</x:v>
       </x:c>
@@ -985,16 +985,14 @@
         <x:v>46306</x:v>
       </x:c>
       <x:c r="G19" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H19" s="10" t="str">
-        <x:v>Laycock</x:v>
-      </x:c>
+        <x:v>Pending listening review</x:v>
+      </x:c>
+      <x:c r="H19" s="10"/>
       <x:c r="I19" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Jake D. Laycock — sole candidate; unverified</x:v>
       </x:c>
       <x:c r="J19" s="10" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="K19" s="10" t="str">
         <x:v>2026-09-11, 2026-09-17, 2026-10-11</x:v>
@@ -1003,7 +1001,7 @@
         <x:v>E016, E115, E287</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="60" customHeight="1">
+    <x:row r="20" ht="150" customHeight="1">
       <x:c r="A20" s="10" t="str">
         <x:v>Jake</x:v>
       </x:c>
@@ -1028,10 +1026,10 @@
       </x:c>
       <x:c r="H20" s="10"/>
       <x:c r="I20" s="10" t="str">
-        <x:v>Multiple candidates</x:v>
+        <x:v>Jake D. Laycock — sole candidate; unverified</x:v>
       </x:c>
       <x:c r="J20" s="10" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="K20" s="10" t="str">
         <x:v>2026-09-11, 2026-09-12, 2026-09-13, 2026-09-16, 2026-09-17, 2026-09-22, 2026-09-30, 2026-10-01, 2026-10-11, 2026-10-15, 2026-10-19</x:v>
@@ -1326,7 +1324,7 @@
         <x:v>E127, E161, E202</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="60" customHeight="1">
+    <x:row r="29" ht="150" customHeight="1">
       <x:c r="A29" s="10" t="str">
         <x:v>McKay</x:v>
       </x:c>
@@ -1347,13 +1345,15 @@
         <x:v>46316</x:v>
       </x:c>
       <x:c r="G29" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Owner confirmed October 21</x:v>
       </x:c>
       <x:c r="H29" s="10"/>
       <x:c r="I29" s="10" t="str">
         <x:v>Mckay A. Valadez</x:v>
       </x:c>
-      <x:c r="J29" s="10"/>
+      <x:c r="J29" s="10" t="str">
+        <x:v>Owner confirms McKay on October 21, clips 66–67 (E336). September 10 clips 261–262 (E009) remain tentative. Two selected examples; only October 21 is owner-confirmed. Identity confirmation does not verify the full transcript wording.</x:v>
+      </x:c>
       <x:c r="K29" s="10" t="str">
         <x:v>2026-09-10, 2026-10-21</x:v>
       </x:c>
@@ -1361,7 +1361,7 @@
         <x:v>E009, E336</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="60" customHeight="1">
+    <x:row r="30" ht="150" customHeight="1">
       <x:c r="A30" s="10" t="str">
         <x:v>McKay</x:v>
       </x:c>
@@ -1369,31 +1369,32 @@
         <x:v>14590102</x:v>
       </x:c>
       <x:c r="C30" s="10" t="n">
-        <x:f>COUNTIFS(Exchanges!$B$8:$B$373,A30,Exchanges!$J$8:$J$373,B30)</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E30" s="12" t="n">
         <x:v>46275</x:v>
       </x:c>
       <x:c r="F30" s="12" t="n">
-        <x:v>46316</x:v>
+        <x:v>46312</x:v>
       </x:c>
       <x:c r="G30" s="10" t="str">
-        <x:v>Repeated across days</x:v>
+        <x:v>Strong association across days</x:v>
       </x:c>
       <x:c r="H30" s="10"/>
       <x:c r="I30" s="10" t="str">
         <x:v>Mckay A. Valadez</x:v>
       </x:c>
-      <x:c r="J30" s="10"/>
+      <x:c r="J30" s="10" t="str">
+        <x:v>Seven supporting exchanges across five earlier dates. October 21 clips 63–64 (E335) have an unclear reply; the pairing remains unverified, is excluded from these counts, and does not confirm McKay that day. The day label remains Strong association.</x:v>
+      </x:c>
       <x:c r="K30" s="10" t="str">
-        <x:v>2026-09-10, 2026-09-14, 2026-09-18, 2026-09-28, 2026-10-17, 2026-10-21</x:v>
+        <x:v>2026-09-10, 2026-09-14, 2026-09-18, 2026-09-28, 2026-10-17</x:v>
       </x:c>
       <x:c r="L30" s="10" t="str">
-        <x:v>E010, E090, E091, E126, E200, E323, E325, E335</x:v>
+        <x:v>E010, E090, E091, E126, E200, E323, E325</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
@@ -2309,7 +2310,7 @@
         <x:v>E259</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="60" customHeight="1">
+    <x:row r="56" ht="150" customHeight="1">
       <x:c r="A56" s="10" t="str">
         <x:v>Laycock</x:v>
       </x:c>
@@ -2330,16 +2331,14 @@
         <x:v>46287</x:v>
       </x:c>
       <x:c r="G56" s="10" t="str">
-        <x:v>Conflicting names on ID</x:v>
-      </x:c>
-      <x:c r="H56" s="10" t="str">
-        <x:v>Jake</x:v>
-      </x:c>
+        <x:v>Pending listening review</x:v>
+      </x:c>
+      <x:c r="H56" s="10"/>
       <x:c r="I56" s="10" t="str">
-        <x:v>Jake D. Laycock</x:v>
+        <x:v>Jake D. Laycock — sole candidate; unverified</x:v>
       </x:c>
       <x:c r="J56" s="10" t="str">
-        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="K56" s="10" t="str">
         <x:v>2026-09-22</x:v>
@@ -3320,7 +3319,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R119bb1e2055f4e50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re91720e67a2e4b13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4007,7 +4006,7 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="60" customHeight="1">
+    <x:row r="16" ht="150" customHeight="1">
       <x:c r="A16" s="13" t="str">
         <x:v>E009</x:v>
       </x:c>
@@ -4048,7 +4047,9 @@
       <x:c r="M16" s="13" t="str">
         <x:v>Transcript association</x:v>
       </x:c>
-      <x:c r="N16" s="13" t="str"/>
+      <x:c r="N16" s="13" t="str">
+        <x:v>Tentative September 10 McKay exchange: both the addressed name and short reply are uncertain. October 21 confirmation does not verify this earlier date.</x:v>
+      </x:c>
       <x:c r="O16" s="18" t="str">
         <x:v>Not reviewed</x:v>
       </x:c>
@@ -4461,7 +4462,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N23" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O23" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -4521,7 +4522,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N24" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O24" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -4641,7 +4642,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N26" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O26" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -5927,7 +5928,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N48" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O48" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6103,7 +6104,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N51" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O51" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6163,7 +6164,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N52" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O52" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6341,7 +6342,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N55" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O55" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6519,7 +6520,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N58" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O58" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6869,7 +6870,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N64" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O64" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -6929,7 +6930,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N65" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O65" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -7047,7 +7048,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N67" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O67" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -7751,7 +7752,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N79" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O79" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -7869,7 +7870,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N81" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O81" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -9267,7 +9268,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N105" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O105" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -9501,7 +9502,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N109" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O109" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -10143,7 +10144,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N120" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O120" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -10261,7 +10262,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N122" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O122" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -11849,7 +11850,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N149" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O149" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -11909,7 +11910,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N150" s="13" t="str">
-        <x:v>Surname hail is marked uncertain in the transcript. This supports a Laycock candidate for 14590025, not for every ID answering Jake.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O150" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -12027,7 +12028,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N152" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O152" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -12261,7 +12262,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N156" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O156" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -15893,7 +15894,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N218" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O218" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -16187,7 +16188,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N223" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O223" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -20285,7 +20286,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N293" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O293" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -20345,7 +20346,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N294" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O294" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -21633,7 +21634,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N316" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O316" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -21693,7 +21694,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N317" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O317" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -21933,7 +21934,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N321" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O321" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -22757,7 +22758,7 @@
         <x:v>Transcript association</x:v>
       </x:c>
       <x:c r="N335" s="13" t="str">
-        <x:v>More than one officer on the roster uses Jake or Jacob. These rows preserve the spoken first name only.</x:v>
+        <x:v>Only one current AFPD Jake/Jacob candidate: Jake D. Laycock. Dain left 2021-08-12; Hager 2024-06-26; Thacker 2025-08-14. Radio identity unverified; Eric must listen before assigning Laycock to either ID.</x:v>
       </x:c>
       <x:c r="O335" s="18" t="str">
         <x:v>Not reviewed</x:v>
@@ -23129,7 +23130,7 @@
         <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="342" ht="60" customHeight="1">
+    <x:row r="342" ht="150" customHeight="1">
       <x:c r="A342" s="13" t="str">
         <x:v>E335</x:v>
       </x:c>
@@ -23168,9 +23169,11 @@
         <x:v>[unclear reponse].</x:v>
       </x:c>
       <x:c r="M342" s="13" t="str">
-        <x:v>Transcript association</x:v>
-      </x:c>
-      <x:c r="N342" s="13" t="str"/>
+        <x:v>Tentative response pairing</x:v>
+      </x:c>
+      <x:c r="N342" s="13" t="str">
+        <x:v>October 21 clips 63–64: the reply is unclear, so this pairing remains unverified and is excluded from supporting example/day counts. 14590102 retains a strong McKay association from seven exchanges across five earlier dates.</x:v>
+      </x:c>
       <x:c r="O342" s="18" t="str">
         <x:v>Not reviewed</x:v>
       </x:c>
@@ -23187,7 +23190,7 @@
         <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="343" ht="60" customHeight="1">
+    <x:row r="343" ht="150" customHeight="1">
       <x:c r="A343" s="13" t="str">
         <x:v>E336</x:v>
       </x:c>
@@ -23226,11 +23229,13 @@
         <x:v>Negative, [remainder unclear].</x:v>
       </x:c>
       <x:c r="M343" s="13" t="str">
-        <x:v>Transcript association</x:v>
-      </x:c>
-      <x:c r="N343" s="13" t="str"/>
+        <x:v>Owner-confirmed identity</x:v>
+      </x:c>
+      <x:c r="N343" s="13" t="str">
+        <x:v>Owner confirms McKay / 14590081 for October 21, clips 66–67. This confirms the identity association; it does not verify the full transcript wording.</x:v>
+      </x:c>
       <x:c r="O343" s="18" t="str">
-        <x:v>Not reviewed</x:v>
+        <x:v>Owner confirmed identity; wording not verified</x:v>
       </x:c>
       <x:c r="P343" s="19" t="str">
         <x:v>https://afpd-accountability.com/records/openmhz/openmhz-afpd-car-to-car-2026-10-21/dcfems-6001-1792613234.m4a</x:v>
@@ -25047,7 +25052,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf72f5adf98714fe9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f70026429094f9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25539,7 +25544,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R418651804c124fb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22956d1535e54a6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26504,7 +26509,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14bc226f72d04874"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra28742cd71954513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>